<commit_message>
weekend contest 10 to 13
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60CD08DB-FE80-A740-B590-724B9B298658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFFD6083-23F6-C145-8EBC-22323CA48ED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-49020" yWindow="-2500" windowWidth="47880" windowHeight="26560" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -1890,46 +1890,62 @@
       <c r="C21" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="3" t="str">
+      <c r="D21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E21" s="4"/>
-      <c r="G21" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="E21" s="4">
+        <v>30</v>
+      </c>
+      <c r="G21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H21" s="4"/>
-      <c r="J21" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="H21" s="4">
+        <v>100</v>
+      </c>
+      <c r="J21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K21" s="4"/>
-      <c r="M21" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="K21" s="4">
+        <v>0</v>
+      </c>
+      <c r="M21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N21" s="4"/>
-      <c r="P21" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="N21" s="4">
+        <v>20</v>
+      </c>
+      <c r="P21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q21" s="4"/>
-      <c r="S21" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q21" s="4">
+        <v>60</v>
+      </c>
+      <c r="S21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T21" s="4"/>
-      <c r="V21" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T21" s="4">
+        <v>70</v>
+      </c>
+      <c r="V21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W21" s="4"/>
-      <c r="Y21" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="W21" s="4">
+        <v>40</v>
+      </c>
+      <c r="Y21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z21" s="4"/>
+        <v>-5</v>
+      </c>
+      <c r="Z21" s="4">
+        <v>50</v>
+      </c>
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
@@ -1941,46 +1957,62 @@
       <c r="C22" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="3" t="str">
+      <c r="D22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E22" s="4"/>
-      <c r="G22" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="E22" s="4">
+        <v>50</v>
+      </c>
+      <c r="G22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H22" s="4"/>
-      <c r="J22" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H22" s="4">
+        <v>60</v>
+      </c>
+      <c r="J22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K22" s="4"/>
-      <c r="M22" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="K22" s="4">
+        <v>40</v>
+      </c>
+      <c r="M22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N22" s="4"/>
-      <c r="P22" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N22" s="4">
+        <v>100</v>
+      </c>
+      <c r="P22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q22" s="4"/>
-      <c r="S22" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Q22" s="4">
+        <v>0</v>
+      </c>
+      <c r="S22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T22" s="4"/>
-      <c r="V22" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T22" s="4">
+        <v>70</v>
+      </c>
+      <c r="V22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W22" s="4"/>
-      <c r="Y22" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W22" s="4">
+        <v>30</v>
+      </c>
+      <c r="Y22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z22" s="4"/>
+        <v>-20</v>
+      </c>
+      <c r="Z22" s="4">
+        <v>20</v>
+      </c>
     </row>
     <row r="23" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
@@ -1992,46 +2024,62 @@
       <c r="C23" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="3" t="str">
+      <c r="D23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E23" s="4"/>
-      <c r="G23" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="E23" s="4">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H23" s="4"/>
-      <c r="J23" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H23" s="4">
+        <v>60</v>
+      </c>
+      <c r="J23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K23" s="4"/>
-      <c r="M23" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K23" s="4">
+        <v>30</v>
+      </c>
+      <c r="M23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N23" s="4"/>
-      <c r="P23" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="N23" s="4">
+        <v>20</v>
+      </c>
+      <c r="P23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q23" s="4"/>
-      <c r="S23" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q23" s="4">
+        <v>70</v>
+      </c>
+      <c r="S23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T23" s="4"/>
-      <c r="V23" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="T23" s="4">
+        <v>50</v>
+      </c>
+      <c r="V23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W23" s="4"/>
-      <c r="Y23" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="W23" s="4">
+        <v>100</v>
+      </c>
+      <c r="Y23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z23" s="4"/>
+        <v>-10</v>
+      </c>
+      <c r="Z23" s="4">
+        <v>40</v>
+      </c>
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
@@ -2043,46 +2091,60 @@
       <c r="C24" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="D24" s="3" t="str">
+      <c r="D24" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E24" s="4"/>
-      <c r="G24" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E24" s="4">
+        <v>40</v>
+      </c>
+      <c r="G24" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H24" s="4"/>
-      <c r="J24" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H24" s="4">
+        <v>60</v>
+      </c>
+      <c r="J24" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K24" s="4"/>
-      <c r="M24" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N24" s="4"/>
-      <c r="P24" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="K24" s="4">
+        <v>100</v>
+      </c>
+      <c r="M24" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="N24" s="4">
+        <v>20</v>
+      </c>
+      <c r="P24" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q24" s="4"/>
-      <c r="S24" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q24" s="4">
+        <v>70</v>
+      </c>
+      <c r="S24" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T24" s="4"/>
-      <c r="V24" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="T24" s="4">
+        <v>50</v>
+      </c>
+      <c r="V24" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W24" s="4"/>
-      <c r="Y24" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Z24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z24" s="4"/>
+        <v>-15</v>
+      </c>
+      <c r="W24" s="4">
+        <v>30</v>
+      </c>
+      <c r="Y24" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="Z24" s="4">
+        <v>20</v>
+      </c>
     </row>
     <row r="25" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
@@ -2094,46 +2156,62 @@
       <c r="C25" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="D25" s="3" t="str">
+      <c r="D25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E25" s="4"/>
-      <c r="G25" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E25" s="4">
+        <v>40</v>
+      </c>
+      <c r="G25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H25" s="4"/>
-      <c r="J25" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="H25" s="4">
+        <v>0</v>
+      </c>
+      <c r="J25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K25" s="4"/>
-      <c r="M25" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="K25" s="4">
+        <v>50</v>
+      </c>
+      <c r="M25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N25" s="4"/>
-      <c r="P25" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N25" s="4">
+        <v>100</v>
+      </c>
+      <c r="P25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q25" s="4"/>
-      <c r="S25" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q25" s="4">
+        <v>20</v>
+      </c>
+      <c r="S25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T25" s="4"/>
-      <c r="V25" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T25" s="4">
+        <v>60</v>
+      </c>
+      <c r="V25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W25" s="4"/>
-      <c r="Y25" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="W25" s="4">
+        <v>70</v>
+      </c>
+      <c r="Y25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z25" s="4"/>
+        <v>-15</v>
+      </c>
+      <c r="Z25" s="4">
+        <v>30</v>
+      </c>
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
@@ -4551,28 +4629,28 @@
       </c>
       <c r="E75" s="10">
         <f>SUM(D13:D72)</f>
-        <v>-20</v>
+        <v>-85</v>
       </c>
       <c r="G75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(G13:G72)</f>
-        <v>-55</v>
+        <v>-15</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K75" s="10">
         <f>SUM(J13:J72)</f>
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N75" s="10">
         <f>SUM(M13:M72)</f>
-        <v>17.5</v>
+        <v>55</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>7</v>
@@ -4586,21 +4664,21 @@
       </c>
       <c r="T75" s="10">
         <f>SUM(S13:S72)</f>
-        <v>-132.5</v>
+        <v>-97.5</v>
       </c>
       <c r="V75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W75" s="10">
         <f>SUM(V13:V72)</f>
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="Y75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z75" s="10">
         <f>SUM(Y13:Y72)</f>
-        <v>-75</v>
+        <v>-147.5</v>
       </c>
       <c r="AA75" s="1">
         <f>SUM(E75,H75,K75,N75,Q75,T75,W75,Z75)</f>

</xml_diff>

<commit_message>
Contest 14 MI vs RR
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFFD6083-23F6-C145-8EBC-22323CA48ED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C10CCA3-C28C-3744-9672-636C37347675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-49020" yWindow="-2500" windowWidth="47880" windowHeight="26560" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -2223,46 +2223,60 @@
       <c r="C26" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="D26" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E26" s="4"/>
-      <c r="G26" s="3" t="str">
+      <c r="D26" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="E26" s="4">
+        <v>20</v>
+      </c>
+      <c r="G26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H26" s="4"/>
-      <c r="J26" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="H26" s="4">
+        <v>40</v>
+      </c>
+      <c r="J26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K26" s="4"/>
-      <c r="M26" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="K26" s="4">
+        <v>100</v>
+      </c>
+      <c r="M26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N26" s="4"/>
-      <c r="P26" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="N26" s="4">
+        <v>60</v>
+      </c>
+      <c r="P26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q26" s="4"/>
-      <c r="S26" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(T26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T26" s="4"/>
-      <c r="V26" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q26" s="4">
+        <v>70</v>
+      </c>
+      <c r="S26" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="T26" s="4">
+        <v>20</v>
+      </c>
+      <c r="V26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W26" s="4"/>
-      <c r="Y26" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="W26" s="4">
+        <v>50</v>
+      </c>
+      <c r="Y26" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z26, ($Z26,$W26,$T26,$Q26,$N26,$K26,$H26,$E26), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z26" s="4"/>
+        <v>-15</v>
+      </c>
+      <c r="Z26" s="4">
+        <v>30</v>
+      </c>
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
@@ -4629,56 +4643,56 @@
       </c>
       <c r="E75" s="10">
         <f>SUM(D13:D72)</f>
-        <v>-85</v>
+        <v>-107.5</v>
       </c>
       <c r="G75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(G13:G72)</f>
-        <v>-15</v>
+        <v>-25</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K75" s="10">
         <f>SUM(J13:J72)</f>
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N75" s="10">
         <f>SUM(M13:M72)</f>
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q75" s="10">
         <f>SUM(P13:P72)</f>
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="S75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T75" s="10">
         <f>SUM(S13:S72)</f>
-        <v>-97.5</v>
+        <v>-120</v>
       </c>
       <c r="V75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W75" s="10">
         <f>SUM(V13:V72)</f>
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="Y75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z75" s="10">
         <f>SUM(Y13:Y72)</f>
-        <v>-147.5</v>
+        <v>-162.5</v>
       </c>
       <c r="AA75" s="1">
         <f>SUM(E75,H75,K75,N75,Q75,T75,W75,Z75)</f>

</xml_diff>

<commit_message>
Contest 15 RCB vs LSG
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C10CCA3-C28C-3744-9672-636C37347675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7CA9BA-F2B4-0547-95D1-05C94CEF9EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-49020" yWindow="-2500" windowWidth="47880" windowHeight="26560" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -2288,46 +2288,62 @@
       <c r="C27" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="D27" s="3" t="str">
+      <c r="D27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E27" s="4"/>
-      <c r="G27" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="E27" s="4">
+        <v>60</v>
+      </c>
+      <c r="G27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H27" s="4"/>
-      <c r="J27" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="H27" s="4">
+        <v>20</v>
+      </c>
+      <c r="J27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K27" s="4"/>
-      <c r="M27" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="K27" s="4">
+        <v>70</v>
+      </c>
+      <c r="M27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N27" s="4"/>
-      <c r="P27" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N27" s="4">
+        <v>100</v>
+      </c>
+      <c r="P27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q27" s="4"/>
-      <c r="S27" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Q27" s="4">
+        <v>40</v>
+      </c>
+      <c r="S27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T27" s="4"/>
-      <c r="V27" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="T27" s="4">
+        <v>30</v>
+      </c>
+      <c r="V27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W27" s="4"/>
-      <c r="Y27" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="W27" s="4">
+        <v>50</v>
+      </c>
+      <c r="Y27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z27" s="4"/>
+        <v>-25</v>
+      </c>
+      <c r="Z27" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
@@ -4643,56 +4659,56 @@
       </c>
       <c r="E75" s="10">
         <f>SUM(D13:D72)</f>
-        <v>-107.5</v>
+        <v>-102.5</v>
       </c>
       <c r="G75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(G13:G72)</f>
-        <v>-25</v>
+        <v>-45</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K75" s="10">
         <f>SUM(J13:J72)</f>
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N75" s="10">
         <f>SUM(M13:M72)</f>
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q75" s="10">
         <f>SUM(P13:P72)</f>
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="S75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T75" s="10">
         <f>SUM(S13:S72)</f>
-        <v>-120</v>
+        <v>-135</v>
       </c>
       <c r="V75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W75" s="10">
         <f>SUM(V13:V72)</f>
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="Y75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z75" s="10">
         <f>SUM(Y13:Y72)</f>
-        <v>-162.5</v>
+        <v>-187.5</v>
       </c>
       <c r="AA75" s="1">
         <f>SUM(E75,H75,K75,N75,Q75,T75,W75,Z75)</f>

</xml_diff>

<commit_message>
Contest 16 DC vs KKR
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7CA9BA-F2B4-0547-95D1-05C94CEF9EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A25AAEBF-9F9D-BE43-BA2A-328B693A3E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-49020" yWindow="-2500" windowWidth="47880" windowHeight="26560" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2355,46 +2355,60 @@
       <c r="C28" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="D28" s="3" t="str">
+      <c r="D28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E28" s="1"/>
-      <c r="G28" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="E28" s="1">
+        <v>50</v>
+      </c>
+      <c r="G28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H28" s="1"/>
-      <c r="J28" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H28" s="1">
+        <v>60</v>
+      </c>
+      <c r="J28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K28" s="1"/>
-      <c r="M28" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N28" s="1"/>
-      <c r="P28" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="K28" s="1">
+        <v>40</v>
+      </c>
+      <c r="M28" s="3">
+        <v>35</v>
+      </c>
+      <c r="N28" s="1">
+        <v>100</v>
+      </c>
+      <c r="P28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q28" s="1"/>
-      <c r="S28" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q28" s="1">
+        <v>20</v>
+      </c>
+      <c r="S28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T28" s="1"/>
-      <c r="V28" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="T28" s="1">
+        <v>30</v>
+      </c>
+      <c r="V28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W28" s="1"/>
-      <c r="Y28" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Z28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z28" s="1"/>
+        <v>-25</v>
+      </c>
+      <c r="W28" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="3">
+        <v>35</v>
+      </c>
+      <c r="Z28" s="1">
+        <v>100</v>
+      </c>
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
@@ -4659,56 +4673,56 @@
       </c>
       <c r="E75" s="10">
         <f>SUM(D13:D72)</f>
-        <v>-102.5</v>
+        <v>-107.5</v>
       </c>
       <c r="G75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(G13:G72)</f>
-        <v>-45</v>
+        <v>-40</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K75" s="10">
         <f>SUM(J13:J72)</f>
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N75" s="10">
         <f>SUM(M13:M72)</f>
-        <v>110</v>
+        <v>145</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q75" s="10">
         <f>SUM(P13:P72)</f>
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="S75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T75" s="10">
         <f>SUM(S13:S72)</f>
-        <v>-135</v>
+        <v>-150</v>
       </c>
       <c r="V75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W75" s="10">
         <f>SUM(V13:V72)</f>
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="Y75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z75" s="10">
         <f>SUM(Y13:Y72)</f>
-        <v>-187.5</v>
+        <v>-152.5</v>
       </c>
       <c r="AA75" s="1">
         <f>SUM(E75,H75,K75,N75,Q75,T75,W75,Z75)</f>

</xml_diff>

<commit_message>
Contest 17 GT vs PBKS
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A25AAEBF-9F9D-BE43-BA2A-328B693A3E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD354168-5268-694E-A3A1-C837CEA6A20B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -446,13 +446,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1256,38 +1256,38 @@
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="18"/>
-      <c r="G11" s="19" t="s">
+      <c r="E11" s="20"/>
+      <c r="G11" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="20"/>
-      <c r="J11" s="19" t="s">
+      <c r="H11" s="19"/>
+      <c r="J11" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="K11" s="20"/>
-      <c r="M11" s="19" t="s">
+      <c r="K11" s="19"/>
+      <c r="M11" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="N11" s="20"/>
-      <c r="P11" s="19" t="s">
+      <c r="N11" s="19"/>
+      <c r="P11" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="Q11" s="20"/>
-      <c r="S11" s="19" t="s">
+      <c r="Q11" s="19"/>
+      <c r="S11" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="T11" s="20"/>
-      <c r="V11" s="19" t="s">
+      <c r="T11" s="19"/>
+      <c r="V11" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="W11" s="20"/>
-      <c r="Y11" s="19" t="s">
+      <c r="W11" s="19"/>
+      <c r="Y11" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="Z11" s="20"/>
+      <c r="Z11" s="19"/>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
@@ -2420,46 +2420,62 @@
       <c r="C29" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D29" s="3" t="str">
+      <c r="D29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E29" s="1"/>
-      <c r="G29" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E29" s="1">
+        <v>70</v>
+      </c>
+      <c r="G29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H29" s="1"/>
-      <c r="J29" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="H29" s="1">
+        <v>0</v>
+      </c>
+      <c r="J29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K29" s="1"/>
-      <c r="M29" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="K29" s="1">
+        <v>40</v>
+      </c>
+      <c r="M29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N29" s="1"/>
-      <c r="P29" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N29" s="1">
+        <v>100</v>
+      </c>
+      <c r="P29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q29" s="1"/>
-      <c r="S29" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="Q29" s="1">
+        <v>50</v>
+      </c>
+      <c r="S29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T29" s="1"/>
-      <c r="V29" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T29" s="1">
+        <v>60</v>
+      </c>
+      <c r="V29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W29" s="1"/>
-      <c r="Y29" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W29" s="1">
+        <v>30</v>
+      </c>
+      <c r="Y29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z29" s="1"/>
+        <v>-20</v>
+      </c>
+      <c r="Z29" s="1">
+        <v>20</v>
+      </c>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
@@ -4673,56 +4689,56 @@
       </c>
       <c r="E75" s="10">
         <f>SUM(D13:D72)</f>
-        <v>-107.5</v>
+        <v>-87.5</v>
       </c>
       <c r="G75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(G13:G72)</f>
-        <v>-40</v>
+        <v>-65</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K75" s="10">
         <f>SUM(J13:J72)</f>
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N75" s="10">
         <f>SUM(M13:M72)</f>
-        <v>145</v>
+        <v>195</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q75" s="10">
         <f>SUM(P13:P72)</f>
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="S75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T75" s="10">
         <f>SUM(S13:S72)</f>
-        <v>-150</v>
+        <v>-145</v>
       </c>
       <c r="V75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W75" s="10">
         <f>SUM(V13:V72)</f>
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="Y75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z75" s="10">
         <f>SUM(Y13:Y72)</f>
-        <v>-152.5</v>
+        <v>-172.5</v>
       </c>
       <c r="AA75" s="1">
         <f>SUM(E75,H75,K75,N75,Q75,T75,W75,Z75)</f>
@@ -4732,15 +4748,15 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="9">
+    <mergeCell ref="I2:X8"/>
+    <mergeCell ref="S11:T11"/>
+    <mergeCell ref="P11:Q11"/>
+    <mergeCell ref="V11:W11"/>
     <mergeCell ref="Y11:Z11"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="J11:K11"/>
     <mergeCell ref="M11:N11"/>
-    <mergeCell ref="I2:X8"/>
-    <mergeCell ref="S11:T11"/>
-    <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="V11:W11"/>
   </mergeCells>
   <conditionalFormatting sqref="E75">
     <cfRule type="cellIs" dxfId="26" priority="141" operator="greaterThan">

</xml_diff>

<commit_message>
Contest 18 through 21
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD354168-5268-694E-A3A1-C837CEA6A20B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87F52B2A-B81E-504C-9105-FDBD0FE89B2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="28300" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2487,46 +2487,62 @@
       <c r="C30" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="D30" s="3" t="str">
+      <c r="D30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E30" s="1"/>
-      <c r="G30" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="E30" s="1">
+        <v>0</v>
+      </c>
+      <c r="G30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H30" s="1"/>
-      <c r="J30" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="H30" s="1">
+        <v>30</v>
+      </c>
+      <c r="J30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K30" s="1"/>
-      <c r="M30" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="K30" s="1">
+        <v>70</v>
+      </c>
+      <c r="M30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N30" s="1"/>
-      <c r="P30" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="N30" s="1">
+        <v>20</v>
+      </c>
+      <c r="P30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q30" s="1"/>
-      <c r="S30" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q30" s="1">
+        <v>100</v>
+      </c>
+      <c r="S30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T30" s="1"/>
-      <c r="V30" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T30" s="1">
+        <v>60</v>
+      </c>
+      <c r="V30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W30" s="1"/>
-      <c r="Y30" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="W30" s="1">
+        <v>40</v>
+      </c>
+      <c r="Y30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z30" s="1"/>
+        <v>-5</v>
+      </c>
+      <c r="Z30" s="1">
+        <v>50</v>
+      </c>
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
@@ -2538,46 +2554,60 @@
       <c r="C31" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="D31" s="3" t="str">
+      <c r="D31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E31" s="1"/>
-      <c r="G31" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E31" s="1">
+        <v>70</v>
+      </c>
+      <c r="G31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H31" s="1"/>
-      <c r="J31" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="H31" s="1">
+        <v>40</v>
+      </c>
+      <c r="J31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K31" s="1"/>
-      <c r="M31" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="K31" s="1">
+        <v>0</v>
+      </c>
+      <c r="M31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N31" s="1"/>
-      <c r="P31" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N31" s="1">
+        <v>100</v>
+      </c>
+      <c r="P31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q31" s="1"/>
-      <c r="S31" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(T31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T31" s="1"/>
-      <c r="V31" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q31" s="1">
+        <v>30</v>
+      </c>
+      <c r="S31" s="3">
+        <v>0</v>
+      </c>
+      <c r="T31" s="1">
+        <v>60</v>
+      </c>
+      <c r="V31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W31" s="1"/>
-      <c r="Y31" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Z31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z31" s="1"/>
+        <v>-20</v>
+      </c>
+      <c r="W31" s="1">
+        <v>20</v>
+      </c>
+      <c r="Y31" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="1">
+        <v>60</v>
+      </c>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
@@ -2589,46 +2619,60 @@
       <c r="C32" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="D32" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E32" s="1"/>
-      <c r="G32" s="3" t="str">
+      <c r="D32" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="E32" s="1">
+        <v>20</v>
+      </c>
+      <c r="G32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H32" s="1"/>
-      <c r="J32" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H32" s="1">
+        <v>60</v>
+      </c>
+      <c r="J32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K32" s="1"/>
-      <c r="M32" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N32" s="1"/>
-      <c r="P32" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K32" s="1">
+        <v>30</v>
+      </c>
+      <c r="M32" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="N32" s="1">
+        <v>20</v>
+      </c>
+      <c r="P32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q32" s="1"/>
-      <c r="S32" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="Q32" s="1">
+        <v>50</v>
+      </c>
+      <c r="S32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T32" s="1"/>
-      <c r="V32" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="T32" s="1">
+        <v>40</v>
+      </c>
+      <c r="V32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W32" s="1"/>
-      <c r="Y32" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="W32" s="1">
+        <v>70</v>
+      </c>
+      <c r="Y32" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z32, ($Z32,$W32,$T32,$Q32,$N32,$K32,$H32,$E32), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z32" s="1"/>
+        <v>50</v>
+      </c>
+      <c r="Z32" s="1">
+        <v>100</v>
+      </c>
     </row>
     <row r="33" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
@@ -2640,46 +2684,62 @@
       <c r="C33" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="D33" s="3" t="str">
+      <c r="D33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E33" s="1"/>
-      <c r="G33" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="E33" s="1">
+        <v>30</v>
+      </c>
+      <c r="G33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H33" s="1"/>
-      <c r="J33" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="H33" s="1">
+        <v>40</v>
+      </c>
+      <c r="J33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K33" s="1"/>
-      <c r="M33" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="K33" s="1">
+        <v>50</v>
+      </c>
+      <c r="M33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N33" s="1"/>
-      <c r="P33" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N33" s="1">
+        <v>100</v>
+      </c>
+      <c r="P33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q33" s="1"/>
-      <c r="S33" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q33" s="1">
+        <v>20</v>
+      </c>
+      <c r="S33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T33" s="1"/>
-      <c r="V33" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="T33" s="1">
+        <v>0</v>
+      </c>
+      <c r="V33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W33" s="1"/>
-      <c r="Y33" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="W33" s="1">
+        <v>60</v>
+      </c>
+      <c r="Y33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z33" s="1"/>
+        <v>20</v>
+      </c>
+      <c r="Z33" s="1">
+        <v>70</v>
+      </c>
     </row>
     <row r="34" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
@@ -4689,56 +4749,56 @@
       </c>
       <c r="E75" s="10">
         <f>SUM(D13:D72)</f>
-        <v>-87.5</v>
+        <v>-130</v>
       </c>
       <c r="G75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(G13:G72)</f>
-        <v>-65</v>
+        <v>-95</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K75" s="10">
         <f>SUM(J13:J72)</f>
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N75" s="10">
         <f>SUM(M13:M72)</f>
-        <v>195</v>
+        <v>252.5</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q75" s="10">
         <f>SUM(P13:P72)</f>
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="S75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T75" s="10">
         <f>SUM(S13:S72)</f>
-        <v>-145</v>
+        <v>-175</v>
       </c>
       <c r="V75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W75" s="10">
         <f>SUM(V13:V72)</f>
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="Y75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z75" s="10">
         <f>SUM(Y13:Y72)</f>
-        <v>-172.5</v>
+        <v>-107.5</v>
       </c>
       <c r="AA75" s="1">
         <f>SUM(E75,H75,K75,N75,Q75,T75,W75,Z75)</f>

</xml_diff>

<commit_message>
Contest 22 CSK vs KKR
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87F52B2A-B81E-504C-9105-FDBD0FE89B2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE4BFA2-1501-CA45-A7AD-32410C693E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="28300" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="26800" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2751,46 +2751,62 @@
       <c r="C34" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="3" t="str">
+      <c r="D34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E34" s="1"/>
-      <c r="G34" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="E34" s="1">
+        <v>60</v>
+      </c>
+      <c r="G34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H34" s="1"/>
-      <c r="J34" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="H34" s="1">
+        <v>100</v>
+      </c>
+      <c r="J34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K34" s="1"/>
-      <c r="M34" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K34" s="1">
+        <v>30</v>
+      </c>
+      <c r="M34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N34" s="1"/>
-      <c r="P34" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N34" s="1">
+        <v>70</v>
+      </c>
+      <c r="P34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q34" s="1"/>
-      <c r="S34" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="Q34" s="1">
+        <v>50</v>
+      </c>
+      <c r="S34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T34" s="1"/>
-      <c r="V34" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="T34" s="1">
+        <v>20</v>
+      </c>
+      <c r="V34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W34" s="1"/>
-      <c r="Y34" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="W34" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z34" s="1"/>
+        <v>-10</v>
+      </c>
+      <c r="Z34" s="1">
+        <v>40</v>
+      </c>
     </row>
     <row r="35" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
@@ -4749,56 +4765,56 @@
       </c>
       <c r="E75" s="10">
         <f>SUM(D13:D72)</f>
-        <v>-130</v>
+        <v>-125</v>
       </c>
       <c r="G75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(G13:G72)</f>
-        <v>-95</v>
+        <v>-45</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K75" s="10">
         <f>SUM(J13:J72)</f>
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N75" s="10">
         <f>SUM(M13:M72)</f>
-        <v>252.5</v>
+        <v>272.5</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q75" s="10">
         <f>SUM(P13:P72)</f>
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="S75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T75" s="10">
         <f>SUM(S13:S72)</f>
-        <v>-175</v>
+        <v>-195</v>
       </c>
       <c r="V75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W75" s="10">
         <f>SUM(V13:V72)</f>
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="Y75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z75" s="10">
         <f>SUM(Y13:Y72)</f>
-        <v>-107.5</v>
+        <v>-117.5</v>
       </c>
       <c r="AA75" s="1">
         <f>SUM(E75,H75,K75,N75,Q75,T75,W75,Z75)</f>

</xml_diff>

<commit_message>
Contest 23 PBKS vs SRH
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE4BFA2-1501-CA45-A7AD-32410C693E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851C93B2-EE12-F94F-A627-E0C64C999A20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="26800" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="27580" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2818,46 +2818,62 @@
       <c r="C35" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="D35" s="3" t="str">
+      <c r="D35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E35" s="1"/>
-      <c r="G35" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E35" s="1">
+        <v>40</v>
+      </c>
+      <c r="G35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H35" s="1"/>
-      <c r="J35" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="H35" s="1">
+        <v>70</v>
+      </c>
+      <c r="J35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K35" s="1"/>
-      <c r="M35" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K35" s="1">
+        <v>20</v>
+      </c>
+      <c r="M35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N35" s="1"/>
-      <c r="P35" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="N35" s="1">
+        <v>60</v>
+      </c>
+      <c r="P35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q35" s="1"/>
-      <c r="S35" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q35" s="1">
+        <v>30</v>
+      </c>
+      <c r="S35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T35" s="1"/>
-      <c r="V35" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="T35" s="1">
+        <v>100</v>
+      </c>
+      <c r="V35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W35" s="1"/>
-      <c r="Y35" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="W35" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z35" s="1"/>
+        <v>-5</v>
+      </c>
+      <c r="Z35" s="1">
+        <v>50</v>
+      </c>
     </row>
     <row r="36" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
@@ -4765,56 +4781,56 @@
       </c>
       <c r="E75" s="10">
         <f>SUM(D13:D72)</f>
-        <v>-125</v>
+        <v>-135</v>
       </c>
       <c r="G75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(G13:G72)</f>
-        <v>-45</v>
+        <v>-25</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K75" s="10">
         <f>SUM(J13:J72)</f>
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N75" s="10">
         <f>SUM(M13:M72)</f>
-        <v>272.5</v>
+        <v>277.5</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q75" s="10">
         <f>SUM(P13:P72)</f>
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="S75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T75" s="10">
         <f>SUM(S13:S72)</f>
-        <v>-195</v>
+        <v>-145</v>
       </c>
       <c r="V75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W75" s="10">
         <f>SUM(V13:V72)</f>
-        <v>130</v>
+        <v>105</v>
       </c>
       <c r="Y75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z75" s="10">
         <f>SUM(Y13:Y72)</f>
-        <v>-117.5</v>
+        <v>-122.5</v>
       </c>
       <c r="AA75" s="1">
         <f>SUM(E75,H75,K75,N75,Q75,T75,W75,Z75)</f>

</xml_diff>

<commit_message>
Contest 24 RR vs GT
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851C93B2-EE12-F94F-A627-E0C64C999A20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B6E49B0-0415-224F-8F12-C13ED186B8CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="27580" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2885,46 +2885,58 @@
       <c r="C36" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="D36" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E36" s="1"/>
-      <c r="G36" s="3" t="str">
+      <c r="D36" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="E36" s="1">
+        <v>20</v>
+      </c>
+      <c r="G36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H36" s="1"/>
-      <c r="J36" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K36" s="1"/>
-      <c r="M36" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N36" s="1"/>
-      <c r="P36" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="H36" s="1">
+        <v>30</v>
+      </c>
+      <c r="J36" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="K36" s="1">
+        <v>20</v>
+      </c>
+      <c r="M36" s="3">
+        <v>-7.5</v>
+      </c>
+      <c r="N36" s="1">
+        <v>50</v>
+      </c>
+      <c r="P36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q36" s="1"/>
-      <c r="S36" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(T36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T36" s="1"/>
-      <c r="V36" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q36" s="1">
+        <v>70</v>
+      </c>
+      <c r="S36" s="3">
+        <v>-7.5</v>
+      </c>
+      <c r="T36" s="1">
+        <v>50</v>
+      </c>
+      <c r="V36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W36" s="1"/>
-      <c r="Y36" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="W36" s="1">
+        <v>60</v>
+      </c>
+      <c r="Y36" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z36, ($Z36,$W36,$T36,$Q36,$N36,$K36,$H36,$E36), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z36" s="1"/>
+        <v>50</v>
+      </c>
+      <c r="Z36" s="1">
+        <v>100</v>
+      </c>
     </row>
     <row r="37" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
@@ -4781,56 +4793,56 @@
       </c>
       <c r="E75" s="10">
         <f>SUM(D13:D72)</f>
-        <v>-135</v>
+        <v>-157.5</v>
       </c>
       <c r="G75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(G13:G72)</f>
-        <v>-25</v>
+        <v>-40</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K75" s="10">
         <f>SUM(J13:J72)</f>
-        <v>30</v>
+        <v>7.5</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N75" s="10">
         <f>SUM(M13:M72)</f>
-        <v>277.5</v>
+        <v>270</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q75" s="10">
         <f>SUM(P13:P72)</f>
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="S75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T75" s="10">
         <f>SUM(S13:S72)</f>
-        <v>-145</v>
+        <v>-152.5</v>
       </c>
       <c r="V75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W75" s="10">
         <f>SUM(V13:V72)</f>
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="Y75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z75" s="10">
         <f>SUM(Y13:Y72)</f>
-        <v>-122.5</v>
+        <v>-72.5</v>
       </c>
       <c r="AA75" s="1">
         <f>SUM(E75,H75,K75,N75,Q75,T75,W75,Z75)</f>

</xml_diff>

<commit_message>
Contest 25 MI vs RCB
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B6E49B0-0415-224F-8F12-C13ED186B8CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D3E61A-9C22-294A-967F-68E88D0B8690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="27580" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2948,46 +2948,62 @@
       <c r="C37" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="D37" s="3" t="str">
+      <c r="D37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E37" s="1"/>
-      <c r="G37" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E37" s="1">
+        <v>40</v>
+      </c>
+      <c r="G37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H37" s="1"/>
-      <c r="J37" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="H37" s="1">
+        <v>30</v>
+      </c>
+      <c r="J37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K37" s="1"/>
-      <c r="M37" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K37" s="1">
+        <v>20</v>
+      </c>
+      <c r="M37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N37" s="1"/>
-      <c r="P37" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="N37" s="1">
+        <v>60</v>
+      </c>
+      <c r="P37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q37" s="1"/>
-      <c r="S37" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Q37" s="1">
+        <v>0</v>
+      </c>
+      <c r="S37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T37" s="1"/>
-      <c r="V37" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="T37" s="1">
+        <v>100</v>
+      </c>
+      <c r="V37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W37" s="1"/>
-      <c r="Y37" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="W37" s="1">
+        <v>70</v>
+      </c>
+      <c r="Y37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z37" s="1"/>
+        <v>-5</v>
+      </c>
+      <c r="Z37" s="1">
+        <v>50</v>
+      </c>
     </row>
     <row r="38" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
@@ -4793,56 +4809,56 @@
       </c>
       <c r="E75" s="10">
         <f>SUM(D13:D72)</f>
-        <v>-157.5</v>
+        <v>-167.5</v>
       </c>
       <c r="G75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H75" s="10">
         <f>SUM(G13:G72)</f>
-        <v>-40</v>
+        <v>-55</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K75" s="10">
         <f>SUM(J13:J72)</f>
-        <v>7.5</v>
+        <v>-12.5</v>
       </c>
       <c r="M75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N75" s="10">
         <f>SUM(M13:M72)</f>
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="P75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q75" s="10">
         <f>SUM(P13:P72)</f>
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="S75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T75" s="10">
         <f>SUM(S13:S72)</f>
-        <v>-152.5</v>
+        <v>-102.5</v>
       </c>
       <c r="V75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W75" s="10">
         <f>SUM(V13:V72)</f>
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="Y75" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z75" s="10">
         <f>SUM(Y13:Y72)</f>
-        <v>-72.5</v>
+        <v>-77.5</v>
       </c>
       <c r="AA75" s="1">
         <f>SUM(E75,H75,K75,N75,Q75,T75,W75,Z75)</f>

</xml_diff>

<commit_message>
Contest 26 through 29
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D3E61A-9C22-294A-967F-68E88D0B8690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABBB209E-1AC5-0A40-A060-B8724B7B1438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="27580" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="27820" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="113">
   <si>
     <t>Points</t>
   </si>
@@ -249,6 +249,138 @@
   </si>
   <si>
     <t>LSG vs DC</t>
+  </si>
+  <si>
+    <t>PBKS vs RR</t>
+  </si>
+  <si>
+    <t>KKR vs LSG</t>
+  </si>
+  <si>
+    <t>MI vs CSK</t>
+  </si>
+  <si>
+    <t>RCB vs SRH</t>
+  </si>
+  <si>
+    <t>KKR vs RR</t>
+  </si>
+  <si>
+    <t>GT vs DC</t>
+  </si>
+  <si>
+    <t>PBKS vs MI</t>
+  </si>
+  <si>
+    <t>LSG vs CSK</t>
+  </si>
+  <si>
+    <t>DC vs SRH</t>
+  </si>
+  <si>
+    <t>KKR vs RCB</t>
+  </si>
+  <si>
+    <t>PBKS vs GT</t>
+  </si>
+  <si>
+    <t>RR vs MI</t>
+  </si>
+  <si>
+    <t>CSK vs LSG</t>
+  </si>
+  <si>
+    <t>DC vs GT</t>
+  </si>
+  <si>
+    <t>SRH vs RCB</t>
+  </si>
+  <si>
+    <t>KKR vs PBKS</t>
+  </si>
+  <si>
+    <t>DC vs MI</t>
+  </si>
+  <si>
+    <t>LSG vs RR</t>
+  </si>
+  <si>
+    <t>GT vs RCB</t>
+  </si>
+  <si>
+    <t>CSK vs SRH</t>
+  </si>
+  <si>
+    <t>KKR vs DC</t>
+  </si>
+  <si>
+    <t>LSG vs MI</t>
+  </si>
+  <si>
+    <t>CSK vs PBKS</t>
+  </si>
+  <si>
+    <t>SRH vs RR</t>
+  </si>
+  <si>
+    <t>MI vs KKR</t>
+  </si>
+  <si>
+    <t>RCB vs GT</t>
+  </si>
+  <si>
+    <t>PBKS vs CSK</t>
+  </si>
+  <si>
+    <t>LSG vs KKR</t>
+  </si>
+  <si>
+    <t>MI vs SRH</t>
+  </si>
+  <si>
+    <t>DC vs RR</t>
+  </si>
+  <si>
+    <t>SRH vs LSG</t>
+  </si>
+  <si>
+    <t>PBKS vs RCB</t>
+  </si>
+  <si>
+    <t>GT vs CSK</t>
+  </si>
+  <si>
+    <t>KKR vs MI</t>
+  </si>
+  <si>
+    <t>CSK vs RR</t>
+  </si>
+  <si>
+    <t>RCB vs DC</t>
+  </si>
+  <si>
+    <t>GT vs KKR</t>
+  </si>
+  <si>
+    <t>DC vs LSG</t>
+  </si>
+  <si>
+    <t>RR vs PBKS</t>
+  </si>
+  <si>
+    <t>SRH vs GT</t>
+  </si>
+  <si>
+    <t>MI vs LSG</t>
+  </si>
+  <si>
+    <t>RCB vs CSK</t>
+  </si>
+  <si>
+    <t>SRH vs PBKS</t>
+  </si>
+  <si>
+    <t>RR vs KKR</t>
   </si>
 </sst>
 </file>
@@ -496,6 +628,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -616,36 +768,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -731,6 +853,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1049,7 +1181,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BE9CB7-B9A7-B347-86F0-C3EB9B5BFBBD}">
-  <dimension ref="A1:AA75"/>
+  <dimension ref="A1:AA89"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
@@ -3015,46 +3147,62 @@
       <c r="C38" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="D38" s="3" t="str">
+      <c r="D38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E38" s="1"/>
-      <c r="G38" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="E38" s="1">
+        <v>0</v>
+      </c>
+      <c r="G38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H38" s="1"/>
-      <c r="J38" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H38" s="1">
+        <v>60</v>
+      </c>
+      <c r="J38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K38" s="1"/>
-      <c r="M38" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="K38" s="1">
+        <v>100</v>
+      </c>
+      <c r="M38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N38" s="1"/>
-      <c r="P38" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N38" s="1">
+        <v>70</v>
+      </c>
+      <c r="P38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q38" s="1"/>
-      <c r="S38" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Q38" s="1">
+        <v>40</v>
+      </c>
+      <c r="S38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T38" s="1"/>
-      <c r="V38" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="T38" s="1">
+        <v>30</v>
+      </c>
+      <c r="V38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W38" s="1"/>
-      <c r="Y38" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="W38" s="1">
+        <v>50</v>
+      </c>
+      <c r="Y38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z38" s="1"/>
+        <v>-20</v>
+      </c>
+      <c r="Z38" s="1">
+        <v>20</v>
+      </c>
     </row>
     <row r="39" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
@@ -3063,47 +3211,63 @@
       <c r="B39" s="1">
         <v>1</v>
       </c>
-      <c r="C39" s="14"/>
-      <c r="D39" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E39" s="1"/>
-      <c r="G39" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H39" s="1"/>
-      <c r="J39" s="3" t="str">
+      <c r="C39" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D39" s="3">
+        <v>35</v>
+      </c>
+      <c r="E39" s="1">
+        <v>100</v>
+      </c>
+      <c r="G39" s="3">
+        <v>35</v>
+      </c>
+      <c r="H39" s="1">
+        <v>100</v>
+      </c>
+      <c r="J39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K39" s="1"/>
-      <c r="M39" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K39" s="1">
+        <v>30</v>
+      </c>
+      <c r="M39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N39" s="1"/>
-      <c r="P39" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="N39" s="1">
+        <v>50</v>
+      </c>
+      <c r="P39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q39" s="1"/>
-      <c r="S39" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q39" s="1">
+        <v>60</v>
+      </c>
+      <c r="S39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T39" s="1"/>
-      <c r="V39" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="T39" s="1">
+        <v>40</v>
+      </c>
+      <c r="V39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W39" s="1"/>
-      <c r="Y39" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="W39" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y39" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z39, ($Z39,$W39,$T39,$Q39,$N39,$K39,$H39,$E39), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z39" s="1"/>
+        <v>-20</v>
+      </c>
+      <c r="Z39" s="1">
+        <v>20</v>
+      </c>
     </row>
     <row r="40" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
@@ -3112,47 +3276,65 @@
       <c r="B40" s="1">
         <v>1</v>
       </c>
-      <c r="C40" s="14"/>
-      <c r="D40" s="3" t="str">
+      <c r="C40" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="D40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E40" s="1"/>
-      <c r="G40" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="E40" s="1">
+        <v>100</v>
+      </c>
+      <c r="G40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H40" s="1"/>
-      <c r="J40" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="H40" s="1">
+        <v>70</v>
+      </c>
+      <c r="J40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K40" s="1"/>
-      <c r="M40" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="K40" s="1">
+        <v>0</v>
+      </c>
+      <c r="M40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N40" s="1"/>
-      <c r="P40" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="N40" s="1">
+        <v>20</v>
+      </c>
+      <c r="P40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q40" s="1"/>
-      <c r="S40" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Q40" s="1">
+        <v>40</v>
+      </c>
+      <c r="S40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T40" s="1"/>
-      <c r="V40" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T40" s="1">
+        <v>60</v>
+      </c>
+      <c r="V40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W40" s="1"/>
-      <c r="Y40" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="W40" s="1">
+        <v>50</v>
+      </c>
+      <c r="Y40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z40" s="1"/>
+        <v>-15</v>
+      </c>
+      <c r="Z40" s="1">
+        <v>30</v>
+      </c>
     </row>
     <row r="41" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
@@ -3161,47 +3343,65 @@
       <c r="B41" s="1">
         <v>1</v>
       </c>
-      <c r="C41" s="14"/>
-      <c r="D41" s="3" t="str">
+      <c r="C41" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E41" s="1"/>
-      <c r="G41" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E41" s="1">
+        <v>40</v>
+      </c>
+      <c r="G41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H41" s="1"/>
-      <c r="J41" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="H41" s="1">
+        <v>50</v>
+      </c>
+      <c r="J41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K41" s="1"/>
-      <c r="M41" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K41" s="1">
+        <v>20</v>
+      </c>
+      <c r="M41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N41" s="1"/>
-      <c r="P41" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N41" s="1">
+        <v>0</v>
+      </c>
+      <c r="P41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q41" s="1"/>
-      <c r="S41" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q41" s="1">
+        <v>60</v>
+      </c>
+      <c r="S41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T41" s="1"/>
-      <c r="V41" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T41" s="1">
+        <v>70</v>
+      </c>
+      <c r="V41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W41" s="1"/>
-      <c r="Y41" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W41" s="1">
+        <v>30</v>
+      </c>
+      <c r="Y41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z41" s="1"/>
+        <v>50</v>
+      </c>
+      <c r="Z41" s="1">
+        <v>100</v>
+      </c>
     </row>
     <row r="42" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
@@ -3210,7 +3410,9 @@
       <c r="B42" s="1">
         <v>1</v>
       </c>
-      <c r="C42" s="14"/>
+      <c r="C42" s="14" t="s">
+        <v>72</v>
+      </c>
       <c r="D42" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3259,7 +3461,9 @@
       <c r="B43" s="1">
         <v>1</v>
       </c>
-      <c r="C43" s="14"/>
+      <c r="C43" s="14" t="s">
+        <v>73</v>
+      </c>
       <c r="D43" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3308,7 +3512,9 @@
       <c r="B44" s="1">
         <v>1</v>
       </c>
-      <c r="C44" s="14"/>
+      <c r="C44" s="14" t="s">
+        <v>74</v>
+      </c>
       <c r="D44" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3357,7 +3563,9 @@
       <c r="B45" s="1">
         <v>1</v>
       </c>
-      <c r="C45" s="14"/>
+      <c r="C45" s="14" t="s">
+        <v>75</v>
+      </c>
       <c r="D45" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3406,7 +3614,9 @@
       <c r="B46" s="1">
         <v>1</v>
       </c>
-      <c r="C46" s="14"/>
+      <c r="C46" s="14" t="s">
+        <v>76</v>
+      </c>
       <c r="D46" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3455,7 +3665,9 @@
       <c r="B47" s="1">
         <v>1</v>
       </c>
-      <c r="C47" s="14"/>
+      <c r="C47" s="14" t="s">
+        <v>77</v>
+      </c>
       <c r="D47" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3504,7 +3716,9 @@
       <c r="B48" s="1">
         <v>1</v>
       </c>
-      <c r="C48" s="14"/>
+      <c r="C48" s="14" t="s">
+        <v>78</v>
+      </c>
       <c r="D48" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3553,7 +3767,9 @@
       <c r="B49" s="1">
         <v>1</v>
       </c>
-      <c r="C49" s="14"/>
+      <c r="C49" s="14" t="s">
+        <v>79</v>
+      </c>
       <c r="D49" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3602,7 +3818,9 @@
       <c r="B50" s="1">
         <v>1</v>
       </c>
-      <c r="C50" s="14"/>
+      <c r="C50" s="14" t="s">
+        <v>80</v>
+      </c>
       <c r="D50" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3651,7 +3869,9 @@
       <c r="B51" s="1">
         <v>1</v>
       </c>
-      <c r="C51" s="14"/>
+      <c r="C51" s="14" t="s">
+        <v>81</v>
+      </c>
       <c r="D51" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3700,7 +3920,9 @@
       <c r="B52" s="1">
         <v>1</v>
       </c>
-      <c r="C52" s="14"/>
+      <c r="C52" s="14" t="s">
+        <v>82</v>
+      </c>
       <c r="D52" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3749,7 +3971,9 @@
       <c r="B53" s="1">
         <v>1</v>
       </c>
-      <c r="C53" s="14"/>
+      <c r="C53" s="14" t="s">
+        <v>83</v>
+      </c>
       <c r="D53" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3798,7 +4022,9 @@
       <c r="B54" s="1">
         <v>1</v>
       </c>
-      <c r="C54" s="14"/>
+      <c r="C54" s="14" t="s">
+        <v>84</v>
+      </c>
       <c r="D54" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3847,7 +4073,9 @@
       <c r="B55" s="1">
         <v>1</v>
       </c>
-      <c r="C55" s="14"/>
+      <c r="C55" s="14" t="s">
+        <v>85</v>
+      </c>
       <c r="D55" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3896,7 +4124,9 @@
       <c r="B56" s="1">
         <v>1</v>
       </c>
-      <c r="C56" s="14"/>
+      <c r="C56" s="14" t="s">
+        <v>86</v>
+      </c>
       <c r="D56" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3945,7 +4175,9 @@
       <c r="B57" s="1">
         <v>1</v>
       </c>
-      <c r="C57" s="14"/>
+      <c r="C57" s="14" t="s">
+        <v>87</v>
+      </c>
       <c r="D57" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -3994,7 +4226,9 @@
       <c r="B58" s="1">
         <v>1</v>
       </c>
-      <c r="C58" s="14"/>
+      <c r="C58" s="14" t="s">
+        <v>88</v>
+      </c>
       <c r="D58" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4043,7 +4277,9 @@
       <c r="B59" s="1">
         <v>1</v>
       </c>
-      <c r="C59" s="14"/>
+      <c r="C59" s="14" t="s">
+        <v>89</v>
+      </c>
       <c r="D59" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4092,7 +4328,9 @@
       <c r="B60" s="1">
         <v>1</v>
       </c>
-      <c r="C60" s="14"/>
+      <c r="C60" s="14" t="s">
+        <v>90</v>
+      </c>
       <c r="D60" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4141,7 +4379,9 @@
       <c r="B61" s="1">
         <v>1</v>
       </c>
-      <c r="C61" s="14"/>
+      <c r="C61" s="14" t="s">
+        <v>91</v>
+      </c>
       <c r="D61" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4190,7 +4430,9 @@
       <c r="B62" s="1">
         <v>1</v>
       </c>
-      <c r="C62" s="14"/>
+      <c r="C62" s="14" t="s">
+        <v>92</v>
+      </c>
       <c r="D62" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4239,7 +4481,9 @@
       <c r="B63" s="1">
         <v>1</v>
       </c>
-      <c r="C63" s="14"/>
+      <c r="C63" s="14" t="s">
+        <v>93</v>
+      </c>
       <c r="D63" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4288,7 +4532,9 @@
       <c r="B64" s="1">
         <v>1</v>
       </c>
-      <c r="C64" s="14"/>
+      <c r="C64" s="14" t="s">
+        <v>94</v>
+      </c>
       <c r="D64" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4330,14 +4576,16 @@
       </c>
       <c r="Z64" s="1"/>
     </row>
-    <row r="65" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>53</v>
       </c>
       <c r="B65" s="1">
         <v>1</v>
       </c>
-      <c r="C65" s="14"/>
+      <c r="C65" s="14" t="s">
+        <v>95</v>
+      </c>
       <c r="D65" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4379,14 +4627,16 @@
       </c>
       <c r="Z65" s="1"/>
     </row>
-    <row r="66" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>54</v>
       </c>
       <c r="B66" s="1">
         <v>1</v>
       </c>
-      <c r="C66" s="14"/>
+      <c r="C66" s="14" t="s">
+        <v>96</v>
+      </c>
       <c r="D66" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4428,14 +4678,16 @@
       </c>
       <c r="Z66" s="1"/>
     </row>
-    <row r="67" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>55</v>
       </c>
       <c r="B67" s="1">
         <v>1</v>
       </c>
-      <c r="C67" s="14"/>
+      <c r="C67" s="14" t="s">
+        <v>97</v>
+      </c>
       <c r="D67" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4477,14 +4729,16 @@
       </c>
       <c r="Z67" s="1"/>
     </row>
-    <row r="68" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>56</v>
       </c>
       <c r="B68" s="1">
         <v>1</v>
       </c>
-      <c r="C68" s="14"/>
+      <c r="C68" s="14" t="s">
+        <v>98</v>
+      </c>
       <c r="D68" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4526,14 +4780,16 @@
       </c>
       <c r="Z68" s="1"/>
     </row>
-    <row r="69" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A69" s="5" t="s">
-        <v>26</v>
+    <row r="69" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A69" s="1">
+        <v>57</v>
       </c>
       <c r="B69" s="1">
         <v>1</v>
       </c>
-      <c r="C69" s="14"/>
+      <c r="C69" s="14" t="s">
+        <v>99</v>
+      </c>
       <c r="D69" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4575,14 +4831,16 @@
       </c>
       <c r="Z69" s="1"/>
     </row>
-    <row r="70" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A70" s="5" t="s">
-        <v>27</v>
+    <row r="70" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A70" s="1">
+        <v>58</v>
       </c>
       <c r="B70" s="1">
         <v>1</v>
       </c>
-      <c r="C70" s="14"/>
+      <c r="C70" s="14" t="s">
+        <v>100</v>
+      </c>
       <c r="D70" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4624,14 +4882,16 @@
       </c>
       <c r="Z70" s="1"/>
     </row>
-    <row r="71" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A71" s="5" t="s">
-        <v>28</v>
+    <row r="71" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A71" s="1">
+        <v>59</v>
       </c>
       <c r="B71" s="1">
         <v>1</v>
       </c>
-      <c r="C71" s="14"/>
+      <c r="C71" s="14" t="s">
+        <v>101</v>
+      </c>
       <c r="D71" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4673,14 +4933,16 @@
       </c>
       <c r="Z71" s="1"/>
     </row>
-    <row r="72" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A72" s="5" t="s">
-        <v>29</v>
+    <row r="72" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A72" s="1">
+        <v>60</v>
       </c>
       <c r="B72" s="1">
         <v>1</v>
       </c>
-      <c r="C72" s="14"/>
+      <c r="C72" s="14" t="s">
+        <v>102</v>
+      </c>
       <c r="D72" s="3" t="str">
         <f>IF(ISERROR(VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
         <v/>
@@ -4722,146 +4984,852 @@
       </c>
       <c r="Z72" s="1"/>
     </row>
-    <row r="73" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A73" s="5"/>
-      <c r="B73" s="1" t="s">
+    <row r="73" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A73" s="1">
+        <v>61</v>
+      </c>
+      <c r="B73" s="1">
+        <v>1</v>
+      </c>
+      <c r="C73" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="D73" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E73" s="1"/>
+      <c r="G73" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H73" s="1"/>
+      <c r="J73" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K73" s="1"/>
+      <c r="M73" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N73" s="1"/>
+      <c r="P73" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q73" s="1"/>
+      <c r="S73" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T73" s="1"/>
+      <c r="V73" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W73" s="1"/>
+      <c r="Y73" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z73" s="1"/>
+    </row>
+    <row r="74" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A74" s="1">
+        <v>62</v>
+      </c>
+      <c r="B74" s="1">
+        <v>1</v>
+      </c>
+      <c r="C74" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="D74" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E74" s="1"/>
+      <c r="G74" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H74" s="1"/>
+      <c r="J74" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K74" s="1"/>
+      <c r="M74" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N74" s="1"/>
+      <c r="P74" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q74" s="1"/>
+      <c r="S74" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T74" s="1"/>
+      <c r="V74" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W74" s="1"/>
+      <c r="Y74" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z74" s="1"/>
+    </row>
+    <row r="75" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A75" s="1">
+        <v>63</v>
+      </c>
+      <c r="B75" s="1">
+        <v>1</v>
+      </c>
+      <c r="C75" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="D75" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E75" s="1"/>
+      <c r="G75" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H75" s="1"/>
+      <c r="J75" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K75" s="1"/>
+      <c r="M75" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N75" s="1"/>
+      <c r="P75" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q75" s="1"/>
+      <c r="S75" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T75" s="1"/>
+      <c r="V75" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W75" s="1"/>
+      <c r="Y75" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z75" s="1"/>
+    </row>
+    <row r="76" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A76" s="1">
+        <v>64</v>
+      </c>
+      <c r="B76" s="1">
+        <v>1</v>
+      </c>
+      <c r="C76" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="D76" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E76" s="1"/>
+      <c r="G76" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H76" s="1"/>
+      <c r="J76" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K76" s="1"/>
+      <c r="M76" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N76" s="1"/>
+      <c r="P76" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q76" s="1"/>
+      <c r="S76" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T76" s="1"/>
+      <c r="V76" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W76" s="1"/>
+      <c r="Y76" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z76" s="1"/>
+    </row>
+    <row r="77" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A77" s="1">
+        <v>65</v>
+      </c>
+      <c r="B77" s="1">
+        <v>1</v>
+      </c>
+      <c r="C77" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="D77" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E77" s="1"/>
+      <c r="G77" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H77" s="1"/>
+      <c r="J77" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K77" s="1"/>
+      <c r="M77" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N77" s="1"/>
+      <c r="P77" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q77" s="1"/>
+      <c r="S77" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T77" s="1"/>
+      <c r="V77" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W77" s="1"/>
+      <c r="Y77" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z77" s="1"/>
+    </row>
+    <row r="78" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A78" s="1">
+        <v>66</v>
+      </c>
+      <c r="B78" s="1">
+        <v>1</v>
+      </c>
+      <c r="C78" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="D78" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E78" s="1"/>
+      <c r="G78" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H78" s="1"/>
+      <c r="J78" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K78" s="1"/>
+      <c r="M78" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N78" s="1"/>
+      <c r="P78" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q78" s="1"/>
+      <c r="S78" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T78" s="1"/>
+      <c r="V78" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W78" s="1"/>
+      <c r="Y78" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z78" s="1"/>
+    </row>
+    <row r="79" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A79" s="1">
+        <v>67</v>
+      </c>
+      <c r="B79" s="1">
+        <v>1</v>
+      </c>
+      <c r="C79" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="D79" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E79" s="1"/>
+      <c r="G79" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H79" s="1"/>
+      <c r="J79" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K79" s="1"/>
+      <c r="M79" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N79" s="1"/>
+      <c r="P79" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q79" s="1"/>
+      <c r="S79" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T79" s="1"/>
+      <c r="V79" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W79" s="1"/>
+      <c r="Y79" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z79" s="1"/>
+    </row>
+    <row r="80" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A80" s="1">
+        <v>68</v>
+      </c>
+      <c r="B80" s="1">
+        <v>1</v>
+      </c>
+      <c r="C80" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="D80" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E80" s="1"/>
+      <c r="G80" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H80" s="1"/>
+      <c r="J80" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K80" s="1"/>
+      <c r="M80" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N80" s="1"/>
+      <c r="P80" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q80" s="1"/>
+      <c r="S80" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T80" s="1"/>
+      <c r="V80" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W80" s="1"/>
+      <c r="Y80" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z80" s="1"/>
+    </row>
+    <row r="81" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A81" s="1">
+        <v>69</v>
+      </c>
+      <c r="B81" s="1">
+        <v>1</v>
+      </c>
+      <c r="C81" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D81" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E81" s="1"/>
+      <c r="G81" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H81" s="1"/>
+      <c r="J81" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K81" s="1"/>
+      <c r="M81" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N81" s="1"/>
+      <c r="P81" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q81" s="1"/>
+      <c r="S81" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T81" s="1"/>
+      <c r="V81" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W81" s="1"/>
+      <c r="Y81" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z81" s="1"/>
+    </row>
+    <row r="82" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A82" s="1">
+        <v>70</v>
+      </c>
+      <c r="B82" s="1">
+        <v>1</v>
+      </c>
+      <c r="C82" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="D82" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E82" s="1"/>
+      <c r="G82" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H82" s="1"/>
+      <c r="J82" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K82" s="1"/>
+      <c r="M82" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N82" s="1"/>
+      <c r="P82" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q82" s="1"/>
+      <c r="S82" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T82" s="1"/>
+      <c r="V82" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W82" s="1"/>
+      <c r="Y82" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z82" s="1"/>
+    </row>
+    <row r="83" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A83" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B83" s="1">
+        <v>1</v>
+      </c>
+      <c r="C83" s="14"/>
+      <c r="D83" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E83" s="1"/>
+      <c r="G83" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H83" s="1"/>
+      <c r="J83" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K83" s="1"/>
+      <c r="M83" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N83" s="1"/>
+      <c r="P83" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q83" s="1"/>
+      <c r="S83" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T83" s="1"/>
+      <c r="V83" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W83" s="1"/>
+      <c r="Y83" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z83" s="1"/>
+    </row>
+    <row r="84" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A84" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B84" s="1">
+        <v>1</v>
+      </c>
+      <c r="C84" s="14"/>
+      <c r="D84" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E84" s="1"/>
+      <c r="G84" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H84" s="1"/>
+      <c r="J84" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K84" s="1"/>
+      <c r="M84" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N84" s="1"/>
+      <c r="P84" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q84" s="1"/>
+      <c r="S84" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T84" s="1"/>
+      <c r="V84" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W84" s="1"/>
+      <c r="Y84" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z84" s="1"/>
+    </row>
+    <row r="85" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A85" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B85" s="1">
+        <v>1</v>
+      </c>
+      <c r="C85" s="14"/>
+      <c r="D85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E85" s="1"/>
+      <c r="G85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H85" s="1"/>
+      <c r="J85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K85" s="1"/>
+      <c r="M85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N85" s="1"/>
+      <c r="P85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q85" s="1"/>
+      <c r="S85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T85" s="1"/>
+      <c r="V85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W85" s="1"/>
+      <c r="Y85" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z85" s="1"/>
+    </row>
+    <row r="86" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A86" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B86" s="1">
+        <v>1</v>
+      </c>
+      <c r="C86" s="14"/>
+      <c r="D86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(E86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="E86" s="1"/>
+      <c r="G86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(H86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="H86" s="1"/>
+      <c r="J86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(K86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="K86" s="1"/>
+      <c r="M86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(N86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="N86" s="1"/>
+      <c r="P86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Q86" s="1"/>
+      <c r="S86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(T86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="T86" s="1"/>
+      <c r="V86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(W86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="W86" s="1"/>
+      <c r="Y86" s="3" t="str">
+        <f>IF(ISERROR(VLOOKUP(RANK(Z86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v/>
+      </c>
+      <c r="Z86" s="1"/>
+    </row>
+    <row r="87" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A87" s="5"/>
+      <c r="B87" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C73" s="8"/>
-      <c r="D73" s="1"/>
-      <c r="E73" s="7" t="s">
+      <c r="C87" s="8"/>
+      <c r="D87" s="1"/>
+      <c r="E87" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G73" s="1"/>
-      <c r="H73" s="7" t="s">
+      <c r="G87" s="1"/>
+      <c r="H87" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="J73" s="1"/>
-      <c r="K73" s="7" t="s">
+      <c r="J87" s="1"/>
+      <c r="K87" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="M73" s="1"/>
-      <c r="N73" s="7" t="s">
+      <c r="M87" s="1"/>
+      <c r="N87" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="P73" s="1"/>
-      <c r="Q73" s="7" t="s">
+      <c r="P87" s="1"/>
+      <c r="Q87" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="S73" s="1"/>
-      <c r="T73" s="7" t="s">
+      <c r="S87" s="1"/>
+      <c r="T87" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="V73" s="1"/>
-      <c r="W73" s="7" t="s">
+      <c r="V87" s="1"/>
+      <c r="W87" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="Y73" s="1"/>
-      <c r="Z73" s="7" t="s">
+      <c r="Y87" s="1"/>
+      <c r="Z87" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="D74" s="1"/>
-      <c r="E74" s="9" t="str">
+    <row r="88" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="D88" s="1"/>
+      <c r="E88" s="9" t="str">
         <f>D12</f>
         <v>Jaya</v>
       </c>
-      <c r="G74" s="1"/>
-      <c r="H74" s="9" t="str">
+      <c r="G88" s="1"/>
+      <c r="H88" s="9" t="str">
         <f>G12</f>
         <v>Justin</v>
       </c>
-      <c r="J74" s="1"/>
-      <c r="K74" s="9" t="str">
+      <c r="J88" s="1"/>
+      <c r="K88" s="9" t="str">
         <f>J12</f>
         <v>Ram</v>
       </c>
-      <c r="M74" s="1"/>
-      <c r="N74" s="9" t="str">
+      <c r="M88" s="1"/>
+      <c r="N88" s="9" t="str">
         <f>M12</f>
         <v>Sibi</v>
       </c>
-      <c r="P74" s="1"/>
-      <c r="Q74" s="9" t="str">
+      <c r="P88" s="1"/>
+      <c r="Q88" s="9" t="str">
         <f>P12</f>
         <v>Sundar</v>
       </c>
-      <c r="S74" s="1"/>
-      <c r="T74" s="9" t="str">
+      <c r="S88" s="1"/>
+      <c r="T88" s="9" t="str">
         <f>S12</f>
         <v>Sampath</v>
       </c>
-      <c r="V74" s="1"/>
-      <c r="W74" s="9" t="str">
+      <c r="V88" s="1"/>
+      <c r="W88" s="9" t="str">
         <f>V12</f>
         <v>Jayanth</v>
       </c>
-      <c r="Y74" s="1"/>
-      <c r="Z74" s="9" t="str">
+      <c r="Y88" s="1"/>
+      <c r="Z88" s="9" t="str">
         <f>Y12</f>
         <v>Vicky</v>
       </c>
     </row>
-    <row r="75" spans="1:27" ht="21" x14ac:dyDescent="0.25">
-      <c r="D75" s="6" t="s">
+    <row r="89" spans="1:27" ht="21" x14ac:dyDescent="0.25">
+      <c r="D89" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E75" s="10">
-        <f>SUM(D13:D72)</f>
-        <v>-167.5</v>
-      </c>
-      <c r="G75" s="6" t="s">
+      <c r="E89" s="10">
+        <f>SUM(D13:D86)</f>
+        <v>-117.5</v>
+      </c>
+      <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H75" s="10">
-        <f>SUM(G13:G72)</f>
-        <v>-55</v>
-      </c>
-      <c r="J75" s="6" t="s">
+      <c r="H89" s="10">
+        <f>SUM(G13:G86)</f>
+        <v>0</v>
+      </c>
+      <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="K75" s="10">
-        <f>SUM(J13:J72)</f>
-        <v>-12.5</v>
-      </c>
-      <c r="M75" s="6" t="s">
+      <c r="K89" s="10">
+        <f>SUM(J13:J86)</f>
+        <v>-22.5</v>
+      </c>
+      <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="N75" s="10">
-        <f>SUM(M13:M72)</f>
-        <v>275</v>
-      </c>
-      <c r="P75" s="6" t="s">
+      <c r="N89" s="10">
+        <f>SUM(M13:M86)</f>
+        <v>245</v>
+      </c>
+      <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="Q75" s="10">
-        <f>SUM(P13:P72)</f>
-        <v>10</v>
-      </c>
-      <c r="S75" s="6" t="s">
+      <c r="Q89" s="10">
+        <f>SUM(P13:P86)</f>
+        <v>0</v>
+      </c>
+      <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="T75" s="10">
-        <f>SUM(S13:S72)</f>
+      <c r="T89" s="10">
+        <f>SUM(S13:S86)</f>
         <v>-102.5</v>
       </c>
-      <c r="V75" s="6" t="s">
+      <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="W75" s="10">
-        <f>SUM(V13:V72)</f>
-        <v>130</v>
-      </c>
-      <c r="Y75" s="6" t="s">
+      <c r="W89" s="10">
+        <f>SUM(V13:V86)</f>
+        <v>80</v>
+      </c>
+      <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="Z75" s="10">
-        <f>SUM(Y13:Y72)</f>
-        <v>-77.5</v>
-      </c>
-      <c r="AA75" s="1">
-        <f>SUM(E75,H75,K75,N75,Q75,T75,W75,Z75)</f>
+      <c r="Z89" s="10">
+        <f>SUM(Y13:Y86)</f>
+        <v>-82.5</v>
+      </c>
+      <c r="AA89" s="1">
+        <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>
         <v>0</v>
       </c>
     </row>
@@ -4878,40 +5846,40 @@
     <mergeCell ref="J11:K11"/>
     <mergeCell ref="M11:N11"/>
   </mergeCells>
-  <conditionalFormatting sqref="E75">
-    <cfRule type="cellIs" dxfId="26" priority="141" operator="greaterThan">
+  <conditionalFormatting sqref="E89">
+    <cfRule type="cellIs" dxfId="26" priority="139" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="25" priority="140" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="139" operator="lessThan">
+    <cfRule type="cellIs" dxfId="24" priority="141" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H75">
-    <cfRule type="cellIs" dxfId="23" priority="36" operator="greaterThan">
+  <conditionalFormatting sqref="H89">
+    <cfRule type="cellIs" dxfId="23" priority="34" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="22" priority="35" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="34" operator="lessThan">
+    <cfRule type="cellIs" dxfId="21" priority="36" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K75">
-    <cfRule type="cellIs" dxfId="20" priority="33" operator="greaterThan">
+  <conditionalFormatting sqref="K89">
+    <cfRule type="cellIs" dxfId="20" priority="31" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="19" priority="32" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="31" operator="lessThan">
+    <cfRule type="cellIs" dxfId="18" priority="33" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N75">
+  <conditionalFormatting sqref="N89">
     <cfRule type="cellIs" dxfId="17" priority="28" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -4922,47 +5890,47 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q75">
-    <cfRule type="cellIs" dxfId="14" priority="26" operator="equal">
+  <conditionalFormatting sqref="Q89">
+    <cfRule type="cellIs" dxfId="14" priority="25" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="27" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="26" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="25" operator="lessThan">
+    <cfRule type="cellIs" dxfId="12" priority="27" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T75">
-    <cfRule type="cellIs" dxfId="11" priority="24" operator="greaterThan">
+  <conditionalFormatting sqref="T89">
+    <cfRule type="cellIs" dxfId="11" priority="22" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="10" priority="23" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W75">
-    <cfRule type="cellIs" dxfId="8" priority="21" operator="greaterThan">
+  <conditionalFormatting sqref="W89">
+    <cfRule type="cellIs" dxfId="8" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="7" priority="20" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="19" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="21" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z75">
-    <cfRule type="cellIs" dxfId="5" priority="18" operator="greaterThan">
+  <conditionalFormatting sqref="Z89">
+    <cfRule type="cellIs" dxfId="5" priority="16" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="4" priority="17" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="16" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Contest 30 RCB vs SRH
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABBB209E-1AC5-0A40-A060-B8724B7B1438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{563CB9AA-B552-714E-9207-BC85CB8EA361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="27820" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="28300" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3413,46 +3413,62 @@
       <c r="C42" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="D42" s="3" t="str">
+      <c r="D42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E42" s="1"/>
-      <c r="G42" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E42" s="1">
+        <v>70</v>
+      </c>
+      <c r="G42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H42" s="1"/>
-      <c r="J42" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="H42" s="1">
+        <v>20</v>
+      </c>
+      <c r="J42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K42" s="1"/>
-      <c r="M42" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="K42" s="1">
+        <v>40</v>
+      </c>
+      <c r="M42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N42" s="1"/>
-      <c r="P42" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N42" s="1">
+        <v>0</v>
+      </c>
+      <c r="P42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q42" s="1"/>
-      <c r="S42" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q42" s="1">
+        <v>30</v>
+      </c>
+      <c r="S42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T42" s="1"/>
-      <c r="V42" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="T42" s="1">
+        <v>100</v>
+      </c>
+      <c r="V42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W42" s="1"/>
-      <c r="Y42" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="W42" s="1">
+        <v>60</v>
+      </c>
+      <c r="Y42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z42" s="1"/>
+        <v>-5</v>
+      </c>
+      <c r="Z42" s="1">
+        <v>50</v>
+      </c>
     </row>
     <row r="43" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
@@ -5777,56 +5793,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-117.5</v>
+        <v>-97.5</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>0</v>
+        <v>-20</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-22.5</v>
+        <v>-32.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>245</v>
+        <v>220</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>0</v>
+        <v>-15</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-102.5</v>
+        <v>-52.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-82.5</v>
+        <v>-87.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 31 KKR vs RR
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{563CB9AA-B552-714E-9207-BC85CB8EA361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0784B34-9D91-9441-988A-E46A64C6D0FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="28300" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -3480,46 +3480,60 @@
       <c r="C43" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="D43" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E43" s="1"/>
-      <c r="G43" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H43" s="1"/>
-      <c r="J43" s="3" t="str">
+      <c r="D43" s="3">
+        <v>-7.5</v>
+      </c>
+      <c r="E43" s="1">
+        <v>50</v>
+      </c>
+      <c r="G43" s="3">
+        <v>-7.5</v>
+      </c>
+      <c r="H43" s="1">
+        <v>50</v>
+      </c>
+      <c r="J43" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K43" s="1"/>
-      <c r="M43" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K43" s="1">
+        <v>20</v>
+      </c>
+      <c r="M43" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N43" s="1"/>
-      <c r="P43" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N43" s="1">
+        <v>100</v>
+      </c>
+      <c r="P43" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q43" s="1"/>
-      <c r="S43" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q43" s="1">
+        <v>30</v>
+      </c>
+      <c r="S43" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T43" s="1"/>
-      <c r="V43" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T43" s="1">
+        <v>70</v>
+      </c>
+      <c r="V43" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W43" s="1"/>
-      <c r="Y43" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="W43" s="1">
+        <v>60</v>
+      </c>
+      <c r="Y43" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z43, ($Z43,$W43,$T43,$Q43,$N43,$K43,$H43,$E43), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z43" s="1"/>
+        <v>-25</v>
+      </c>
+      <c r="Z43" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="44" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
@@ -5793,56 +5807,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-97.5</v>
+        <v>-105</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>-20</v>
+        <v>-27.5</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-32.5</v>
+        <v>-52.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>220</v>
+        <v>270</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-15</v>
+        <v>-30</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-52.5</v>
+        <v>-32.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-87.5</v>
+        <v>-112.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 33 PBKS vs MI
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0784B34-9D91-9441-988A-E46A64C6D0FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C8329FC-B732-6A49-A799-DDE002C10DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="28300" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -578,6 +578,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -586,9 +589,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -613,6 +613,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -738,11 +748,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -758,11 +768,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -853,16 +863,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1212,24 +1212,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
-      <c r="S2" s="21"/>
-      <c r="T2" s="21"/>
-      <c r="U2" s="21"/>
-      <c r="V2" s="21"/>
-      <c r="W2" s="21"/>
-      <c r="X2" s="21"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
+      <c r="S2" s="18"/>
+      <c r="T2" s="18"/>
+      <c r="U2" s="18"/>
+      <c r="V2" s="18"/>
+      <c r="W2" s="18"/>
+      <c r="X2" s="18"/>
     </row>
     <row r="3" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1238,22 +1238,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="21"/>
-      <c r="P3" s="21"/>
-      <c r="Q3" s="21"/>
-      <c r="R3" s="21"/>
-      <c r="S3" s="21"/>
-      <c r="T3" s="21"/>
-      <c r="U3" s="21"/>
-      <c r="V3" s="21"/>
-      <c r="W3" s="21"/>
-      <c r="X3" s="21"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="18"/>
+      <c r="S3" s="18"/>
+      <c r="T3" s="18"/>
+      <c r="U3" s="18"/>
+      <c r="V3" s="18"/>
+      <c r="W3" s="18"/>
+      <c r="X3" s="18"/>
     </row>
     <row r="4" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1262,22 +1262,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="21"/>
-      <c r="O4" s="21"/>
-      <c r="P4" s="21"/>
-      <c r="Q4" s="21"/>
-      <c r="R4" s="21"/>
-      <c r="S4" s="21"/>
-      <c r="T4" s="21"/>
-      <c r="U4" s="21"/>
-      <c r="V4" s="21"/>
-      <c r="W4" s="21"/>
-      <c r="X4" s="21"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="Q4" s="18"/>
+      <c r="R4" s="18"/>
+      <c r="S4" s="18"/>
+      <c r="T4" s="18"/>
+      <c r="U4" s="18"/>
+      <c r="V4" s="18"/>
+      <c r="W4" s="18"/>
+      <c r="X4" s="18"/>
     </row>
     <row r="5" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1286,22 +1286,22 @@
       <c r="B5" s="1">
         <v>-5</v>
       </c>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="21"/>
-      <c r="N5" s="21"/>
-      <c r="O5" s="21"/>
-      <c r="P5" s="21"/>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="21"/>
-      <c r="S5" s="21"/>
-      <c r="T5" s="21"/>
-      <c r="U5" s="21"/>
-      <c r="V5" s="21"/>
-      <c r="W5" s="21"/>
-      <c r="X5" s="21"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="18"/>
+      <c r="W5" s="18"/>
+      <c r="X5" s="18"/>
     </row>
     <row r="6" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1310,22 +1310,22 @@
       <c r="B6" s="1">
         <v>-10</v>
       </c>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="21"/>
-      <c r="O6" s="21"/>
-      <c r="P6" s="21"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="21"/>
-      <c r="S6" s="21"/>
-      <c r="T6" s="21"/>
-      <c r="U6" s="21"/>
-      <c r="V6" s="21"/>
-      <c r="W6" s="21"/>
-      <c r="X6" s="21"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
+      <c r="P6" s="18"/>
+      <c r="Q6" s="18"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="18"/>
+      <c r="T6" s="18"/>
+      <c r="U6" s="18"/>
+      <c r="V6" s="18"/>
+      <c r="W6" s="18"/>
+      <c r="X6" s="18"/>
     </row>
     <row r="7" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1334,22 +1334,22 @@
       <c r="B7" s="1">
         <v>-15</v>
       </c>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21"/>
-      <c r="T7" s="21"/>
-      <c r="U7" s="21"/>
-      <c r="V7" s="21"/>
-      <c r="W7" s="21"/>
-      <c r="X7" s="21"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="18"/>
+      <c r="Q7" s="18"/>
+      <c r="R7" s="18"/>
+      <c r="S7" s="18"/>
+      <c r="T7" s="18"/>
+      <c r="U7" s="18"/>
+      <c r="V7" s="18"/>
+      <c r="W7" s="18"/>
+      <c r="X7" s="18"/>
     </row>
     <row r="8" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1358,22 +1358,22 @@
       <c r="B8" s="1">
         <v>-20</v>
       </c>
-      <c r="I8" s="21"/>
-      <c r="J8" s="21"/>
-      <c r="K8" s="21"/>
-      <c r="L8" s="21"/>
-      <c r="M8" s="21"/>
-      <c r="N8" s="21"/>
-      <c r="O8" s="21"/>
-      <c r="P8" s="21"/>
-      <c r="Q8" s="21"/>
-      <c r="R8" s="21"/>
-      <c r="S8" s="21"/>
-      <c r="T8" s="21"/>
-      <c r="U8" s="21"/>
-      <c r="V8" s="21"/>
-      <c r="W8" s="21"/>
-      <c r="X8" s="21"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
+      <c r="M8" s="18"/>
+      <c r="N8" s="18"/>
+      <c r="O8" s="18"/>
+      <c r="P8" s="18"/>
+      <c r="Q8" s="18"/>
+      <c r="R8" s="18"/>
+      <c r="S8" s="18"/>
+      <c r="T8" s="18"/>
+      <c r="U8" s="18"/>
+      <c r="V8" s="18"/>
+      <c r="W8" s="18"/>
+      <c r="X8" s="18"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1388,38 +1388,38 @@
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="20"/>
-      <c r="G11" s="18" t="s">
+      <c r="E11" s="21"/>
+      <c r="G11" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="19"/>
-      <c r="J11" s="18" t="s">
+      <c r="H11" s="20"/>
+      <c r="J11" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="K11" s="19"/>
-      <c r="M11" s="18" t="s">
+      <c r="K11" s="20"/>
+      <c r="M11" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="N11" s="19"/>
-      <c r="P11" s="18" t="s">
+      <c r="N11" s="20"/>
+      <c r="P11" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="Q11" s="19"/>
-      <c r="S11" s="18" t="s">
+      <c r="Q11" s="20"/>
+      <c r="S11" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T11" s="19"/>
-      <c r="V11" s="18" t="s">
+      <c r="T11" s="20"/>
+      <c r="V11" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="W11" s="19"/>
-      <c r="Y11" s="18" t="s">
+      <c r="W11" s="20"/>
+      <c r="Y11" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="Z11" s="19"/>
+      <c r="Z11" s="20"/>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
@@ -3545,46 +3545,62 @@
       <c r="C44" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="D44" s="3" t="str">
+      <c r="D44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E44" s="1"/>
-      <c r="G44" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="E44" s="1">
+        <v>0</v>
+      </c>
+      <c r="G44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H44" s="1"/>
-      <c r="J44" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="H44" s="1">
+        <v>100</v>
+      </c>
+      <c r="J44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K44" s="1"/>
-      <c r="M44" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="K44" s="1">
+        <v>50</v>
+      </c>
+      <c r="M44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N44" s="1"/>
-      <c r="P44" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="N44" s="1">
+        <v>20</v>
+      </c>
+      <c r="P44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q44" s="1"/>
-      <c r="S44" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q44" s="1">
+        <v>60</v>
+      </c>
+      <c r="S44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T44" s="1"/>
-      <c r="V44" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T44" s="1">
+        <v>70</v>
+      </c>
+      <c r="V44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W44" s="1"/>
-      <c r="Y44" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W44" s="1">
+        <v>30</v>
+      </c>
+      <c r="Y44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z44" s="1"/>
+        <v>-10</v>
+      </c>
+      <c r="Z44" s="1">
+        <v>40</v>
+      </c>
     </row>
     <row r="45" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
@@ -3596,48 +3612,64 @@
       <c r="C45" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="D45" s="3" t="str">
+      <c r="D45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E45" s="1"/>
-      <c r="G45" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="E45" s="1">
+        <v>60</v>
+      </c>
+      <c r="G45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H45" s="1"/>
-      <c r="J45" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="H45" s="1">
+        <v>40</v>
+      </c>
+      <c r="J45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K45" s="1"/>
-      <c r="M45" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="K45" s="1">
+        <v>70</v>
+      </c>
+      <c r="M45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N45" s="1"/>
-      <c r="P45" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="N45" s="1">
+        <v>30</v>
+      </c>
+      <c r="P45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q45" s="1"/>
-      <c r="S45" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Q45" s="1">
+        <v>0</v>
+      </c>
+      <c r="S45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T45" s="1"/>
-      <c r="V45" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="T45" s="1">
+        <v>50</v>
+      </c>
+      <c r="V45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W45" s="1"/>
-      <c r="Y45" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="W45" s="1">
+        <v>100</v>
+      </c>
+      <c r="Y45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z45" s="1"/>
-    </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.2">
+        <v>-20</v>
+      </c>
+      <c r="Z45" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="46" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>34</v>
       </c>
@@ -3688,7 +3720,7 @@
       </c>
       <c r="Z46" s="1"/>
     </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>35</v>
       </c>
@@ -3739,7 +3771,7 @@
       </c>
       <c r="Z47" s="1"/>
     </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>36</v>
       </c>
@@ -3790,7 +3822,7 @@
       </c>
       <c r="Z48" s="1"/>
     </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>37</v>
       </c>
@@ -3841,7 +3873,7 @@
       </c>
       <c r="Z49" s="1"/>
     </row>
-    <row r="50" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>38</v>
       </c>
@@ -3892,7 +3924,7 @@
       </c>
       <c r="Z50" s="1"/>
     </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>39</v>
       </c>
@@ -3943,7 +3975,7 @@
       </c>
       <c r="Z51" s="1"/>
     </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>40</v>
       </c>
@@ -3994,7 +4026,7 @@
       </c>
       <c r="Z52" s="1"/>
     </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>41</v>
       </c>
@@ -4045,7 +4077,7 @@
       </c>
       <c r="Z53" s="1"/>
     </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>42</v>
       </c>
@@ -4096,7 +4128,7 @@
       </c>
       <c r="Z54" s="1"/>
     </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>43</v>
       </c>
@@ -4147,7 +4179,7 @@
       </c>
       <c r="Z55" s="1"/>
     </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
         <v>44</v>
       </c>
@@ -4198,7 +4230,7 @@
       </c>
       <c r="Z56" s="1"/>
     </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>45</v>
       </c>
@@ -4249,7 +4281,7 @@
       </c>
       <c r="Z57" s="1"/>
     </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>46</v>
       </c>
@@ -4300,7 +4332,7 @@
       </c>
       <c r="Z58" s="1"/>
     </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>47</v>
       </c>
@@ -4351,7 +4383,7 @@
       </c>
       <c r="Z59" s="1"/>
     </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>48</v>
       </c>
@@ -4402,7 +4434,7 @@
       </c>
       <c r="Z60" s="1"/>
     </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>49</v>
       </c>
@@ -4453,7 +4485,7 @@
       </c>
       <c r="Z61" s="1"/>
     </row>
-    <row r="62" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
         <v>50</v>
       </c>
@@ -4504,7 +4536,7 @@
       </c>
       <c r="Z62" s="1"/>
     </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
         <v>51</v>
       </c>
@@ -4555,7 +4587,7 @@
       </c>
       <c r="Z63" s="1"/>
     </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
         <v>52</v>
       </c>
@@ -4606,7 +4638,7 @@
       </c>
       <c r="Z64" s="1"/>
     </row>
-    <row r="65" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>53</v>
       </c>
@@ -4657,7 +4689,7 @@
       </c>
       <c r="Z65" s="1"/>
     </row>
-    <row r="66" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>54</v>
       </c>
@@ -4708,7 +4740,7 @@
       </c>
       <c r="Z66" s="1"/>
     </row>
-    <row r="67" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>55</v>
       </c>
@@ -4759,7 +4791,7 @@
       </c>
       <c r="Z67" s="1"/>
     </row>
-    <row r="68" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>56</v>
       </c>
@@ -4810,7 +4842,7 @@
       </c>
       <c r="Z68" s="1"/>
     </row>
-    <row r="69" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>57</v>
       </c>
@@ -4861,7 +4893,7 @@
       </c>
       <c r="Z69" s="1"/>
     </row>
-    <row r="70" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>58</v>
       </c>
@@ -4912,7 +4944,7 @@
       </c>
       <c r="Z70" s="1"/>
     </row>
-    <row r="71" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>59</v>
       </c>
@@ -4963,7 +4995,7 @@
       </c>
       <c r="Z71" s="1"/>
     </row>
-    <row r="72" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>60</v>
       </c>
@@ -5014,7 +5046,7 @@
       </c>
       <c r="Z72" s="1"/>
     </row>
-    <row r="73" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>61</v>
       </c>
@@ -5065,7 +5097,7 @@
       </c>
       <c r="Z73" s="1"/>
     </row>
-    <row r="74" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>62</v>
       </c>
@@ -5116,7 +5148,7 @@
       </c>
       <c r="Z74" s="1"/>
     </row>
-    <row r="75" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>63</v>
       </c>
@@ -5167,7 +5199,7 @@
       </c>
       <c r="Z75" s="1"/>
     </row>
-    <row r="76" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>64</v>
       </c>
@@ -5218,7 +5250,7 @@
       </c>
       <c r="Z76" s="1"/>
     </row>
-    <row r="77" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
         <v>65</v>
       </c>
@@ -5269,7 +5301,7 @@
       </c>
       <c r="Z77" s="1"/>
     </row>
-    <row r="78" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
         <v>66</v>
       </c>
@@ -5320,7 +5352,7 @@
       </c>
       <c r="Z78" s="1"/>
     </row>
-    <row r="79" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" s="1">
         <v>67</v>
       </c>
@@ -5371,7 +5403,7 @@
       </c>
       <c r="Z79" s="1"/>
     </row>
-    <row r="80" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" s="1">
         <v>68</v>
       </c>
@@ -5422,7 +5454,7 @@
       </c>
       <c r="Z80" s="1"/>
     </row>
-    <row r="81" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
         <v>69</v>
       </c>
@@ -5473,7 +5505,7 @@
       </c>
       <c r="Z81" s="1"/>
     </row>
-    <row r="82" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" s="1">
         <v>70</v>
       </c>
@@ -5807,56 +5839,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-105</v>
+        <v>-125</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>-27.5</v>
+        <v>12.5</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-52.5</v>
+        <v>-37.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>270</v>
+        <v>235</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-30</v>
+        <v>-50</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-32.5</v>
+        <v>-17.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>90</v>
+        <v>125</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-112.5</v>
+        <v>-142.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>
@@ -5866,46 +5898,46 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="9">
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="M11:N11"/>
     <mergeCell ref="I2:X8"/>
     <mergeCell ref="S11:T11"/>
     <mergeCell ref="P11:Q11"/>
     <mergeCell ref="V11:W11"/>
     <mergeCell ref="Y11:Z11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="M11:N11"/>
   </mergeCells>
   <conditionalFormatting sqref="E89">
-    <cfRule type="cellIs" dxfId="26" priority="139" operator="lessThan">
+    <cfRule type="cellIs" dxfId="26" priority="141" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="25" priority="140" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="141" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="139" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H89">
-    <cfRule type="cellIs" dxfId="23" priority="34" operator="lessThan">
+    <cfRule type="cellIs" dxfId="23" priority="36" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="22" priority="35" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="36" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="34" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K89">
-    <cfRule type="cellIs" dxfId="20" priority="31" operator="lessThan">
+    <cfRule type="cellIs" dxfId="20" priority="33" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="19" priority="32" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="33" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="31" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5921,46 +5953,46 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q89">
-    <cfRule type="cellIs" dxfId="14" priority="25" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="26" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="27" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="27" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="25" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T89">
-    <cfRule type="cellIs" dxfId="11" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="10" priority="23" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="24" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="22" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W89">
-    <cfRule type="cellIs" dxfId="8" priority="19" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="21" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="7" priority="20" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="19" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z89">
-    <cfRule type="cellIs" dxfId="5" priority="16" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="4" priority="17" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="18" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="16" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Contest 34 through 37
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C8329FC-B732-6A49-A799-DDE002C10DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C03825-D269-B14D-8AEA-0C0BFCD5EA0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="28300" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3669,7 +3669,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>34</v>
       </c>
@@ -3679,48 +3679,64 @@
       <c r="C46" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="D46" s="3" t="str">
+      <c r="D46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E46" s="1"/>
-      <c r="G46" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E46" s="1">
+        <v>40</v>
+      </c>
+      <c r="G46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H46" s="1"/>
-      <c r="J46" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="H46" s="1">
+        <v>20</v>
+      </c>
+      <c r="J46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K46" s="1"/>
-      <c r="M46" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="K46" s="1">
+        <v>70</v>
+      </c>
+      <c r="M46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N46" s="1"/>
-      <c r="P46" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N46" s="1">
+        <v>0</v>
+      </c>
+      <c r="P46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q46" s="1"/>
-      <c r="S46" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q46" s="1">
+        <v>30</v>
+      </c>
+      <c r="S46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T46" s="1"/>
-      <c r="V46" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T46" s="1">
+        <v>60</v>
+      </c>
+      <c r="V46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W46" s="1"/>
-      <c r="Y46" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="W46" s="1">
+        <v>100</v>
+      </c>
+      <c r="Y46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z46" s="1"/>
-    </row>
-    <row r="47" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-5</v>
+      </c>
+      <c r="Z46" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>35</v>
       </c>
@@ -3730,48 +3746,64 @@
       <c r="C47" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="D47" s="3" t="str">
+      <c r="D47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E47" s="1"/>
-      <c r="G47" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="E47" s="1">
+        <v>50</v>
+      </c>
+      <c r="G47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H47" s="1"/>
-      <c r="J47" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="H47" s="1">
+        <v>20</v>
+      </c>
+      <c r="J47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K47" s="1"/>
-      <c r="M47" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="K47" s="1">
+        <v>0</v>
+      </c>
+      <c r="M47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N47" s="1"/>
-      <c r="P47" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N47" s="1">
+        <v>100</v>
+      </c>
+      <c r="P47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q47" s="1"/>
-      <c r="S47" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q47" s="1">
+        <v>70</v>
+      </c>
+      <c r="S47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T47" s="1"/>
-      <c r="V47" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="T47" s="1">
+        <v>30</v>
+      </c>
+      <c r="V47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W47" s="1"/>
-      <c r="Y47" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="W47" s="1">
+        <v>60</v>
+      </c>
+      <c r="Y47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z47" s="1"/>
-    </row>
-    <row r="48" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-10</v>
+      </c>
+      <c r="Z47" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="48" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>36</v>
       </c>
@@ -3781,48 +3813,64 @@
       <c r="C48" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="D48" s="3" t="str">
+      <c r="D48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E48" s="1"/>
-      <c r="G48" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E48" s="1">
+        <v>40</v>
+      </c>
+      <c r="G48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H48" s="1"/>
-      <c r="J48" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H48" s="1">
+        <v>60</v>
+      </c>
+      <c r="J48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K48" s="1"/>
-      <c r="M48" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="K48" s="1">
+        <v>100</v>
+      </c>
+      <c r="M48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N48" s="1"/>
-      <c r="P48" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N48" s="1">
+        <v>70</v>
+      </c>
+      <c r="P48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q48" s="1"/>
-      <c r="S48" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q48" s="1">
+        <v>30</v>
+      </c>
+      <c r="S48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T48" s="1"/>
-      <c r="V48" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="T48" s="1">
+        <v>20</v>
+      </c>
+      <c r="V48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W48" s="1"/>
-      <c r="Y48" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="W48" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z48" s="1"/>
-    </row>
-    <row r="49" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-5</v>
+      </c>
+      <c r="Z48" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="49" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>37</v>
       </c>
@@ -3832,46 +3880,62 @@
       <c r="C49" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="D49" s="3" t="str">
+      <c r="D49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E49" s="1"/>
-      <c r="G49" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="E49" s="1">
+        <v>100</v>
+      </c>
+      <c r="G49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H49" s="1"/>
-      <c r="J49" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H49" s="1">
+        <v>60</v>
+      </c>
+      <c r="J49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K49" s="1"/>
-      <c r="M49" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K49" s="1">
+        <v>30</v>
+      </c>
+      <c r="M49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N49" s="1"/>
-      <c r="P49" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N49" s="1">
+        <v>70</v>
+      </c>
+      <c r="P49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q49" s="1"/>
-      <c r="S49" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q49" s="1">
+        <v>20</v>
+      </c>
+      <c r="S49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T49" s="1"/>
-      <c r="V49" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="T49" s="1">
+        <v>0</v>
+      </c>
+      <c r="V49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W49" s="1"/>
-      <c r="Y49" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="W49" s="1">
+        <v>50</v>
+      </c>
+      <c r="Y49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z49" s="1"/>
+        <v>-10</v>
+      </c>
+      <c r="Z49" s="1">
+        <v>40</v>
+      </c>
     </row>
     <row r="50" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
@@ -5839,56 +5903,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-125</v>
+        <v>-100</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>12.5</v>
+        <v>-17.5</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-37.5</v>
+        <v>-7.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>235</v>
+        <v>300</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-50</v>
+        <v>-80</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-17.5</v>
+        <v>-72.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-142.5</v>
+        <v>-172.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 38 RR vs MI
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C03825-D269-B14D-8AEA-0C0BFCD5EA0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C47FC323-9DA6-FF4F-B667-3FAD17700CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="28300" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -3937,7 +3937,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="50" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>38</v>
       </c>
@@ -3947,46 +3947,62 @@
       <c r="C50" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="D50" s="3" t="str">
+      <c r="D50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E50" s="1"/>
-      <c r="G50" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="E50" s="1">
+        <v>60</v>
+      </c>
+      <c r="G50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H50" s="1"/>
-      <c r="J50" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="H50" s="1">
+        <v>70</v>
+      </c>
+      <c r="J50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K50" s="1"/>
-      <c r="M50" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K50" s="1">
+        <v>20</v>
+      </c>
+      <c r="M50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N50" s="1"/>
-      <c r="P50" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N50" s="1">
+        <v>100</v>
+      </c>
+      <c r="P50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q50" s="1"/>
-      <c r="S50" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q50" s="1">
+        <v>30</v>
+      </c>
+      <c r="S50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T50" s="1"/>
-      <c r="V50" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="T50" s="1">
+        <v>50</v>
+      </c>
+      <c r="V50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W50" s="1"/>
-      <c r="Y50" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="W50" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z50" s="1"/>
+        <v>-10</v>
+      </c>
+      <c r="Z50" s="1">
+        <v>40</v>
+      </c>
     </row>
     <row r="51" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
@@ -5903,56 +5919,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-100</v>
+        <v>-95</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>-17.5</v>
+        <v>2.5</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-7.5</v>
+        <v>-27.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-80</v>
+        <v>-95</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-72.5</v>
+        <v>-77.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-172.5</v>
+        <v>-182.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 39 CSK vs LSG
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C47FC323-9DA6-FF4F-B667-3FAD17700CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA88FCD-F40E-7D4B-842E-119D567E6E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="28300" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -4004,7 +4004,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="51" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>39</v>
       </c>
@@ -4014,46 +4014,62 @@
       <c r="C51" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="D51" s="3" t="str">
+      <c r="D51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E51" s="1"/>
-      <c r="G51" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E51" s="1">
+        <v>40</v>
+      </c>
+      <c r="G51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H51" s="1"/>
-      <c r="J51" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="H51" s="1">
+        <v>30</v>
+      </c>
+      <c r="J51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K51" s="1"/>
-      <c r="M51" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K51" s="1">
+        <v>20</v>
+      </c>
+      <c r="M51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N51" s="1"/>
-      <c r="P51" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="N51" s="1">
+        <v>50</v>
+      </c>
+      <c r="P51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q51" s="1"/>
-      <c r="S51" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q51" s="1">
+        <v>100</v>
+      </c>
+      <c r="S51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T51" s="1"/>
-      <c r="V51" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T51" s="1">
+        <v>70</v>
+      </c>
+      <c r="V51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W51" s="1"/>
-      <c r="Y51" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="W51" s="1">
+        <v>60</v>
+      </c>
+      <c r="Y51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z51" s="1"/>
+        <v>-25</v>
+      </c>
+      <c r="Z51" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="52" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
@@ -5919,56 +5935,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-95</v>
+        <v>-105</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>2.5</v>
+        <v>-12.5</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-27.5</v>
+        <v>-47.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-95</v>
+        <v>-45</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-77.5</v>
+        <v>-57.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-182.5</v>
+        <v>-207.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 40 DC vs GT
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA88FCD-F40E-7D4B-842E-119D567E6E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AE8BB5-20C7-9740-A225-56750A06F90B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-3180" windowWidth="51200" windowHeight="28300" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -578,8 +578,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -587,8 +587,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1212,24 +1212,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
-      <c r="N2" s="18"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="18"/>
-      <c r="Q2" s="18"/>
-      <c r="R2" s="18"/>
-      <c r="S2" s="18"/>
-      <c r="T2" s="18"/>
-      <c r="U2" s="18"/>
-      <c r="V2" s="18"/>
-      <c r="W2" s="18"/>
-      <c r="X2" s="18"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="21"/>
+      <c r="T2" s="21"/>
+      <c r="U2" s="21"/>
+      <c r="V2" s="21"/>
+      <c r="W2" s="21"/>
+      <c r="X2" s="21"/>
     </row>
     <row r="3" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1238,22 +1238,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
-      <c r="Q3" s="18"/>
-      <c r="R3" s="18"/>
-      <c r="S3" s="18"/>
-      <c r="T3" s="18"/>
-      <c r="U3" s="18"/>
-      <c r="V3" s="18"/>
-      <c r="W3" s="18"/>
-      <c r="X3" s="18"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="21"/>
+      <c r="P3" s="21"/>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="21"/>
+      <c r="T3" s="21"/>
+      <c r="U3" s="21"/>
+      <c r="V3" s="21"/>
+      <c r="W3" s="21"/>
+      <c r="X3" s="21"/>
     </row>
     <row r="4" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1262,22 +1262,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
-      <c r="O4" s="18"/>
-      <c r="P4" s="18"/>
-      <c r="Q4" s="18"/>
-      <c r="R4" s="18"/>
-      <c r="S4" s="18"/>
-      <c r="T4" s="18"/>
-      <c r="U4" s="18"/>
-      <c r="V4" s="18"/>
-      <c r="W4" s="18"/>
-      <c r="X4" s="18"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21"/>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="21"/>
+      <c r="S4" s="21"/>
+      <c r="T4" s="21"/>
+      <c r="U4" s="21"/>
+      <c r="V4" s="21"/>
+      <c r="W4" s="21"/>
+      <c r="X4" s="21"/>
     </row>
     <row r="5" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1286,22 +1286,22 @@
       <c r="B5" s="1">
         <v>-5</v>
       </c>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
-      <c r="O5" s="18"/>
-      <c r="P5" s="18"/>
-      <c r="Q5" s="18"/>
-      <c r="R5" s="18"/>
-      <c r="S5" s="18"/>
-      <c r="T5" s="18"/>
-      <c r="U5" s="18"/>
-      <c r="V5" s="18"/>
-      <c r="W5" s="18"/>
-      <c r="X5" s="18"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
+      <c r="N5" s="21"/>
+      <c r="O5" s="21"/>
+      <c r="P5" s="21"/>
+      <c r="Q5" s="21"/>
+      <c r="R5" s="21"/>
+      <c r="S5" s="21"/>
+      <c r="T5" s="21"/>
+      <c r="U5" s="21"/>
+      <c r="V5" s="21"/>
+      <c r="W5" s="21"/>
+      <c r="X5" s="21"/>
     </row>
     <row r="6" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1310,22 +1310,22 @@
       <c r="B6" s="1">
         <v>-10</v>
       </c>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="18"/>
-      <c r="P6" s="18"/>
-      <c r="Q6" s="18"/>
-      <c r="R6" s="18"/>
-      <c r="S6" s="18"/>
-      <c r="T6" s="18"/>
-      <c r="U6" s="18"/>
-      <c r="V6" s="18"/>
-      <c r="W6" s="18"/>
-      <c r="X6" s="18"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21"/>
+      <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
+      <c r="V6" s="21"/>
+      <c r="W6" s="21"/>
+      <c r="X6" s="21"/>
     </row>
     <row r="7" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1334,22 +1334,22 @@
       <c r="B7" s="1">
         <v>-15</v>
       </c>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="18"/>
-      <c r="N7" s="18"/>
-      <c r="O7" s="18"/>
-      <c r="P7" s="18"/>
-      <c r="Q7" s="18"/>
-      <c r="R7" s="18"/>
-      <c r="S7" s="18"/>
-      <c r="T7" s="18"/>
-      <c r="U7" s="18"/>
-      <c r="V7" s="18"/>
-      <c r="W7" s="18"/>
-      <c r="X7" s="18"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="21"/>
+      <c r="L7" s="21"/>
+      <c r="M7" s="21"/>
+      <c r="N7" s="21"/>
+      <c r="O7" s="21"/>
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="21"/>
+      <c r="S7" s="21"/>
+      <c r="T7" s="21"/>
+      <c r="U7" s="21"/>
+      <c r="V7" s="21"/>
+      <c r="W7" s="21"/>
+      <c r="X7" s="21"/>
     </row>
     <row r="8" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1358,22 +1358,22 @@
       <c r="B8" s="1">
         <v>-20</v>
       </c>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18"/>
-      <c r="N8" s="18"/>
-      <c r="O8" s="18"/>
-      <c r="P8" s="18"/>
-      <c r="Q8" s="18"/>
-      <c r="R8" s="18"/>
-      <c r="S8" s="18"/>
-      <c r="T8" s="18"/>
-      <c r="U8" s="18"/>
-      <c r="V8" s="18"/>
-      <c r="W8" s="18"/>
-      <c r="X8" s="18"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="21"/>
+      <c r="K8" s="21"/>
+      <c r="L8" s="21"/>
+      <c r="M8" s="21"/>
+      <c r="N8" s="21"/>
+      <c r="O8" s="21"/>
+      <c r="P8" s="21"/>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="21"/>
+      <c r="S8" s="21"/>
+      <c r="T8" s="21"/>
+      <c r="U8" s="21"/>
+      <c r="V8" s="21"/>
+      <c r="W8" s="21"/>
+      <c r="X8" s="21"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1388,10 +1388,10 @@
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="D11" s="21" t="s">
+      <c r="D11" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="21"/>
+      <c r="E11" s="18"/>
       <c r="G11" s="19" t="s">
         <v>14</v>
       </c>
@@ -4071,7 +4071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>40</v>
       </c>
@@ -4081,46 +4081,60 @@
       <c r="C52" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="D52" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E52" s="1"/>
-      <c r="G52" s="3" t="str">
+      <c r="D52" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="E52" s="1">
+        <v>20</v>
+      </c>
+      <c r="G52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H52" s="1"/>
-      <c r="J52" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="H52" s="1">
+        <v>30</v>
+      </c>
+      <c r="J52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K52" s="1"/>
-      <c r="M52" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="K52" s="1">
+        <v>60</v>
+      </c>
+      <c r="M52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N52" s="1"/>
-      <c r="P52" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N52" s="1">
+        <v>70</v>
+      </c>
+      <c r="P52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q52" s="1"/>
-      <c r="S52" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(T52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T52" s="1"/>
-      <c r="V52" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Q52" s="1">
+        <v>40</v>
+      </c>
+      <c r="S52" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="T52" s="1">
+        <v>20</v>
+      </c>
+      <c r="V52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W52" s="1"/>
-      <c r="Y52" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="W52" s="1">
+        <v>100</v>
+      </c>
+      <c r="Y52" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z52, ($Z52,$W52,$T52,$Q52,$N52,$K52,$H52,$E52), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z52" s="1"/>
+        <v>-5</v>
+      </c>
+      <c r="Z52" s="1">
+        <v>50</v>
+      </c>
     </row>
     <row r="53" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
@@ -5935,56 +5949,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-105</v>
+        <v>-127.5</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>-12.5</v>
+        <v>-27.5</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-47.5</v>
+        <v>-42.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>345</v>
+        <v>365</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-45</v>
+        <v>-55</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-57.5</v>
+        <v>-80</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-207.5</v>
+        <v>-212.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>
@@ -5994,6 +6008,7 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="9">
+    <mergeCell ref="Y11:Z11"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="J11:K11"/>
@@ -6002,7 +6017,6 @@
     <mergeCell ref="S11:T11"/>
     <mergeCell ref="P11:Q11"/>
     <mergeCell ref="V11:W11"/>
-    <mergeCell ref="Y11:Z11"/>
   </mergeCells>
   <conditionalFormatting sqref="E89">
     <cfRule type="cellIs" dxfId="26" priority="141" operator="greaterThan">

</xml_diff>

<commit_message>
Contest 41 SRH vs RCB
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AE8BB5-20C7-9740-A225-56750A06F90B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04CBABC-E3C8-BC4F-B819-979F878E0D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -4136,7 +4136,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="53" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>41</v>
       </c>
@@ -4146,46 +4146,62 @@
       <c r="C53" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="D53" s="3" t="str">
+      <c r="D53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E53" s="1"/>
-      <c r="G53" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="E53" s="1">
+        <v>50</v>
+      </c>
+      <c r="G53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H53" s="1"/>
-      <c r="J53" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H53" s="1">
+        <v>60</v>
+      </c>
+      <c r="J53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K53" s="1"/>
-      <c r="M53" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K53" s="1">
+        <v>20</v>
+      </c>
+      <c r="M53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N53" s="1"/>
-      <c r="P53" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="N53" s="1">
+        <v>40</v>
+      </c>
+      <c r="P53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q53" s="1"/>
-      <c r="S53" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Q53" s="1">
+        <v>0</v>
+      </c>
+      <c r="S53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T53" s="1"/>
-      <c r="V53" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T53" s="1">
+        <v>70</v>
+      </c>
+      <c r="V53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W53" s="1"/>
-      <c r="Y53" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W53" s="1">
+        <v>30</v>
+      </c>
+      <c r="Y53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z53" s="1"/>
+        <v>50</v>
+      </c>
+      <c r="Z53" s="1">
+        <v>100</v>
+      </c>
     </row>
     <row r="54" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
@@ -5949,56 +5965,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-127.5</v>
+        <v>-132.5</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>-27.5</v>
+        <v>-22.5</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-42.5</v>
+        <v>-62.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>365</v>
+        <v>355</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-55</v>
+        <v>-80</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-80</v>
+        <v>-60</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-212.5</v>
+        <v>-162.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 42 through 46
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04CBABC-E3C8-BC4F-B819-979F878E0D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD9BE28-F314-4A45-B1D1-2A13FCE4C063}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="-50420" yWindow="-3060" windowWidth="49000" windowHeight="27520" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4203,7 +4203,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="54" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>42</v>
       </c>
@@ -4213,48 +4213,60 @@
       <c r="C54" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="D54" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E54" s="1"/>
-      <c r="G54" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H54" s="1"/>
-      <c r="J54" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K54" s="1"/>
-      <c r="M54" s="3" t="str">
+      <c r="D54" s="3">
+        <v>0</v>
+      </c>
+      <c r="E54" s="1">
+        <v>60</v>
+      </c>
+      <c r="G54" s="3">
+        <v>0</v>
+      </c>
+      <c r="H54" s="1">
+        <v>60</v>
+      </c>
+      <c r="J54" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="K54" s="1">
+        <v>20</v>
+      </c>
+      <c r="M54" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N54" s="1"/>
-      <c r="P54" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N54" s="1">
+        <v>70</v>
+      </c>
+      <c r="P54" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q54" s="1"/>
-      <c r="S54" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(T54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T54" s="1"/>
-      <c r="V54" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Q54" s="1">
+        <v>40</v>
+      </c>
+      <c r="S54" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="T54" s="1">
+        <v>20</v>
+      </c>
+      <c r="V54" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W54" s="1"/>
-      <c r="Y54" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W54" s="1">
+        <v>30</v>
+      </c>
+      <c r="Y54" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z54, ($Z54,$W54,$T54,$Q54,$N54,$K54,$H54,$E54), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z54" s="1"/>
-    </row>
-    <row r="55" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+      <c r="Z54" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="55" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>43</v>
       </c>
@@ -4264,48 +4276,64 @@
       <c r="C55" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="D55" s="3" t="str">
+      <c r="D55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E55" s="1"/>
-      <c r="G55" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="E55" s="1">
+        <v>30</v>
+      </c>
+      <c r="G55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H55" s="1"/>
-      <c r="J55" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="H55" s="1">
+        <v>20</v>
+      </c>
+      <c r="J55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K55" s="1"/>
-      <c r="M55" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="K55" s="1">
+        <v>70</v>
+      </c>
+      <c r="M55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N55" s="1"/>
-      <c r="P55" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="N55" s="1">
+        <v>50</v>
+      </c>
+      <c r="P55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q55" s="1"/>
-      <c r="S55" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q55" s="1">
+        <v>60</v>
+      </c>
+      <c r="S55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T55" s="1"/>
-      <c r="V55" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="T55" s="1">
+        <v>0</v>
+      </c>
+      <c r="V55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W55" s="1"/>
-      <c r="Y55" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="W55" s="1">
+        <v>100</v>
+      </c>
+      <c r="Y55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z55" s="1"/>
-    </row>
-    <row r="56" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-10</v>
+      </c>
+      <c r="Z55" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="56" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
         <v>44</v>
       </c>
@@ -4315,48 +4343,62 @@
       <c r="C56" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="D56" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E56" s="1"/>
-      <c r="G56" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H56" s="1"/>
-      <c r="J56" s="3" t="str">
+      <c r="D56" s="3">
+        <v>12.5</v>
+      </c>
+      <c r="E56" s="1">
+        <v>70</v>
+      </c>
+      <c r="G56" s="3">
+        <v>12.5</v>
+      </c>
+      <c r="H56" s="1">
+        <v>70</v>
+      </c>
+      <c r="J56" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K56" s="1"/>
-      <c r="M56" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K56" s="1">
+        <v>20</v>
+      </c>
+      <c r="M56" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N56" s="1"/>
-      <c r="P56" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="N56" s="1">
+        <v>30</v>
+      </c>
+      <c r="P56" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q56" s="1"/>
-      <c r="S56" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Q56" s="1">
+        <v>0</v>
+      </c>
+      <c r="S56" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T56" s="1"/>
-      <c r="V56" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="T56" s="1">
+        <v>100</v>
+      </c>
+      <c r="V56" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W56" s="1"/>
-      <c r="Y56" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="W56" s="1">
+        <v>40</v>
+      </c>
+      <c r="Y56" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z56, ($Z56,$W56,$T56,$Q56,$N56,$K56,$H56,$E56), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z56" s="1"/>
-    </row>
-    <row r="57" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-5</v>
+      </c>
+      <c r="Z56" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="57" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>45</v>
       </c>
@@ -4366,48 +4408,64 @@
       <c r="C57" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="D57" s="3" t="str">
+      <c r="D57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E57" s="1"/>
-      <c r="G57" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="E57" s="1">
+        <v>100</v>
+      </c>
+      <c r="G57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H57" s="1"/>
-      <c r="J57" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="H57" s="1">
+        <v>50</v>
+      </c>
+      <c r="J57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K57" s="1"/>
-      <c r="M57" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K57" s="1">
+        <v>30</v>
+      </c>
+      <c r="M57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N57" s="1"/>
-      <c r="P57" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N57" s="1">
+        <v>70</v>
+      </c>
+      <c r="P57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q57" s="1"/>
-      <c r="S57" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q57" s="1">
+        <v>20</v>
+      </c>
+      <c r="S57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T57" s="1"/>
-      <c r="V57" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="T57" s="1">
+        <v>40</v>
+      </c>
+      <c r="V57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W57" s="1"/>
-      <c r="Y57" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="W57" s="1">
+        <v>60</v>
+      </c>
+      <c r="Y57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z57" s="1"/>
-    </row>
-    <row r="58" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-25</v>
+      </c>
+      <c r="Z57" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>46</v>
       </c>
@@ -4417,46 +4475,62 @@
       <c r="C58" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="D58" s="3" t="str">
+      <c r="D58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E58" s="1"/>
-      <c r="G58" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E58" s="1">
+        <v>70</v>
+      </c>
+      <c r="G58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H58" s="1"/>
-      <c r="J58" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="H58" s="1">
+        <v>100</v>
+      </c>
+      <c r="J58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K58" s="1"/>
-      <c r="M58" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="K58" s="1">
+        <v>50</v>
+      </c>
+      <c r="M58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N58" s="1"/>
-      <c r="P58" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N58" s="1">
+        <v>0</v>
+      </c>
+      <c r="P58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q58" s="1"/>
-      <c r="S58" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Q58" s="1">
+        <v>40</v>
+      </c>
+      <c r="S58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T58" s="1"/>
-      <c r="V58" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="T58" s="1">
+        <v>30</v>
+      </c>
+      <c r="V58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W58" s="1"/>
-      <c r="Y58" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="W58" s="1">
+        <v>20</v>
+      </c>
+      <c r="Y58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z58" s="1"/>
+        <v>5</v>
+      </c>
+      <c r="Z58" s="1">
+        <v>60</v>
+      </c>
     </row>
     <row r="59" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
@@ -5965,56 +6039,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-132.5</v>
+        <v>-65</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>-22.5</v>
+        <v>15</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-62.5</v>
+        <v>-105</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-80</v>
+        <v>-140</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-60</v>
+        <v>-82.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-162.5</v>
+        <v>-147.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 47 KKR vs DC
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD9BE28-F314-4A45-B1D1-2A13FCE4C063}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A50E33-A2C7-8F4F-9D3B-04AA20C082D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-50420" yWindow="-3060" windowWidth="49000" windowHeight="27520" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -4532,7 +4532,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="59" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>47</v>
       </c>
@@ -4542,46 +4542,62 @@
       <c r="C59" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="D59" s="3" t="str">
+      <c r="D59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E59" s="1"/>
-      <c r="G59" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="E59" s="1">
+        <v>100</v>
+      </c>
+      <c r="G59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H59" s="1"/>
-      <c r="J59" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H59" s="1">
+        <v>60</v>
+      </c>
+      <c r="J59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K59" s="1"/>
-      <c r="M59" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="K59" s="1">
+        <v>0</v>
+      </c>
+      <c r="M59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N59" s="1"/>
-      <c r="P59" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="N59" s="1">
+        <v>40</v>
+      </c>
+      <c r="P59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q59" s="1"/>
-      <c r="S59" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q59" s="1">
+        <v>20</v>
+      </c>
+      <c r="S59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T59" s="1"/>
-      <c r="V59" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T59" s="1">
+        <v>70</v>
+      </c>
+      <c r="V59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W59" s="1"/>
-      <c r="Y59" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W59" s="1">
+        <v>30</v>
+      </c>
+      <c r="Y59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z59" s="1"/>
+        <v>-5</v>
+      </c>
+      <c r="Z59" s="1">
+        <v>50</v>
+      </c>
     </row>
     <row r="60" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
@@ -6039,56 +6055,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-65</v>
+        <v>-15</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-105</v>
+        <v>-130</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>350</v>
+        <v>340</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-140</v>
+        <v>-160</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-82.5</v>
+        <v>-62.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-147.5</v>
+        <v>-152.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 48 and 49
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A50E33-A2C7-8F4F-9D3B-04AA20C082D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448ABD38-FEEF-2D45-8152-9C04402324DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-50420" yWindow="-3060" windowWidth="49000" windowHeight="27520" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -4599,7 +4599,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="60" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>48</v>
       </c>
@@ -4609,48 +4609,62 @@
       <c r="C60" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="D60" s="3" t="str">
+      <c r="D60" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E60" s="1"/>
-      <c r="G60" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E60" s="1">
+        <v>70</v>
+      </c>
+      <c r="G60" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H60" s="1"/>
-      <c r="J60" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K60" s="1"/>
-      <c r="M60" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="H60" s="1">
+        <v>100</v>
+      </c>
+      <c r="J60" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="K60" s="1">
+        <v>20</v>
+      </c>
+      <c r="M60" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N60" s="1"/>
-      <c r="P60" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="N60" s="1">
+        <v>30</v>
+      </c>
+      <c r="P60" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q60" s="1"/>
-      <c r="S60" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q60" s="1">
+        <v>60</v>
+      </c>
+      <c r="S60" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T60" s="1"/>
-      <c r="V60" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(W60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W60" s="1"/>
-      <c r="Y60" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="T60" s="1">
+        <v>40</v>
+      </c>
+      <c r="V60" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="W60" s="1">
+        <v>20</v>
+      </c>
+      <c r="Y60" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z60" s="1"/>
-    </row>
-    <row r="61" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-5</v>
+      </c>
+      <c r="Z60" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="61" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>49</v>
       </c>
@@ -4660,46 +4674,62 @@
       <c r="C61" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="D61" s="3" t="str">
+      <c r="D61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E61" s="1"/>
-      <c r="G61" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E61" s="1">
+        <v>40</v>
+      </c>
+      <c r="G61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H61" s="1"/>
-      <c r="J61" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="H61" s="1">
+        <v>30</v>
+      </c>
+      <c r="J61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K61" s="1"/>
-      <c r="M61" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="K61" s="1">
+        <v>0</v>
+      </c>
+      <c r="M61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N61" s="1"/>
-      <c r="P61" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N61" s="1">
+        <v>70</v>
+      </c>
+      <c r="P61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q61" s="1"/>
-      <c r="S61" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="Q61" s="1">
+        <v>50</v>
+      </c>
+      <c r="S61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T61" s="1"/>
-      <c r="V61" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="T61" s="1">
+        <v>100</v>
+      </c>
+      <c r="V61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W61" s="1"/>
-      <c r="Y61" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="W61" s="1">
+        <v>20</v>
+      </c>
+      <c r="Y61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z61" s="1"/>
+        <v>5</v>
+      </c>
+      <c r="Z61" s="1">
+        <v>60</v>
+      </c>
     </row>
     <row r="62" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
@@ -6055,28 +6085,28 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-15</v>
+        <v>-5</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-130</v>
+        <v>-177.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
@@ -6090,14 +6120,14 @@
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-62.5</v>
+        <v>-22.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>160</v>
+        <v>117.5</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Contest 50 SRH vs RR
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448ABD38-FEEF-2D45-8152-9C04402324DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F913774D-F06C-4B4A-B4B2-228D05B0AD97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-50420" yWindow="-3060" windowWidth="49000" windowHeight="27520" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4731,7 +4731,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
         <v>50</v>
       </c>
@@ -4741,46 +4741,62 @@
       <c r="C62" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="D62" s="3" t="str">
+      <c r="D62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E62" s="1"/>
-      <c r="G62" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E62" s="1">
+        <v>70</v>
+      </c>
+      <c r="G62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H62" s="1"/>
-      <c r="J62" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="H62" s="1">
+        <v>30</v>
+      </c>
+      <c r="J62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K62" s="1"/>
-      <c r="M62" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="K62" s="1">
+        <v>0</v>
+      </c>
+      <c r="M62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N62" s="1"/>
-      <c r="P62" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="N62" s="1">
+        <v>50</v>
+      </c>
+      <c r="P62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q62" s="1"/>
-      <c r="S62" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Q62" s="1">
+        <v>40</v>
+      </c>
+      <c r="S62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T62" s="1"/>
-      <c r="V62" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T62" s="1">
+        <v>60</v>
+      </c>
+      <c r="V62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W62" s="1"/>
-      <c r="Y62" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="W62" s="1">
+        <v>20</v>
+      </c>
+      <c r="Y62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z62" s="1"/>
+        <v>50</v>
+      </c>
+      <c r="Z62" s="1">
+        <v>100</v>
+      </c>
     </row>
     <row r="63" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
@@ -6085,56 +6101,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-5</v>
+        <v>15</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-177.5</v>
+        <v>-202.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-160</v>
+        <v>-170</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-22.5</v>
+        <v>-17.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>117.5</v>
+        <v>97.5</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-152.5</v>
+        <v>-102.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contests 51 through 51
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F913774D-F06C-4B4A-B4B2-228D05B0AD97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD50C5AC-59E5-F142-9CCE-3994C34055FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="-50420" yWindow="-3060" windowWidth="49000" windowHeight="27520" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4798,7 +4798,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="63" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
         <v>51</v>
       </c>
@@ -4808,48 +4808,64 @@
       <c r="C63" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="D63" s="3" t="str">
+      <c r="D63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E63" s="1"/>
-      <c r="G63" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="E63" s="1">
+        <v>30</v>
+      </c>
+      <c r="G63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H63" s="1"/>
-      <c r="J63" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="H63" s="1">
+        <v>70</v>
+      </c>
+      <c r="J63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K63" s="1"/>
-      <c r="M63" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="K63" s="1">
+        <v>0</v>
+      </c>
+      <c r="M63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N63" s="1"/>
-      <c r="P63" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="N63" s="1">
+        <v>60</v>
+      </c>
+      <c r="P63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q63" s="1"/>
-      <c r="S63" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="Q63" s="1">
+        <v>40</v>
+      </c>
+      <c r="S63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T63" s="1"/>
-      <c r="V63" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="T63" s="1">
+        <v>20</v>
+      </c>
+      <c r="V63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W63" s="1"/>
-      <c r="Y63" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="W63" s="1">
+        <v>50</v>
+      </c>
+      <c r="Y63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z63" s="1"/>
-    </row>
-    <row r="64" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+      <c r="Z63" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="64" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
         <v>52</v>
       </c>
@@ -4859,48 +4875,64 @@
       <c r="C64" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="D64" s="3" t="str">
+      <c r="D64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E64" s="1"/>
-      <c r="G64" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E64" s="1">
+        <v>70</v>
+      </c>
+      <c r="G64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H64" s="1"/>
-      <c r="J64" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H64" s="1">
+        <v>60</v>
+      </c>
+      <c r="J64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K64" s="1"/>
-      <c r="M64" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K64" s="1">
+        <v>30</v>
+      </c>
+      <c r="M64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N64" s="1"/>
-      <c r="P64" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N64" s="1">
+        <v>0</v>
+      </c>
+      <c r="P64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q64" s="1"/>
-      <c r="S64" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q64" s="1">
+        <v>100</v>
+      </c>
+      <c r="S64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T64" s="1"/>
-      <c r="V64" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="T64" s="1">
+        <v>50</v>
+      </c>
+      <c r="V64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W64" s="1"/>
-      <c r="Y64" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="W64" s="1">
+        <v>20</v>
+      </c>
+      <c r="Y64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z64" s="1"/>
-    </row>
-    <row r="65" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-10</v>
+      </c>
+      <c r="Z64" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="65" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>53</v>
       </c>
@@ -4910,48 +4942,64 @@
       <c r="C65" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="D65" s="3" t="str">
+      <c r="D65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E65" s="1"/>
-      <c r="G65" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E65" s="1">
+        <v>70</v>
+      </c>
+      <c r="G65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H65" s="1"/>
-      <c r="J65" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="H65" s="1">
+        <v>100</v>
+      </c>
+      <c r="J65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K65" s="1"/>
-      <c r="M65" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K65" s="1">
+        <v>30</v>
+      </c>
+      <c r="M65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N65" s="1"/>
-      <c r="P65" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="N65" s="1">
+        <v>60</v>
+      </c>
+      <c r="P65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q65" s="1"/>
-      <c r="S65" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Q65" s="1">
+        <v>0</v>
+      </c>
+      <c r="S65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T65" s="1"/>
-      <c r="V65" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="T65" s="1">
+        <v>40</v>
+      </c>
+      <c r="V65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W65" s="1"/>
-      <c r="Y65" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="W65" s="1">
+        <v>20</v>
+      </c>
+      <c r="Y65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z65" s="1"/>
-    </row>
-    <row r="66" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-5</v>
+      </c>
+      <c r="Z65" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="66" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>54</v>
       </c>
@@ -4961,46 +5009,62 @@
       <c r="C66" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="D66" s="3" t="str">
+      <c r="D66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E66" s="1"/>
-      <c r="G66" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E66" s="1">
+        <v>40</v>
+      </c>
+      <c r="G66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H66" s="1"/>
-      <c r="J66" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H66" s="1">
+        <v>60</v>
+      </c>
+      <c r="J66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K66" s="1"/>
-      <c r="M66" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="K66" s="1">
+        <v>100</v>
+      </c>
+      <c r="M66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N66" s="1"/>
-      <c r="P66" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N66" s="1">
+        <v>0</v>
+      </c>
+      <c r="P66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q66" s="1"/>
-      <c r="S66" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q66" s="1">
+        <v>20</v>
+      </c>
+      <c r="S66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T66" s="1"/>
-      <c r="V66" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="T66" s="1">
+        <v>50</v>
+      </c>
+      <c r="V66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W66" s="1"/>
-      <c r="Y66" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W66" s="1">
+        <v>30</v>
+      </c>
+      <c r="Y66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z66" s="1"/>
+        <v>20</v>
+      </c>
+      <c r="Z66" s="1">
+        <v>70</v>
+      </c>
     </row>
     <row r="67" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
@@ -6101,56 +6165,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>40</v>
+        <v>120</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-202.5</v>
+        <v>-207.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>340</v>
+        <v>300</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-170</v>
+        <v>-175</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-17.5</v>
+        <v>-57.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>97.5</v>
+        <v>37.5</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-102.5</v>
+        <v>-47.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 55 MI vs SRH
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD50C5AC-59E5-F142-9CCE-3994C34055FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7093C4A8-04E9-7A4A-B2D7-8EB13EA2FE62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-50420" yWindow="-3060" windowWidth="49000" windowHeight="27520" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="-50420" yWindow="-3180" windowWidth="49000" windowHeight="26800" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5066,7 +5066,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="67" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>55</v>
       </c>
@@ -5076,46 +5076,62 @@
       <c r="C67" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="D67" s="3" t="str">
+      <c r="D67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E67" s="1"/>
-      <c r="G67" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E67" s="1">
+        <v>70</v>
+      </c>
+      <c r="G67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H67" s="1"/>
-      <c r="J67" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="H67" s="1">
+        <v>100</v>
+      </c>
+      <c r="J67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K67" s="1"/>
-      <c r="M67" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="K67" s="1">
+        <v>50</v>
+      </c>
+      <c r="M67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N67" s="1"/>
-      <c r="P67" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="N67" s="1">
+        <v>40</v>
+      </c>
+      <c r="P67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q67" s="1"/>
-      <c r="S67" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q67" s="1">
+        <v>60</v>
+      </c>
+      <c r="S67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T67" s="1"/>
-      <c r="V67" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="T67" s="1">
+        <v>20</v>
+      </c>
+      <c r="V67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W67" s="1"/>
-      <c r="Y67" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="W67" s="1">
+        <v>30</v>
+      </c>
+      <c r="Y67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z67" s="1"/>
+        <v>-25</v>
+      </c>
+      <c r="Z67" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="68" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
@@ -6165,56 +6181,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-207.5</v>
+        <v>-212.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-175</v>
+        <v>-170</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-57.5</v>
+        <v>-77.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>37.5</v>
+        <v>22.5</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-47.5</v>
+        <v>-72.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 56 DC vs RR
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7093C4A8-04E9-7A4A-B2D7-8EB13EA2FE62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DBD84F-B1B0-CE4A-9E0D-E06C0D3C31EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-50420" yWindow="-3180" windowWidth="49000" windowHeight="26800" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -5133,7 +5133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>56</v>
       </c>
@@ -5143,46 +5143,62 @@
       <c r="C68" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="D68" s="3" t="str">
+      <c r="D68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E68" s="1"/>
-      <c r="G68" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E68" s="1">
+        <v>40</v>
+      </c>
+      <c r="G68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H68" s="1"/>
-      <c r="J68" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="H68" s="1">
+        <v>20</v>
+      </c>
+      <c r="J68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K68" s="1"/>
-      <c r="M68" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="K68" s="1">
+        <v>30</v>
+      </c>
+      <c r="M68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N68" s="1"/>
-      <c r="P68" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="N68" s="1">
+        <v>50</v>
+      </c>
+      <c r="P68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q68" s="1"/>
-      <c r="S68" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="Q68" s="1">
+        <v>0</v>
+      </c>
+      <c r="S68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T68" s="1"/>
-      <c r="V68" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T68" s="1">
+        <v>60</v>
+      </c>
+      <c r="V68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W68" s="1"/>
-      <c r="Y68" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="W68" s="1">
+        <v>100</v>
+      </c>
+      <c r="Y68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z68" s="1"/>
+        <v>20</v>
+      </c>
+      <c r="Z68" s="1">
+        <v>70</v>
+      </c>
     </row>
     <row r="69" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
@@ -6181,56 +6197,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-212.5</v>
+        <v>-227.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-170</v>
+        <v>-195</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-77.5</v>
+        <v>-72.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>22.5</v>
+        <v>72.5</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-72.5</v>
+        <v>-52.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 57 SRH vs LSG
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DBD84F-B1B0-CE4A-9E0D-E06C0D3C31EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA84D95-98CD-8546-8BB2-3720664E459C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-50420" yWindow="-3180" windowWidth="49000" windowHeight="26800" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -5200,7 +5200,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="69" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>57</v>
       </c>
@@ -5210,46 +5210,62 @@
       <c r="C69" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="D69" s="3" t="str">
+      <c r="D69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E69" s="1"/>
-      <c r="G69" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E69" s="1">
+        <v>40</v>
+      </c>
+      <c r="G69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H69" s="1"/>
-      <c r="J69" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="H69" s="1">
+        <v>20</v>
+      </c>
+      <c r="J69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K69" s="1"/>
-      <c r="M69" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="K69" s="1">
+        <v>0</v>
+      </c>
+      <c r="M69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N69" s="1"/>
-      <c r="P69" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N69" s="1">
+        <v>100</v>
+      </c>
+      <c r="P69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q69" s="1"/>
-      <c r="S69" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q69" s="1">
+        <v>70</v>
+      </c>
+      <c r="S69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T69" s="1"/>
-      <c r="V69" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="T69" s="1">
+        <v>30</v>
+      </c>
+      <c r="V69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W69" s="1"/>
-      <c r="Y69" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="W69" s="1">
+        <v>60</v>
+      </c>
+      <c r="Y69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z69" s="1"/>
+        <v>-5</v>
+      </c>
+      <c r="Z69" s="1">
+        <v>50</v>
+      </c>
     </row>
     <row r="70" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
@@ -6197,56 +6213,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-227.5</v>
+        <v>-252.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>285</v>
+        <v>335</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-195</v>
+        <v>-175</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-72.5</v>
+        <v>-87.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>72.5</v>
+        <v>77.5</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-52.5</v>
+        <v>-57.5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contests 59 through 62
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA84D95-98CD-8546-8BB2-3720664E459C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2E0E4C-97D4-E44D-B7C0-CDF168036E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-50420" yWindow="-3180" windowWidth="49000" windowHeight="26800" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -5267,7 +5267,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="70" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>58</v>
       </c>
@@ -5277,48 +5277,62 @@
       <c r="C70" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="D70" s="3" t="str">
+      <c r="D70" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E70" s="1"/>
-      <c r="G70" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H70" s="1"/>
-      <c r="J70" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="E70" s="1">
+        <v>60</v>
+      </c>
+      <c r="G70" s="3">
+        <v>-17.5</v>
+      </c>
+      <c r="H70" s="1">
+        <v>30</v>
+      </c>
+      <c r="J70" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K70" s="1"/>
-      <c r="M70" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="K70" s="1">
+        <v>70</v>
+      </c>
+      <c r="M70" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N70" s="1"/>
-      <c r="P70" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N70" s="1">
+        <v>0</v>
+      </c>
+      <c r="P70" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q70" s="1"/>
-      <c r="S70" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="Q70" s="1">
+        <v>50</v>
+      </c>
+      <c r="S70" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T70" s="1"/>
-      <c r="V70" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="T70" s="1">
+        <v>100</v>
+      </c>
+      <c r="V70" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W70" s="1"/>
-      <c r="Y70" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Z70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z70" s="1"/>
-    </row>
-    <row r="71" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-10</v>
+      </c>
+      <c r="W70" s="1">
+        <v>40</v>
+      </c>
+      <c r="Y70" s="3">
+        <v>-17.5</v>
+      </c>
+      <c r="Z70" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="71" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>59</v>
       </c>
@@ -5328,48 +5342,64 @@
       <c r="C71" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="D71" s="3" t="str">
+      <c r="D71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E71" s="1"/>
-      <c r="G71" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="E71" s="1">
+        <v>60</v>
+      </c>
+      <c r="G71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H71" s="1"/>
-      <c r="J71" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="H71" s="1">
+        <v>40</v>
+      </c>
+      <c r="J71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K71" s="1"/>
-      <c r="M71" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="K71" s="1">
+        <v>0</v>
+      </c>
+      <c r="M71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N71" s="1"/>
-      <c r="P71" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N71" s="1">
+        <v>70</v>
+      </c>
+      <c r="P71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q71" s="1"/>
-      <c r="S71" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q71" s="1">
+        <v>30</v>
+      </c>
+      <c r="S71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T71" s="1"/>
-      <c r="V71" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="T71" s="1">
+        <v>50</v>
+      </c>
+      <c r="V71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W71" s="1"/>
-      <c r="Y71" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="W71" s="1">
+        <v>100</v>
+      </c>
+      <c r="Y71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z71" s="1"/>
-    </row>
-    <row r="72" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-20</v>
+      </c>
+      <c r="Z71" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="72" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>60</v>
       </c>
@@ -5379,48 +5409,64 @@
       <c r="C72" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="D72" s="3" t="str">
+      <c r="D72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E72" s="1"/>
-      <c r="G72" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="E72" s="1">
+        <v>50</v>
+      </c>
+      <c r="G72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H72" s="1"/>
-      <c r="J72" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="H72" s="1">
+        <v>30</v>
+      </c>
+      <c r="J72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K72" s="1"/>
-      <c r="M72" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="K72" s="1">
+        <v>40</v>
+      </c>
+      <c r="M72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N72" s="1"/>
-      <c r="P72" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N72" s="1">
+        <v>100</v>
+      </c>
+      <c r="P72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q72" s="1"/>
-      <c r="S72" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q72" s="1">
+        <v>20</v>
+      </c>
+      <c r="S72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T72" s="1"/>
-      <c r="V72" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T72" s="1">
+        <v>60</v>
+      </c>
+      <c r="V72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W72" s="1"/>
-      <c r="Y72" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="W72" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z72" s="1"/>
-    </row>
-    <row r="73" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>20</v>
+      </c>
+      <c r="Z72" s="1">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="73" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>61</v>
       </c>
@@ -5430,48 +5476,64 @@
       <c r="C73" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="D73" s="3" t="str">
+      <c r="D73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E73" s="1"/>
-      <c r="G73" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E73" s="1">
+        <v>70</v>
+      </c>
+      <c r="G73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H73" s="1"/>
-      <c r="J73" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="H73" s="1">
+        <v>60</v>
+      </c>
+      <c r="J73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K73" s="1"/>
-      <c r="M73" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K73" s="1">
+        <v>20</v>
+      </c>
+      <c r="M73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N73" s="1"/>
-      <c r="P73" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N73" s="1">
+        <v>0</v>
+      </c>
+      <c r="P73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q73" s="1"/>
-      <c r="S73" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q73" s="1">
+        <v>30</v>
+      </c>
+      <c r="S73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T73" s="1"/>
-      <c r="V73" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="T73" s="1">
+        <v>100</v>
+      </c>
+      <c r="V73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W73" s="1"/>
-      <c r="Y73" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="W73" s="1">
+        <v>40</v>
+      </c>
+      <c r="Y73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z73" s="1"/>
-    </row>
-    <row r="74" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-5</v>
+      </c>
+      <c r="Z73" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="74" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>62</v>
       </c>
@@ -5481,46 +5543,60 @@
       <c r="C74" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="D74" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E74" s="1"/>
-      <c r="G74" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H74" s="1"/>
-      <c r="J74" s="3" t="str">
+      <c r="D74" s="3">
+        <v>-7.5</v>
+      </c>
+      <c r="E74" s="1">
+        <v>50</v>
+      </c>
+      <c r="G74" s="3">
+        <v>-7.5</v>
+      </c>
+      <c r="H74" s="1">
+        <v>50</v>
+      </c>
+      <c r="J74" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K74" s="1"/>
-      <c r="M74" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="K74" s="1">
+        <v>60</v>
+      </c>
+      <c r="M74" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N74" s="1"/>
-      <c r="P74" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N74" s="1">
+        <v>0</v>
+      </c>
+      <c r="P74" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q74" s="1"/>
-      <c r="S74" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q74" s="1">
+        <v>70</v>
+      </c>
+      <c r="S74" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T74" s="1"/>
-      <c r="V74" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="T74" s="1">
+        <v>100</v>
+      </c>
+      <c r="V74" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W74" s="1"/>
-      <c r="Y74" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="W74" s="1">
+        <v>20</v>
+      </c>
+      <c r="Y74" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z74, ($Z74,$W74,$T74,$Q74,$N74,$K74,$H74,$E74), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z74" s="1"/>
+        <v>-15</v>
+      </c>
+      <c r="Z74" s="1">
+        <v>30</v>
+      </c>
     </row>
     <row r="75" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
@@ -6213,56 +6289,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>30</v>
+        <v>47.5</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>130</v>
+        <v>85</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-252.5</v>
+        <v>-282.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-175</v>
+        <v>-210</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>-87.5</v>
+        <v>62.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>77.5</v>
+        <v>62.5</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-57.5</v>
+        <v>-95</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>
@@ -6376,7 +6452,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25E9A583-41BF-8143-84DF-F8B494A614D1}">
-  <dimension ref="E18:L81"/>
+  <dimension ref="E18:M82"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
@@ -7001,7 +7077,7 @@
         <v>-240</v>
       </c>
     </row>
-    <row r="81" spans="9:11" ht="21" x14ac:dyDescent="0.25">
+    <row r="81" spans="9:13" ht="21" x14ac:dyDescent="0.25">
       <c r="I81" s="1">
         <v>9</v>
       </c>
@@ -7010,6 +7086,20 @@
       </c>
       <c r="K81" s="10">
         <v>-410.35714285714289</v>
+      </c>
+    </row>
+    <row r="82" spans="9:13" x14ac:dyDescent="0.2">
+      <c r="K82">
+        <f>SUM(K73:K81)</f>
+        <v>0</v>
+      </c>
+      <c r="L82">
+        <f>SUM(K73:K76)</f>
+        <v>963.21428571428578</v>
+      </c>
+      <c r="M82">
+        <f>L82/9</f>
+        <v>107.02380952380953</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Results contest 64 DC vs LSG
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2E0E4C-97D4-E44D-B7C0-CDF168036E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C0A4F6-4BCD-9843-871D-F4DA047603CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-50420" yWindow="-3180" windowWidth="49000" windowHeight="26800" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -5598,7 +5598,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="75" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>63</v>
       </c>
@@ -5608,48 +5608,56 @@
       <c r="C75" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="D75" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E75" s="1"/>
-      <c r="G75" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H75" s="1"/>
-      <c r="J75" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K75" s="1"/>
-      <c r="M75" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N75" s="1"/>
-      <c r="P75" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Q75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q75" s="1"/>
-      <c r="S75" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(T75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T75" s="1"/>
-      <c r="V75" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(W75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W75" s="1"/>
-      <c r="Y75" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Z75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z75, ($Z75,$W75,$T75,$Q75,$N75,$K75,$H75,$E75), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z75" s="1"/>
-    </row>
-    <row r="76" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+      <c r="D75" s="3">
+        <v>0</v>
+      </c>
+      <c r="E75" s="1">
+        <v>0</v>
+      </c>
+      <c r="G75" s="3">
+        <v>0</v>
+      </c>
+      <c r="H75" s="1">
+        <v>0</v>
+      </c>
+      <c r="J75" s="3">
+        <v>0</v>
+      </c>
+      <c r="K75" s="1">
+        <v>0</v>
+      </c>
+      <c r="M75" s="3">
+        <v>0</v>
+      </c>
+      <c r="N75" s="1">
+        <v>0</v>
+      </c>
+      <c r="P75" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q75" s="1">
+        <v>0</v>
+      </c>
+      <c r="S75" s="3">
+        <v>0</v>
+      </c>
+      <c r="T75" s="1">
+        <v>0</v>
+      </c>
+      <c r="V75" s="3">
+        <v>0</v>
+      </c>
+      <c r="W75" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y75" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z75" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>64</v>
       </c>
@@ -5659,46 +5667,59 @@
       <c r="C76" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="D76" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E76" s="1"/>
-      <c r="G76" s="3" t="str">
+      <c r="D76" s="3">
+        <v>-20</v>
+      </c>
+      <c r="E76" s="1">
+        <v>0</v>
+      </c>
+      <c r="G76" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H76" s="1"/>
-      <c r="J76" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K76" s="1"/>
-      <c r="M76" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="H76" s="1">
+        <v>50</v>
+      </c>
+      <c r="J76" s="3">
+        <v>-20</v>
+      </c>
+      <c r="K76" s="1">
+        <v>0</v>
+      </c>
+      <c r="M76" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N76" s="1"/>
-      <c r="P76" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="N76" s="1">
+        <v>40</v>
+      </c>
+      <c r="P76" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q76" s="1"/>
-      <c r="S76" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q76" s="1">
+        <v>100</v>
+      </c>
+      <c r="S76" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T76" s="1"/>
-      <c r="V76" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(W76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W76" s="1"/>
-      <c r="Y76" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T76" s="1">
+        <v>60</v>
+      </c>
+      <c r="V76" s="3">
+        <v>-20</v>
+      </c>
+      <c r="W76" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y76" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z76, ($Z76,$W76,$T76,$Q76,$N76,$K76,$H76,$E76), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z76" s="1"/>
+        <v>20</v>
+      </c>
+      <c r="Z76" s="1">
+        <v>70</v>
+      </c>
     </row>
     <row r="77" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
@@ -6289,56 +6310,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>47.5</v>
+        <v>27.5</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-282.5</v>
+        <v>-302.5</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-210</v>
+        <v>-160</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>62.5</v>
+        <v>67.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>62.5</v>
+        <v>42.5</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-95</v>
+        <v>-75</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contest 65 RR vs PBKS
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C0A4F6-4BCD-9843-871D-F4DA047603CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071CB9EE-D570-3A46-9D14-258D18884350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-50420" yWindow="-3180" windowWidth="49000" windowHeight="26800" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5721,7 +5721,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="77" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
         <v>65</v>
       </c>
@@ -5731,46 +5731,60 @@
       <c r="C77" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="D77" s="3" t="str">
+      <c r="D77" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E77" s="1"/>
-      <c r="G77" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E77" s="1">
+        <v>70</v>
+      </c>
+      <c r="G77" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H77" s="1"/>
-      <c r="J77" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K77" s="1"/>
-      <c r="M77" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="H77" s="1">
+        <v>20</v>
+      </c>
+      <c r="J77" s="3">
+        <v>-12.5</v>
+      </c>
+      <c r="K77" s="1">
+        <v>40</v>
+      </c>
+      <c r="M77" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N77" s="1"/>
-      <c r="P77" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="N77" s="1">
+        <v>100</v>
+      </c>
+      <c r="P77" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q77" s="1"/>
-      <c r="S77" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q77" s="1">
+        <v>60</v>
+      </c>
+      <c r="S77" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T77" s="1"/>
-      <c r="V77" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(W77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W77" s="1"/>
-      <c r="Y77" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="T77" s="1">
+        <v>0</v>
+      </c>
+      <c r="V77" s="3">
+        <v>-12.5</v>
+      </c>
+      <c r="W77" s="1">
+        <v>40</v>
+      </c>
+      <c r="Y77" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z77" s="1"/>
+        <v>-5</v>
+      </c>
+      <c r="Z77" s="1">
+        <v>50</v>
+      </c>
     </row>
     <row r="78" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
@@ -6310,56 +6324,56 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>27.5</v>
+        <v>47.5</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-302.5</v>
+        <v>-315</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>320</v>
+        <v>370</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-160</v>
+        <v>-155</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>67.5</v>
+        <v>42.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>42.5</v>
+        <v>30</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-75</v>
+        <v>-80</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>

</xml_diff>

<commit_message>
Contests 66 through 70
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071CB9EE-D570-3A46-9D14-258D18884350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF71A22-7B77-A84F-B296-4C22AA4A6583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -122,12 +122,6 @@
     <t>JAYAGAN ARMY</t>
   </si>
   <si>
-    <t>Qualifier 1</t>
-  </si>
-  <si>
-    <t>Eliminator</t>
-  </si>
-  <si>
     <t>Qualifier 2</t>
   </si>
   <si>
@@ -381,6 +375,12 @@
   </si>
   <si>
     <t>RR vs KKR</t>
+  </si>
+  <si>
+    <t>Qualifier 1 KKR vs SRH</t>
+  </si>
+  <si>
+    <t>Eliminator RR vs RCB</t>
   </si>
 </sst>
 </file>
@@ -1184,6 +1184,7 @@
   <dimension ref="A1:AA89"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.5" bestFit="1" customWidth="1"/>
@@ -1213,7 +1214,7 @@
         <v>50</v>
       </c>
       <c r="I2" s="21" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="J2" s="21"/>
       <c r="K2" s="21"/>
@@ -1409,11 +1410,11 @@
       </c>
       <c r="Q11" s="20"/>
       <c r="S11" s="19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="T11" s="20"/>
       <c r="V11" s="19" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="W11" s="20"/>
       <c r="Y11" s="19" t="s">
@@ -1462,13 +1463,13 @@
         <v>0</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="T12" s="6" t="s">
         <v>0</v>
       </c>
       <c r="V12" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="W12" s="6" t="s">
         <v>0</v>
@@ -1555,7 +1556,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1620,7 +1621,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1685,7 +1686,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1752,7 +1753,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1819,7 +1820,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1886,7 +1887,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D19" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E19, ($Z19,$W19,$T19,$Q19,$N19,$K19,$H19,$E19), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E19, ($Z19,$W19,$T19,$Q19,$N19,$K19,$H19,$E19), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1953,7 +1954,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D20" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E20, ($Z20,$W20,$T20,$Q20,$N20,$K20,$H20,$E20), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E20, ($Z20,$W20,$T20,$Q20,$N20,$K20,$H20,$E20), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2020,7 +2021,7 @@
         <v>1</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2087,7 +2088,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2154,7 +2155,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2221,7 +2222,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D24" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2286,7 +2287,7 @@
         <v>1</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2353,7 +2354,7 @@
         <v>1</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D26" s="3">
         <v>-22.5</v>
@@ -2418,7 +2419,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2485,7 +2486,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2550,7 +2551,7 @@
         <v>1</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2617,7 +2618,7 @@
         <v>1</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2684,7 +2685,7 @@
         <v>1</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2749,7 +2750,7 @@
         <v>1</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D32" s="3">
         <v>-22.5</v>
@@ -2814,7 +2815,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2881,7 +2882,7 @@
         <v>1</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2948,7 +2949,7 @@
         <v>1</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3015,7 +3016,7 @@
         <v>1</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D36" s="3">
         <v>-22.5</v>
@@ -3078,7 +3079,7 @@
         <v>1</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3145,7 +3146,7 @@
         <v>1</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3212,7 +3213,7 @@
         <v>1</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D39" s="3">
         <v>35</v>
@@ -3277,7 +3278,7 @@
         <v>1</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3344,7 +3345,7 @@
         <v>1</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3411,7 +3412,7 @@
         <v>1</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3478,7 +3479,7 @@
         <v>1</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D43" s="3">
         <v>-7.5</v>
@@ -3543,7 +3544,7 @@
         <v>1</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3610,7 +3611,7 @@
         <v>1</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3677,7 +3678,7 @@
         <v>1</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3744,7 +3745,7 @@
         <v>1</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3811,7 +3812,7 @@
         <v>1</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3878,7 +3879,7 @@
         <v>1</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3945,7 +3946,7 @@
         <v>1</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4012,7 +4013,7 @@
         <v>1</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4079,7 +4080,7 @@
         <v>1</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D52" s="3">
         <v>-22.5</v>
@@ -4144,7 +4145,7 @@
         <v>1</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4211,7 +4212,7 @@
         <v>1</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D54" s="3">
         <v>0</v>
@@ -4274,7 +4275,7 @@
         <v>1</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4341,7 +4342,7 @@
         <v>1</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D56" s="3">
         <v>12.5</v>
@@ -4406,7 +4407,7 @@
         <v>1</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4473,7 +4474,7 @@
         <v>1</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4540,7 +4541,7 @@
         <v>1</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4607,7 +4608,7 @@
         <v>1</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D60" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4672,7 +4673,7 @@
         <v>1</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4739,7 +4740,7 @@
         <v>1</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4806,7 +4807,7 @@
         <v>1</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4873,7 +4874,7 @@
         <v>1</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4940,7 +4941,7 @@
         <v>1</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5007,7 +5008,7 @@
         <v>1</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5074,7 +5075,7 @@
         <v>1</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5141,7 +5142,7 @@
         <v>1</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5208,7 +5209,7 @@
         <v>1</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5275,7 +5276,7 @@
         <v>1</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D70" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5340,7 +5341,7 @@
         <v>1</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5407,7 +5408,7 @@
         <v>1</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5474,7 +5475,7 @@
         <v>1</v>
       </c>
       <c r="C73" s="14" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5541,7 +5542,7 @@
         <v>1</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D74" s="3">
         <v>-7.5</v>
@@ -5606,7 +5607,7 @@
         <v>1</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D75" s="3">
         <v>0</v>
@@ -5665,7 +5666,7 @@
         <v>1</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D76" s="3">
         <v>-20</v>
@@ -5729,7 +5730,7 @@
         <v>1</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D77" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5786,7 +5787,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="78" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
         <v>66</v>
       </c>
@@ -5794,50 +5795,58 @@
         <v>1</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="D78" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E78" s="1"/>
-      <c r="G78" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H78" s="1"/>
-      <c r="J78" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K78" s="1"/>
-      <c r="M78" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N78" s="1"/>
-      <c r="P78" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Q78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q78" s="1"/>
-      <c r="S78" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(T78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T78" s="1"/>
-      <c r="V78" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(W78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W78" s="1"/>
-      <c r="Y78" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Z78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z78, ($Z78,$W78,$T78,$Q78,$N78,$K78,$H78,$E78), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z78" s="1"/>
-    </row>
-    <row r="79" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="D78" s="3">
+        <v>0</v>
+      </c>
+      <c r="E78" s="1">
+        <v>0</v>
+      </c>
+      <c r="G78" s="3">
+        <v>0</v>
+      </c>
+      <c r="H78" s="1">
+        <v>0</v>
+      </c>
+      <c r="J78" s="3">
+        <v>0</v>
+      </c>
+      <c r="K78" s="1">
+        <v>0</v>
+      </c>
+      <c r="M78" s="3">
+        <v>0</v>
+      </c>
+      <c r="N78" s="1">
+        <v>0</v>
+      </c>
+      <c r="P78" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="1">
+        <v>0</v>
+      </c>
+      <c r="S78" s="3">
+        <v>0</v>
+      </c>
+      <c r="T78" s="1">
+        <v>0</v>
+      </c>
+      <c r="V78" s="3">
+        <v>0</v>
+      </c>
+      <c r="W78" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y78" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z78" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A79" s="1">
         <v>67</v>
       </c>
@@ -5845,50 +5854,66 @@
         <v>1</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="D79" s="3" t="str">
+        <v>107</v>
+      </c>
+      <c r="D79" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E79" s="1"/>
-      <c r="G79" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="E79" s="1">
+        <v>40</v>
+      </c>
+      <c r="G79" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H79" s="1"/>
-      <c r="J79" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="H79" s="1">
+        <v>100</v>
+      </c>
+      <c r="J79" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K79" s="1"/>
-      <c r="M79" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="K79" s="1">
+        <v>60</v>
+      </c>
+      <c r="M79" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N79" s="1"/>
-      <c r="P79" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="N79" s="1">
+        <v>70</v>
+      </c>
+      <c r="P79" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q79" s="1"/>
-      <c r="S79" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="Q79" s="1">
+        <v>20</v>
+      </c>
+      <c r="S79" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T79" s="1"/>
-      <c r="V79" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="T79" s="1">
+        <v>50</v>
+      </c>
+      <c r="V79" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W79" s="1"/>
-      <c r="Y79" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="W79" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y79" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z79" s="1"/>
-    </row>
-    <row r="80" spans="1:26" hidden="1" x14ac:dyDescent="0.2">
+        <v>-15</v>
+      </c>
+      <c r="Z79" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="80" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A80" s="1">
         <v>68</v>
       </c>
@@ -5896,50 +5921,66 @@
         <v>1</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="D80" s="3" t="str">
+        <v>108</v>
+      </c>
+      <c r="D80" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E80" s="1"/>
-      <c r="G80" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="E80" s="1">
+        <v>0</v>
+      </c>
+      <c r="G80" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H80" s="1"/>
-      <c r="J80" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="H80" s="1">
+        <v>50</v>
+      </c>
+      <c r="J80" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K80" s="1"/>
-      <c r="M80" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K80" s="1">
+        <v>20</v>
+      </c>
+      <c r="M80" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N80" s="1"/>
-      <c r="P80" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="N80" s="1">
+        <v>40</v>
+      </c>
+      <c r="P80" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q80" s="1"/>
-      <c r="S80" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q80" s="1">
+        <v>60</v>
+      </c>
+      <c r="S80" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T80" s="1"/>
-      <c r="V80" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="T80" s="1">
+        <v>30</v>
+      </c>
+      <c r="V80" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W80" s="1"/>
-      <c r="Y80" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="W80" s="1">
+        <v>70</v>
+      </c>
+      <c r="Y80" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z80" s="1"/>
-    </row>
-    <row r="81" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+      <c r="Z80" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="81" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
         <v>69</v>
       </c>
@@ -5947,50 +5988,64 @@
         <v>1</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="D81" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E81" s="1"/>
-      <c r="G81" s="3" t="str">
+        <v>109</v>
+      </c>
+      <c r="D81" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="E81" s="1">
+        <v>20</v>
+      </c>
+      <c r="G81" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H81" s="1"/>
-      <c r="J81" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="H81" s="1">
+        <v>40</v>
+      </c>
+      <c r="J81" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K81" s="1"/>
-      <c r="M81" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N81" s="1"/>
-      <c r="P81" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="K81" s="1">
+        <v>50</v>
+      </c>
+      <c r="M81" s="3">
+        <v>-22.5</v>
+      </c>
+      <c r="N81" s="1">
+        <v>20</v>
+      </c>
+      <c r="P81" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q81" s="1"/>
-      <c r="S81" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="Q81" s="1">
+        <v>30</v>
+      </c>
+      <c r="S81" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T81" s="1"/>
-      <c r="V81" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="T81" s="1">
+        <v>70</v>
+      </c>
+      <c r="V81" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W81" s="1"/>
-      <c r="Y81" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="W81" s="1">
+        <v>60</v>
+      </c>
+      <c r="Y81" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z81, ($Z81,$W81,$T81,$Q81,$N81,$K81,$H81,$E81), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z81" s="1"/>
-    </row>
-    <row r="82" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+      <c r="Z81" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="82" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A82" s="1">
         <v>70</v>
       </c>
@@ -5998,52 +6053,60 @@
         <v>1</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="D82" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E82" s="1"/>
-      <c r="G82" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H82" s="1"/>
-      <c r="J82" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K82" s="1"/>
-      <c r="M82" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N82" s="1"/>
-      <c r="P82" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Q82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q82" s="1"/>
-      <c r="S82" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(T82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T82" s="1"/>
-      <c r="V82" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(W82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W82" s="1"/>
-      <c r="Y82" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Z82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z82, ($Z82,$W82,$T82,$Q82,$N82,$K82,$H82,$E82), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z82" s="1"/>
+        <v>110</v>
+      </c>
+      <c r="D82" s="3">
+        <v>0</v>
+      </c>
+      <c r="E82" s="1">
+        <v>0</v>
+      </c>
+      <c r="G82" s="3">
+        <v>0</v>
+      </c>
+      <c r="H82" s="1">
+        <v>0</v>
+      </c>
+      <c r="J82" s="3">
+        <v>0</v>
+      </c>
+      <c r="K82" s="1">
+        <v>0</v>
+      </c>
+      <c r="M82" s="3">
+        <v>0</v>
+      </c>
+      <c r="N82" s="1">
+        <v>0</v>
+      </c>
+      <c r="P82" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q82" s="1">
+        <v>0</v>
+      </c>
+      <c r="S82" s="3">
+        <v>0</v>
+      </c>
+      <c r="T82" s="1">
+        <v>0</v>
+      </c>
+      <c r="V82" s="3">
+        <v>0</v>
+      </c>
+      <c r="W82" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y82" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z82" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="83" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A83" s="5" t="s">
-        <v>26</v>
+        <v>111</v>
       </c>
       <c r="B83" s="1">
         <v>1</v>
@@ -6092,7 +6155,7 @@
     </row>
     <row r="84" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A84" s="5" t="s">
-        <v>27</v>
+        <v>112</v>
       </c>
       <c r="B84" s="1">
         <v>1</v>
@@ -6141,7 +6204,7 @@
     </row>
     <row r="85" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A85" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B85" s="1">
         <v>1</v>
@@ -6190,7 +6253,7 @@
     </row>
     <row r="86" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A86" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B86" s="1">
         <v>1</v>
@@ -6324,35 +6387,35 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>47.5</v>
+        <v>-10</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-315</v>
+        <v>-335</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>370</v>
+        <v>357.5</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-155</v>
+        <v>-185</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
@@ -6373,7 +6436,7 @@
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-80</v>
+        <v>5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>
@@ -6505,7 +6568,7 @@
     <row r="23" spans="5:10" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="27" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E27" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>17</v>
@@ -6514,7 +6577,7 @@
         <v>18</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>24</v>
@@ -6531,7 +6594,7 @@
         <v>5</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J28" s="6" t="s">
         <v>13</v>
@@ -6605,7 +6668,7 @@
     </row>
     <row r="35" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E35" s="15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F35" s="12" t="s">
         <v>24</v>
@@ -6627,7 +6690,7 @@
     </row>
     <row r="39" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E39" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F39" s="6" t="s">
         <v>17</v>
@@ -6636,7 +6699,7 @@
         <v>18</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J39" s="6" t="s">
         <v>9</v>
@@ -6653,7 +6716,7 @@
         <v>20</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J40" s="6" t="s">
         <v>5</v>
@@ -6727,7 +6790,7 @@
     </row>
     <row r="47" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E47" s="15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F47" s="12" t="s">
         <v>20</v>
@@ -6754,7 +6817,7 @@
     </row>
     <row r="50" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E50" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>17</v>
@@ -6763,7 +6826,7 @@
         <v>18</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J50" s="6" t="s">
         <v>13</v>
@@ -6780,7 +6843,7 @@
         <v>10</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J51" s="6" t="s">
         <v>9</v>
@@ -6854,7 +6917,7 @@
     </row>
     <row r="58" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E58" s="15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F58" s="12" t="s">
         <v>19</v>
@@ -6881,7 +6944,7 @@
     </row>
     <row r="61" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E61" s="16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F61" s="6" t="s">
         <v>17</v>
@@ -6890,7 +6953,7 @@
         <v>18</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J61" s="6" t="s">
         <v>20</v>
@@ -6907,7 +6970,7 @@
         <v>5</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J62" s="6" t="s">
         <v>24</v>
@@ -6981,7 +7044,7 @@
     </row>
     <row r="69" spans="5:12" ht="19" x14ac:dyDescent="0.25">
       <c r="E69" s="15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F69" s="12" t="s">
         <v>19</v>
@@ -7006,7 +7069,7 @@
         <v>11</v>
       </c>
       <c r="J72" s="16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K72" s="16" t="s">
         <v>7</v>
@@ -7023,7 +7086,7 @@
         <v>473.92857142857144</v>
       </c>
       <c r="L73" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="74" spans="5:12" ht="21" x14ac:dyDescent="0.25">
@@ -7031,13 +7094,13 @@
         <v>2</v>
       </c>
       <c r="J74" s="15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K74" s="10">
         <v>366.42857142857144</v>
       </c>
       <c r="L74" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="75" spans="5:12" ht="21" x14ac:dyDescent="0.25">
@@ -7051,7 +7114,7 @@
         <v>112.85714285714283</v>
       </c>
       <c r="L75" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="76" spans="5:12" ht="21" x14ac:dyDescent="0.25">
@@ -7065,7 +7128,7 @@
         <v>10</v>
       </c>
       <c r="L76" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="77" spans="5:12" ht="21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Qualifier 1 KKR vs SRH
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF71A22-7B77-A84F-B296-4C22AA4A6583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C62B9FF-99D4-614B-BEFD-1A0AF851B377}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="-50420" yWindow="-3180" windowWidth="49000" windowHeight="26800" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="125">
   <si>
     <t>Points</t>
   </si>
@@ -122,6 +122,12 @@
     <t>JAYAGAN ARMY</t>
   </si>
   <si>
+    <t>Qualifier 1</t>
+  </si>
+  <si>
+    <t>Eliminator</t>
+  </si>
+  <si>
     <t>Qualifier 2</t>
   </si>
   <si>
@@ -131,9 +137,6 @@
     <t>Vikcy</t>
   </si>
   <si>
-    <t>Qualifier 1 DC vs CSK</t>
-  </si>
-  <si>
     <t>Eliminator RCB vs KKR</t>
   </si>
   <si>
@@ -381,13 +384,46 @@
   </si>
   <si>
     <t>Eliminator RR vs RCB</t>
+  </si>
+  <si>
+    <t>Rapaka</t>
+  </si>
+  <si>
+    <t>Winner Prediction - Coins</t>
+  </si>
+  <si>
+    <t>Scorecard</t>
+  </si>
+  <si>
+    <t>Format 1</t>
+  </si>
+  <si>
+    <t>Format 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final score </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finals </t>
+  </si>
+  <si>
+    <t>Total coins</t>
+  </si>
+  <si>
+    <t>Outgoing</t>
+  </si>
+  <si>
+    <t>Coins</t>
+  </si>
+  <si>
+    <t>Incoming</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -434,8 +470,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -472,8 +530,25 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC5E0B3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -546,12 +621,87 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -590,12 +740,52 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="20% - Accent6" xfId="1" builtinId="50"/>
+    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="33">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -613,16 +803,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -748,6 +928,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -763,16 +953,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -863,6 +1043,76 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1181,7 +1431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BE9CB7-B9A7-B347-86F0-C3EB9B5BFBBD}">
-  <dimension ref="A1:AA89"/>
+  <dimension ref="A1:AA107"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
@@ -1214,7 +1464,7 @@
         <v>50</v>
       </c>
       <c r="I2" s="21" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J2" s="21"/>
       <c r="K2" s="21"/>
@@ -1410,11 +1660,11 @@
       </c>
       <c r="Q11" s="20"/>
       <c r="S11" s="19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="T11" s="20"/>
       <c r="V11" s="19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="W11" s="20"/>
       <c r="Y11" s="19" t="s">
@@ -1463,13 +1713,13 @@
         <v>0</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="T12" s="6" t="s">
         <v>0</v>
       </c>
       <c r="V12" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W12" s="6" t="s">
         <v>0</v>
@@ -1556,7 +1806,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1621,7 +1871,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1686,7 +1936,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1753,7 +2003,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1820,7 +2070,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1887,7 +2137,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D19" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E19, ($Z19,$W19,$T19,$Q19,$N19,$K19,$H19,$E19), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E19, ($Z19,$W19,$T19,$Q19,$N19,$K19,$H19,$E19), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1954,7 +2204,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D20" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E20, ($Z20,$W20,$T20,$Q20,$N20,$K20,$H20,$E20), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E20, ($Z20,$W20,$T20,$Q20,$N20,$K20,$H20,$E20), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2021,7 +2271,7 @@
         <v>1</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2088,7 +2338,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2155,7 +2405,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2222,7 +2472,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D24" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2287,7 +2537,7 @@
         <v>1</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2354,7 +2604,7 @@
         <v>1</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D26" s="3">
         <v>-22.5</v>
@@ -2419,7 +2669,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2486,7 +2736,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2551,7 +2801,7 @@
         <v>1</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2618,7 +2868,7 @@
         <v>1</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2685,7 +2935,7 @@
         <v>1</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2750,7 +3000,7 @@
         <v>1</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D32" s="3">
         <v>-22.5</v>
@@ -2815,7 +3065,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2882,7 +3132,7 @@
         <v>1</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2949,7 +3199,7 @@
         <v>1</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3016,7 +3266,7 @@
         <v>1</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D36" s="3">
         <v>-22.5</v>
@@ -3079,7 +3329,7 @@
         <v>1</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3146,7 +3396,7 @@
         <v>1</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3213,7 +3463,7 @@
         <v>1</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D39" s="3">
         <v>35</v>
@@ -3278,7 +3528,7 @@
         <v>1</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3345,7 +3595,7 @@
         <v>1</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3412,7 +3662,7 @@
         <v>1</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3479,7 +3729,7 @@
         <v>1</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D43" s="3">
         <v>-7.5</v>
@@ -3544,7 +3794,7 @@
         <v>1</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3611,7 +3861,7 @@
         <v>1</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3678,7 +3928,7 @@
         <v>1</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3745,7 +3995,7 @@
         <v>1</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3812,7 +4062,7 @@
         <v>1</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3879,7 +4129,7 @@
         <v>1</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3946,7 +4196,7 @@
         <v>1</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4013,7 +4263,7 @@
         <v>1</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4080,7 +4330,7 @@
         <v>1</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D52" s="3">
         <v>-22.5</v>
@@ -4145,7 +4395,7 @@
         <v>1</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4212,7 +4462,7 @@
         <v>1</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D54" s="3">
         <v>0</v>
@@ -4275,7 +4525,7 @@
         <v>1</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4342,7 +4592,7 @@
         <v>1</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D56" s="3">
         <v>12.5</v>
@@ -4407,7 +4657,7 @@
         <v>1</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4474,7 +4724,7 @@
         <v>1</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4541,7 +4791,7 @@
         <v>1</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4608,7 +4858,7 @@
         <v>1</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D60" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4673,7 +4923,7 @@
         <v>1</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4740,7 +4990,7 @@
         <v>1</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4807,7 +5057,7 @@
         <v>1</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4874,7 +5124,7 @@
         <v>1</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4941,7 +5191,7 @@
         <v>1</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5008,7 +5258,7 @@
         <v>1</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5075,7 +5325,7 @@
         <v>1</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5142,7 +5392,7 @@
         <v>1</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5209,7 +5459,7 @@
         <v>1</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5276,7 +5526,7 @@
         <v>1</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D70" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5341,7 +5591,7 @@
         <v>1</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5408,7 +5658,7 @@
         <v>1</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5475,7 +5725,7 @@
         <v>1</v>
       </c>
       <c r="C73" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5542,7 +5792,7 @@
         <v>1</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D74" s="3">
         <v>-7.5</v>
@@ -5607,7 +5857,7 @@
         <v>1</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D75" s="3">
         <v>0</v>
@@ -5666,7 +5916,7 @@
         <v>1</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D76" s="3">
         <v>-20</v>
@@ -5730,7 +5980,7 @@
         <v>1</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D77" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5795,7 +6045,7 @@
         <v>1</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D78" s="3">
         <v>0</v>
@@ -5854,7 +6104,7 @@
         <v>1</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D79" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5921,7 +6171,7 @@
         <v>1</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D80" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5988,7 +6238,7 @@
         <v>1</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D81" s="3">
         <v>-22.5</v>
@@ -6053,7 +6303,7 @@
         <v>1</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D82" s="3">
         <v>0</v>
@@ -6106,56 +6356,72 @@
     </row>
     <row r="83" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A83" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B83" s="1">
         <v>1</v>
       </c>
       <c r="C83" s="14"/>
-      <c r="D83" s="3" t="str">
+      <c r="D83" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E83" s="1"/>
-      <c r="G83" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="E83" s="1">
+        <v>70</v>
+      </c>
+      <c r="G83" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H83" s="1"/>
-      <c r="J83" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="H83" s="1">
+        <v>30</v>
+      </c>
+      <c r="J83" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K83" s="1"/>
-      <c r="M83" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="K83" s="1">
+        <v>20</v>
+      </c>
+      <c r="M83" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N83" s="1"/>
-      <c r="P83" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N83" s="1">
+        <v>0</v>
+      </c>
+      <c r="P83" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q83" s="1"/>
-      <c r="S83" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q83" s="1">
+        <v>100</v>
+      </c>
+      <c r="S83" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T83" s="1"/>
-      <c r="V83" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="T83" s="1">
+        <v>50</v>
+      </c>
+      <c r="V83" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W83" s="1"/>
-      <c r="Y83" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="W83" s="1">
+        <v>60</v>
+      </c>
+      <c r="Y83" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z83" s="1"/>
+        <v>-10</v>
+      </c>
+      <c r="Z83" s="1">
+        <v>40</v>
+      </c>
     </row>
     <row r="84" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A84" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B84" s="1">
         <v>1</v>
@@ -6204,7 +6470,7 @@
     </row>
     <row r="85" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A85" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B85" s="1">
         <v>1</v>
@@ -6253,7 +6519,7 @@
     </row>
     <row r="86" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A86" s="5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B86" s="1">
         <v>1</v>
@@ -6387,66 +6653,449 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>-10</v>
+        <v>10</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-335</v>
+        <v>-355</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>357.5</v>
+        <v>332.5</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-185</v>
+        <v>-135</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>42.5</v>
+        <v>37.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>5</v>
+        <v>-5</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>
         <v>0</v>
       </c>
     </row>
+    <row r="97" spans="4:22" ht="19" x14ac:dyDescent="0.25">
+      <c r="E97" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="F97" s="26"/>
+      <c r="G97" s="26"/>
+      <c r="H97" s="26"/>
+      <c r="I97" s="27"/>
+      <c r="P97" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="Q97" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="R97" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="S97" s="31"/>
+      <c r="T97" s="32"/>
+      <c r="U97" s="29" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="98" spans="4:22" ht="19" x14ac:dyDescent="0.25">
+      <c r="E98" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F98" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="G98" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="H98" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="I98" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="P98" s="34"/>
+      <c r="Q98" s="29"/>
+      <c r="R98" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="S98" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="T98" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="U98" s="29"/>
+    </row>
+    <row r="99" spans="4:22" ht="21" x14ac:dyDescent="0.25">
+      <c r="D99" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E99" s="1">
+        <v>3</v>
+      </c>
+      <c r="F99" s="1"/>
+      <c r="G99" s="1"/>
+      <c r="H99" s="1"/>
+      <c r="I99" s="15">
+        <f>SUM(E99:H99)</f>
+        <v>3</v>
+      </c>
+      <c r="P99" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q99" s="10">
+        <f>E89</f>
+        <v>10</v>
+      </c>
+      <c r="R99" s="35">
+        <v>-400</v>
+      </c>
+      <c r="S99" s="10">
+        <f>I99</f>
+        <v>3</v>
+      </c>
+      <c r="T99" s="10">
+        <f>IFERROR((-SUM($R$99:$R$106)/SUM($S$99:$S$106))*$S99, 0)</f>
+        <v>3200</v>
+      </c>
+      <c r="U99" s="10">
+        <f>SUM(Q99,R99,T99)</f>
+        <v>2810</v>
+      </c>
+      <c r="V99" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="100" spans="4:22" ht="21" x14ac:dyDescent="0.25">
+      <c r="D100" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E100" s="1">
+        <v>0</v>
+      </c>
+      <c r="F100" s="1"/>
+      <c r="G100" s="1"/>
+      <c r="H100" s="1"/>
+      <c r="I100" s="15">
+        <f t="shared" ref="I100:I106" si="0">SUM(E100:H100)</f>
+        <v>0</v>
+      </c>
+      <c r="P100" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q100" s="10">
+        <f>H89</f>
+        <v>80</v>
+      </c>
+      <c r="R100" s="35">
+        <v>-400</v>
+      </c>
+      <c r="S100" s="10">
+        <f t="shared" ref="S100:S106" si="1">I100</f>
+        <v>0</v>
+      </c>
+      <c r="T100" s="10">
+        <f t="shared" ref="T100:T106" si="2">IFERROR((-SUM($R$99:$R$106)/SUM($S$99:$S$106))*$S100, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="U100" s="10">
+        <f t="shared" ref="U100:U106" si="3">SUM(Q100,R100,T100)</f>
+        <v>-320</v>
+      </c>
+      <c r="V100" s="15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="101" spans="4:22" ht="21" x14ac:dyDescent="0.25">
+      <c r="D101" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E101" s="1">
+        <v>0</v>
+      </c>
+      <c r="F101" s="1"/>
+      <c r="G101" s="1"/>
+      <c r="H101" s="1"/>
+      <c r="I101" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P101" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q101" s="10">
+        <f>K89</f>
+        <v>-355</v>
+      </c>
+      <c r="R101" s="35">
+        <v>-400</v>
+      </c>
+      <c r="S101" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T101" s="10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U101" s="10">
+        <f t="shared" si="3"/>
+        <v>-755</v>
+      </c>
+      <c r="V101" s="15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="4:22" ht="21" x14ac:dyDescent="0.25">
+      <c r="D102" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E102" s="1">
+        <v>0</v>
+      </c>
+      <c r="F102" s="1"/>
+      <c r="G102" s="1"/>
+      <c r="H102" s="1"/>
+      <c r="I102" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P102" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q102" s="10">
+        <f>N89</f>
+        <v>332.5</v>
+      </c>
+      <c r="R102" s="35">
+        <v>-400</v>
+      </c>
+      <c r="S102" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T102" s="10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U102" s="10">
+        <f t="shared" si="3"/>
+        <v>-67.5</v>
+      </c>
+      <c r="V102" s="15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="103" spans="4:22" ht="21" x14ac:dyDescent="0.25">
+      <c r="D103" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E103" s="1">
+        <v>0</v>
+      </c>
+      <c r="F103" s="1"/>
+      <c r="G103" s="1"/>
+      <c r="H103" s="1"/>
+      <c r="I103" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P103" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q103" s="10">
+        <f>Q89</f>
+        <v>-135</v>
+      </c>
+      <c r="R103" s="35">
+        <v>-400</v>
+      </c>
+      <c r="S103" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T103" s="10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U103" s="10">
+        <f t="shared" si="3"/>
+        <v>-535</v>
+      </c>
+      <c r="V103" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="104" spans="4:22" ht="21" x14ac:dyDescent="0.25">
+      <c r="D104" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="E104" s="1">
+        <v>0</v>
+      </c>
+      <c r="F104" s="1"/>
+      <c r="G104" s="1"/>
+      <c r="H104" s="1"/>
+      <c r="I104" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P104" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q104" s="10">
+        <f>T89</f>
+        <v>37.5</v>
+      </c>
+      <c r="R104" s="35">
+        <v>-400</v>
+      </c>
+      <c r="S104" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T104" s="10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U104" s="10">
+        <f t="shared" si="3"/>
+        <v>-362.5</v>
+      </c>
+      <c r="V104" s="15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="105" spans="4:22" ht="21" x14ac:dyDescent="0.25">
+      <c r="D105" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="E105" s="1">
+        <v>0</v>
+      </c>
+      <c r="F105" s="1"/>
+      <c r="G105" s="1"/>
+      <c r="H105" s="1"/>
+      <c r="I105" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P105" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q105" s="10">
+        <f>W89</f>
+        <v>35</v>
+      </c>
+      <c r="R105" s="35">
+        <v>-400</v>
+      </c>
+      <c r="S105" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T105" s="10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U105" s="10">
+        <f t="shared" si="3"/>
+        <v>-365</v>
+      </c>
+      <c r="V105" s="15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="106" spans="4:22" ht="21" x14ac:dyDescent="0.25">
+      <c r="D106" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E106" s="1">
+        <v>0</v>
+      </c>
+      <c r="F106" s="1"/>
+      <c r="G106" s="1"/>
+      <c r="H106" s="1"/>
+      <c r="I106" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P106" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q106" s="10">
+        <f>Z89</f>
+        <v>-5</v>
+      </c>
+      <c r="R106" s="35">
+        <v>-400</v>
+      </c>
+      <c r="S106" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T106" s="10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U106" s="10">
+        <f t="shared" si="3"/>
+        <v>-405</v>
+      </c>
+      <c r="V106" s="15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="107" spans="4:22" ht="21" x14ac:dyDescent="0.25">
+      <c r="U107" s="36">
+        <f>SUM(U99:U106)</f>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <dataConsolidate/>
-  <mergeCells count="9">
+  <mergeCells count="14">
     <mergeCell ref="Y11:Z11"/>
+    <mergeCell ref="E97:H97"/>
+    <mergeCell ref="P97:P98"/>
+    <mergeCell ref="Q97:Q98"/>
+    <mergeCell ref="R97:T97"/>
+    <mergeCell ref="U97:U98"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="J11:K11"/>
@@ -6457,39 +7106,61 @@
     <mergeCell ref="V11:W11"/>
   </mergeCells>
   <conditionalFormatting sqref="E89">
-    <cfRule type="cellIs" dxfId="26" priority="141" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="32" priority="145" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="140" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="146" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="139" operator="lessThan">
+    <cfRule type="cellIs" dxfId="30" priority="147" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H89">
-    <cfRule type="cellIs" dxfId="23" priority="36" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="40" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="41" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="42" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K89">
+    <cfRule type="cellIs" dxfId="26" priority="37" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="38" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="39" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N89">
+    <cfRule type="cellIs" dxfId="23" priority="34" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="22" priority="35" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="34" operator="lessThan">
+    <cfRule type="cellIs" dxfId="21" priority="36" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K89">
-    <cfRule type="cellIs" dxfId="20" priority="33" operator="greaterThan">
+  <conditionalFormatting sqref="Q89">
+    <cfRule type="cellIs" dxfId="20" priority="31" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="19" priority="32" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="31" operator="lessThan">
+    <cfRule type="cellIs" dxfId="18" priority="33" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N89">
+  <conditionalFormatting sqref="T89">
     <cfRule type="cellIs" dxfId="17" priority="28" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -6500,47 +7171,47 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q89">
-    <cfRule type="cellIs" dxfId="14" priority="26" operator="equal">
+  <conditionalFormatting sqref="W89">
+    <cfRule type="cellIs" dxfId="14" priority="25" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="27" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="26" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="25" operator="lessThan">
+    <cfRule type="cellIs" dxfId="12" priority="27" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T89">
-    <cfRule type="cellIs" dxfId="11" priority="24" operator="greaterThan">
+  <conditionalFormatting sqref="Z89">
+    <cfRule type="cellIs" dxfId="11" priority="22" operator="lessThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="10" priority="23" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W89">
-    <cfRule type="cellIs" dxfId="8" priority="21" operator="greaterThan">
+  <conditionalFormatting sqref="Q99:Q106">
+    <cfRule type="cellIs" dxfId="8" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="19" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z89">
-    <cfRule type="cellIs" dxfId="5" priority="18" operator="greaterThan">
+  <conditionalFormatting sqref="U99:U106">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="16" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6550,7 +7221,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25E9A583-41BF-8143-84DF-F8B494A614D1}">
-  <dimension ref="E18:M82"/>
+  <dimension ref="E7:M78"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
@@ -6560,6 +7231,85 @@
     <col min="11" max="11" width="16.1640625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="7" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E8" s="22">
+        <v>5</v>
+      </c>
+      <c r="F8" s="25">
+        <f>(3200/SUM($E$8:$E$15))*E8</f>
+        <v>69.86899563318778</v>
+      </c>
+    </row>
+    <row r="9" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E9" s="23">
+        <v>100</v>
+      </c>
+      <c r="F9" s="25">
+        <f t="shared" ref="F9:F15" si="0">(3200/SUM($E$8:$E$15))*E9</f>
+        <v>1397.3799126637555</v>
+      </c>
+    </row>
+    <row r="10" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E10" s="23">
+        <v>3</v>
+      </c>
+      <c r="F10" s="25">
+        <f t="shared" si="0"/>
+        <v>41.921397379912662</v>
+      </c>
+    </row>
+    <row r="11" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E11" s="23">
+        <v>0</v>
+      </c>
+      <c r="F11" s="25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E12" s="23">
+        <v>22</v>
+      </c>
+      <c r="F12" s="25">
+        <f t="shared" si="0"/>
+        <v>307.42358078602621</v>
+      </c>
+    </row>
+    <row r="13" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E13" s="23">
+        <v>26</v>
+      </c>
+      <c r="F13" s="25">
+        <f t="shared" si="0"/>
+        <v>363.31877729257644</v>
+      </c>
+    </row>
+    <row r="14" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E14" s="23">
+        <v>61</v>
+      </c>
+      <c r="F14" s="25">
+        <f t="shared" si="0"/>
+        <v>852.40174672489081</v>
+      </c>
+    </row>
+    <row r="15" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E15" s="23">
+        <v>12</v>
+      </c>
+      <c r="F15" s="25">
+        <f t="shared" si="0"/>
+        <v>167.68558951965065</v>
+      </c>
+    </row>
+    <row r="16" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="F16" s="24">
+        <f>SUM(F8:F15)</f>
+        <v>3200</v>
+      </c>
+    </row>
     <row r="18" spans="5:10" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="19" spans="5:10" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="20" spans="5:10" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -6568,7 +7318,7 @@
     <row r="23" spans="5:10" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="27" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E27" s="6" t="s">
-        <v>29</v>
+        <v>112</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>17</v>
@@ -6577,10 +7327,10 @@
         <v>18</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="5:10" ht="19" x14ac:dyDescent="0.25">
@@ -6594,10 +7344,10 @@
         <v>5</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="5:10" ht="19" x14ac:dyDescent="0.25">
@@ -6605,10 +7355,10 @@
         <v>5</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>8</v>
+        <v>114</v>
       </c>
     </row>
     <row r="30" spans="5:10" ht="19" x14ac:dyDescent="0.25">
@@ -6616,10 +7366,10 @@
         <v>9</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G30" s="12" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31" spans="5:10" ht="19" x14ac:dyDescent="0.25">
@@ -6627,10 +7377,10 @@
         <v>12</v>
       </c>
       <c r="F31" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="G31" s="12" t="s">
         <v>12</v>
-      </c>
-      <c r="G31" s="12" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="32" spans="5:10" ht="19" x14ac:dyDescent="0.25">
@@ -6638,573 +7388,422 @@
         <v>10</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E33" s="15" t="s">
-        <v>13</v>
+        <v>114</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>19</v>
+        <v>114</v>
       </c>
     </row>
     <row r="34" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E34" s="15" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E35" s="15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F35" s="12" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="36" spans="5:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="E36" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="F36" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G36" s="12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="39" spans="5:10" x14ac:dyDescent="0.2">
-      <c r="E39" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F39" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="38" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="E38" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F38" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G39" s="6" t="s">
+      <c r="G38" s="6" t="s">
         <v>18</v>
       </c>
+      <c r="I38" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J38" s="6"/>
+    </row>
+    <row r="39" spans="5:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="E39" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
       <c r="I39" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="J39" s="6" t="s">
-        <v>9</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="J39" s="6"/>
     </row>
     <row r="40" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E40" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F40" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G40" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I40" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J40" s="6" t="s">
-        <v>5</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
     </row>
     <row r="41" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E41" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="F41" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G41" s="12" t="s">
-        <v>8</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
     </row>
     <row r="42" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E42" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="F42" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="G42" s="12" t="s">
-        <v>9</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F42" s="12"/>
+      <c r="G42" s="12"/>
     </row>
     <row r="43" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E43" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="F43" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="G43" s="12" t="s">
-        <v>5</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F43" s="12"/>
+      <c r="G43" s="12"/>
     </row>
     <row r="44" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E44" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="F44" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="G44" s="12" t="s">
-        <v>9</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="F44" s="12"/>
+      <c r="G44" s="12"/>
+      <c r="I44" s="12"/>
     </row>
     <row r="45" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E45" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="F45" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G45" s="12" t="s">
-        <v>5</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="F45" s="12"/>
+      <c r="G45" s="12"/>
     </row>
     <row r="46" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E46" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F46" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F46" s="12"/>
+      <c r="G46" s="12"/>
+    </row>
+    <row r="47" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="E47" s="13"/>
+      <c r="F47" s="17"/>
+      <c r="G47" s="17"/>
+    </row>
+    <row r="48" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="E48" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I48" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J48" s="6"/>
+    </row>
+    <row r="49" spans="5:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="E49" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="G46" s="12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="47" spans="5:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="E47" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="F47" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="G47" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="48" spans="5:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="E48" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="F48" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="G48" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="49" spans="5:10" x14ac:dyDescent="0.2">
-      <c r="E49" s="13"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="17"/>
-    </row>
-    <row r="50" spans="5:10" x14ac:dyDescent="0.2">
-      <c r="E50" s="6" t="s">
+      <c r="F49" s="12"/>
+      <c r="G49" s="12"/>
+      <c r="I49" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F50" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G50" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="I50" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="J50" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="J49" s="6"/>
+    </row>
+    <row r="50" spans="5:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="E50" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="F50" s="12"/>
+      <c r="G50" s="12"/>
     </row>
     <row r="51" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E51" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F51" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="G51" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="I51" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J51" s="6" t="s">
         <v>9</v>
       </c>
+      <c r="F51" s="12"/>
+      <c r="G51" s="12"/>
     </row>
     <row r="52" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E52" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="F52" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="G52" s="12" t="s">
-        <v>9</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F52" s="12"/>
+      <c r="G52" s="12"/>
     </row>
     <row r="53" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E53" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="F53" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="G53" s="12" t="s">
-        <v>24</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F53" s="12"/>
+      <c r="G53" s="12"/>
     </row>
     <row r="54" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E54" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="F54" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G54" s="12" t="s">
-        <v>9</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="F54" s="12"/>
+      <c r="G54" s="12"/>
     </row>
     <row r="55" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E55" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="F55" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="G55" s="12" t="s">
-        <v>10</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="F55" s="12"/>
+      <c r="G55" s="12"/>
     </row>
     <row r="56" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E56" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="F56" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="G56" s="12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="57" spans="5:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="E57" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F57" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G57" s="12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="58" spans="5:10" ht="19" x14ac:dyDescent="0.25">
-      <c r="E58" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="F58" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G58" s="12" t="s">
-        <v>24</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="F56" s="12"/>
+      <c r="G56" s="12"/>
+    </row>
+    <row r="57" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="E57" s="13"/>
+      <c r="F57" s="17"/>
+      <c r="G57" s="17"/>
+    </row>
+    <row r="58" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="E58" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I58" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J58" s="6"/>
     </row>
     <row r="59" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E59" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="F59" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" s="12"/>
+      <c r="G59" s="12"/>
+      <c r="I59" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J59" s="6"/>
+    </row>
+    <row r="60" spans="5:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="E60" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="F60" s="12"/>
+      <c r="G60" s="12"/>
+    </row>
+    <row r="61" spans="5:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="E61" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G59" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="60" spans="5:10" x14ac:dyDescent="0.2">
-      <c r="E60" s="13"/>
-      <c r="F60" s="17"/>
-      <c r="G60" s="17"/>
-    </row>
-    <row r="61" spans="5:10" x14ac:dyDescent="0.2">
-      <c r="E61" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="F61" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G61" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="I61" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="J61" s="6" t="s">
-        <v>20</v>
-      </c>
+      <c r="F61" s="12"/>
+      <c r="G61" s="12"/>
     </row>
     <row r="62" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E62" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F62" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="G62" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="I62" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J62" s="6" t="s">
-        <v>24</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F62" s="12"/>
+      <c r="G62" s="12"/>
     </row>
     <row r="63" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E63" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="F63" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="G63" s="12" t="s">
-        <v>13</v>
-      </c>
+      <c r="F63" s="12"/>
+      <c r="G63" s="12"/>
     </row>
     <row r="64" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E64" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="F64" s="12"/>
+      <c r="G64" s="12"/>
+    </row>
+    <row r="65" spans="5:13" ht="19" x14ac:dyDescent="0.25">
+      <c r="E65" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F65" s="12"/>
+      <c r="G65" s="12"/>
+    </row>
+    <row r="66" spans="5:13" ht="19" x14ac:dyDescent="0.25">
+      <c r="E66" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="F66" s="12"/>
+      <c r="G66" s="12"/>
+    </row>
+    <row r="68" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="I68" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="J68" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="K68" s="16" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="69" spans="5:13" ht="21" x14ac:dyDescent="0.25">
+      <c r="I69" s="1">
+        <v>1</v>
+      </c>
+      <c r="J69" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="F64" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="G64" s="12" t="s">
+      <c r="K69" s="10">
+        <v>473.92857142857144</v>
+      </c>
+      <c r="L69" s="16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="70" spans="5:13" ht="21" x14ac:dyDescent="0.25">
+      <c r="I70" s="1">
+        <v>2</v>
+      </c>
+      <c r="J70" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="K70" s="10">
+        <v>366.42857142857144</v>
+      </c>
+      <c r="L70" s="16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="71" spans="5:13" ht="21" x14ac:dyDescent="0.25">
+      <c r="I71" s="1">
+        <v>3</v>
+      </c>
+      <c r="J71" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="K71" s="10">
+        <v>112.85714285714283</v>
+      </c>
+      <c r="L71" s="16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="72" spans="5:13" ht="21" x14ac:dyDescent="0.25">
+      <c r="I72" s="1">
+        <v>4</v>
+      </c>
+      <c r="J72" s="15" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="65" spans="5:12" ht="19" x14ac:dyDescent="0.25">
-      <c r="E65" s="15" t="s">
+      <c r="K72" s="10">
+        <v>10</v>
+      </c>
+      <c r="L72" s="16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="73" spans="5:13" ht="21" x14ac:dyDescent="0.25">
+      <c r="I73" s="1">
+        <v>5</v>
+      </c>
+      <c r="J73" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="K73" s="10">
+        <v>-12.142857142857139</v>
+      </c>
+    </row>
+    <row r="74" spans="5:13" ht="21" x14ac:dyDescent="0.25">
+      <c r="I74" s="1">
+        <v>6</v>
+      </c>
+      <c r="J74" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="F65" s="12" t="s">
+      <c r="K74" s="10">
+        <v>-78.928571428571445</v>
+      </c>
+    </row>
+    <row r="75" spans="5:13" ht="21" x14ac:dyDescent="0.25">
+      <c r="I75" s="1">
+        <v>7</v>
+      </c>
+      <c r="J75" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="K75" s="10">
+        <v>-221.78571428571428</v>
+      </c>
+    </row>
+    <row r="76" spans="5:13" ht="21" x14ac:dyDescent="0.25">
+      <c r="I76" s="1">
         <v>8</v>
       </c>
-      <c r="G65" s="12" t="s">
+      <c r="J76" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="K76" s="10">
+        <v>-240</v>
+      </c>
+    </row>
+    <row r="77" spans="5:13" ht="21" x14ac:dyDescent="0.25">
+      <c r="I77" s="1">
         <v>9</v>
       </c>
-    </row>
-    <row r="66" spans="5:12" ht="19" x14ac:dyDescent="0.25">
-      <c r="E66" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="F66" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="G66" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="67" spans="5:12" ht="19" x14ac:dyDescent="0.25">
-      <c r="E67" s="15" t="s">
+      <c r="J77" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="F67" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G67" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="68" spans="5:12" ht="19" x14ac:dyDescent="0.25">
-      <c r="E68" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F68" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G68" s="12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="69" spans="5:12" ht="19" x14ac:dyDescent="0.25">
-      <c r="E69" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="F69" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G69" s="12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="70" spans="5:12" ht="19" x14ac:dyDescent="0.25">
-      <c r="E70" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="F70" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G70" s="12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="72" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="I72" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="J72" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="K72" s="16" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="73" spans="5:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="I73" s="1">
-        <v>1</v>
-      </c>
-      <c r="J73" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="K73" s="10">
-        <v>473.92857142857144</v>
-      </c>
-      <c r="L73" s="16" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="74" spans="5:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="I74" s="1">
-        <v>2</v>
-      </c>
-      <c r="J74" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="K74" s="10">
-        <v>366.42857142857144</v>
-      </c>
-      <c r="L74" s="16" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="75" spans="5:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="I75" s="1">
-        <v>3</v>
-      </c>
-      <c r="J75" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="K75" s="10">
-        <v>112.85714285714283</v>
-      </c>
-      <c r="L75" s="16" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="76" spans="5:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="I76" s="1">
-        <v>4</v>
-      </c>
-      <c r="J76" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K76" s="10">
-        <v>10</v>
-      </c>
-      <c r="L76" s="16" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="77" spans="5:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="I77" s="1">
-        <v>5</v>
-      </c>
-      <c r="J77" s="15" t="s">
-        <v>10</v>
-      </c>
       <c r="K77" s="10">
-        <v>-12.142857142857139</v>
-      </c>
-    </row>
-    <row r="78" spans="5:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="I78" s="1">
-        <v>6</v>
-      </c>
-      <c r="J78" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="K78" s="10">
-        <v>-78.928571428571445</v>
-      </c>
-    </row>
-    <row r="79" spans="5:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="I79" s="1">
-        <v>7</v>
-      </c>
-      <c r="J79" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="K79" s="10">
-        <v>-221.78571428571428</v>
-      </c>
-    </row>
-    <row r="80" spans="5:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="I80" s="1">
-        <v>8</v>
-      </c>
-      <c r="J80" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="K80" s="10">
-        <v>-240</v>
-      </c>
-    </row>
-    <row r="81" spans="9:13" ht="21" x14ac:dyDescent="0.25">
-      <c r="I81" s="1">
-        <v>9</v>
-      </c>
-      <c r="J81" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="K81" s="10">
         <v>-410.35714285714289</v>
       </c>
     </row>
-    <row r="82" spans="9:13" x14ac:dyDescent="0.2">
-      <c r="K82">
-        <f>SUM(K73:K81)</f>
-        <v>0</v>
-      </c>
-      <c r="L82">
-        <f>SUM(K73:K76)</f>
+    <row r="78" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="K78">
+        <f>SUM(K69:K77)</f>
+        <v>0</v>
+      </c>
+      <c r="L78">
+        <f>SUM(K69:K72)</f>
         <v>963.21428571428578</v>
       </c>
-      <c r="M82">
-        <f>L82/9</f>
+      <c r="M78">
+        <f>L78/9</f>
         <v>107.02380952380953</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="I73:K81">
-    <sortCondition descending="1" ref="K73:K81"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="I69:K77">
+    <sortCondition descending="1" ref="K69:K77"/>
   </sortState>
-  <conditionalFormatting sqref="K73:K81">
+  <conditionalFormatting sqref="K69:K77">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Eliminator RR vs RCB
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64819EAA-1326-5B43-BC93-1B8CCFF4DE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F931FC-B1F3-6644-8DB1-B9FC19EF8BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-50420" yWindow="-3180" windowWidth="49000" windowHeight="26800" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="123">
   <si>
     <t>Points</t>
   </si>
@@ -137,9 +137,6 @@
     <t>Vikcy</t>
   </si>
   <si>
-    <t>Eliminator RCB vs KKR</t>
-  </si>
-  <si>
     <t>Rank 1</t>
   </si>
   <si>
@@ -383,6 +380,9 @@
     <t>Qualifier 1 KKR vs SRH</t>
   </si>
   <si>
+    <t>Eliminator RR vs RCB</t>
+  </si>
+  <si>
     <t>Rapaka</t>
   </si>
   <si>
@@ -396,9 +396,6 @@
   </si>
   <si>
     <t>Format 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Final score </t>
   </si>
   <si>
     <t xml:space="preserve">Finals </t>
@@ -545,7 +542,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -670,26 +667,13 @@
     </border>
     <border>
       <left/>
-      <right/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -698,7 +682,7 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -752,31 +736,35 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent6" xfId="1" builtinId="50"/>
@@ -1429,7 +1417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BE9CB7-B9A7-B347-86F0-C3EB9B5BFBBD}">
-  <dimension ref="A1:AA107"/>
+  <dimension ref="A1:AA108"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.83203125" bestFit="1" customWidth="1"/>
@@ -1462,7 +1450,7 @@
         <v>50</v>
       </c>
       <c r="I2" s="21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J2" s="21"/>
       <c r="K2" s="21"/>
@@ -1658,11 +1646,11 @@
       </c>
       <c r="Q11" s="20"/>
       <c r="S11" s="19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="T11" s="20"/>
       <c r="V11" s="19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="W11" s="20"/>
       <c r="Y11" s="19" t="s">
@@ -1711,13 +1699,13 @@
         <v>0</v>
       </c>
       <c r="S12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="T12" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="V12" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="T12" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="V12" s="6" t="s">
-        <v>41</v>
       </c>
       <c r="W12" s="6" t="s">
         <v>0</v>
@@ -1804,7 +1792,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1869,7 +1857,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1934,7 +1922,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2001,7 +1989,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2068,7 +2056,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2135,7 +2123,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D19" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E19, ($Z19,$W19,$T19,$Q19,$N19,$K19,$H19,$E19), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E19, ($Z19,$W19,$T19,$Q19,$N19,$K19,$H19,$E19), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2202,7 +2190,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D20" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E20, ($Z20,$W20,$T20,$Q20,$N20,$K20,$H20,$E20), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E20, ($Z20,$W20,$T20,$Q20,$N20,$K20,$H20,$E20), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2269,7 +2257,7 @@
         <v>1</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2336,7 +2324,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2403,7 +2391,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2470,7 +2458,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D24" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2535,7 +2523,7 @@
         <v>1</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2602,7 +2590,7 @@
         <v>1</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D26" s="3">
         <v>-22.5</v>
@@ -2667,7 +2655,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2734,7 +2722,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2799,7 +2787,7 @@
         <v>1</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2866,7 +2854,7 @@
         <v>1</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2933,7 +2921,7 @@
         <v>1</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2998,7 +2986,7 @@
         <v>1</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D32" s="3">
         <v>-22.5</v>
@@ -3063,7 +3051,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3130,7 +3118,7 @@
         <v>1</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3197,7 +3185,7 @@
         <v>1</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3264,7 +3252,7 @@
         <v>1</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D36" s="3">
         <v>-22.5</v>
@@ -3327,7 +3315,7 @@
         <v>1</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3394,7 +3382,7 @@
         <v>1</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3461,7 +3449,7 @@
         <v>1</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D39" s="3">
         <v>35</v>
@@ -3526,7 +3514,7 @@
         <v>1</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3593,7 +3581,7 @@
         <v>1</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3660,7 +3648,7 @@
         <v>1</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3727,7 +3715,7 @@
         <v>1</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D43" s="3">
         <v>-7.5</v>
@@ -3792,7 +3780,7 @@
         <v>1</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3859,7 +3847,7 @@
         <v>1</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3926,7 +3914,7 @@
         <v>1</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3993,7 +3981,7 @@
         <v>1</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4060,7 +4048,7 @@
         <v>1</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4127,7 +4115,7 @@
         <v>1</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4194,7 +4182,7 @@
         <v>1</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4261,7 +4249,7 @@
         <v>1</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4328,7 +4316,7 @@
         <v>1</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D52" s="3">
         <v>-22.5</v>
@@ -4393,7 +4381,7 @@
         <v>1</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4460,7 +4448,7 @@
         <v>1</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D54" s="3">
         <v>0</v>
@@ -4523,7 +4511,7 @@
         <v>1</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4590,7 +4578,7 @@
         <v>1</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D56" s="3">
         <v>12.5</v>
@@ -4655,7 +4643,7 @@
         <v>1</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4722,7 +4710,7 @@
         <v>1</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4789,7 +4777,7 @@
         <v>1</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4856,7 +4844,7 @@
         <v>1</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D60" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4921,7 +4909,7 @@
         <v>1</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4988,7 +4976,7 @@
         <v>1</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5055,7 +5043,7 @@
         <v>1</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5122,7 +5110,7 @@
         <v>1</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5189,7 +5177,7 @@
         <v>1</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5256,7 +5244,7 @@
         <v>1</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5323,7 +5311,7 @@
         <v>1</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5390,7 +5378,7 @@
         <v>1</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5457,7 +5445,7 @@
         <v>1</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5524,7 +5512,7 @@
         <v>1</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D70" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5589,7 +5577,7 @@
         <v>1</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5656,7 +5644,7 @@
         <v>1</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5723,7 +5711,7 @@
         <v>1</v>
       </c>
       <c r="C73" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5790,7 +5778,7 @@
         <v>1</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D74" s="3">
         <v>-7.5</v>
@@ -5855,7 +5843,7 @@
         <v>1</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D75" s="3">
         <v>0</v>
@@ -5914,7 +5902,7 @@
         <v>1</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D76" s="3">
         <v>-20</v>
@@ -5978,7 +5966,7 @@
         <v>1</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D77" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -6043,7 +6031,7 @@
         <v>1</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D78" s="3">
         <v>0</v>
@@ -6102,7 +6090,7 @@
         <v>1</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D79" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -6169,7 +6157,7 @@
         <v>1</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D80" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -6236,7 +6224,7 @@
         <v>1</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D81" s="3">
         <v>-22.5</v>
@@ -6301,7 +6289,7 @@
         <v>1</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D82" s="3">
         <v>0</v>
@@ -6360,7 +6348,7 @@
         <v>1</v>
       </c>
       <c r="C83" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D83" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -6427,48 +6415,64 @@
         <v>1</v>
       </c>
       <c r="C84" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(E84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>20</v>
+      </c>
+      <c r="E84" s="1">
+        <v>70</v>
+      </c>
+      <c r="G84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(H84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-20</v>
+      </c>
+      <c r="H84" s="1">
+        <v>20</v>
+      </c>
+      <c r="J84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(K84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>50</v>
+      </c>
+      <c r="K84" s="1">
+        <v>100</v>
+      </c>
+      <c r="M84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(N84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>-15</v>
+      </c>
+      <c r="N84" s="1">
+        <v>30</v>
+      </c>
+      <c r="P84" s="3">
+        <f>IF(ISERROR(VLOOKUP(RANK(Q84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
+        <v>5</v>
+      </c>
+      <c r="Q84" s="1">
         <v>60</v>
       </c>
-      <c r="D84" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(E84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E84" s="1"/>
-      <c r="G84" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(H84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H84" s="1"/>
-      <c r="J84" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(K84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K84" s="1"/>
-      <c r="M84" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(N84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N84" s="1"/>
-      <c r="P84" s="3" t="str">
-        <f>IF(ISERROR(VLOOKUP(RANK(Q84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q84" s="1"/>
-      <c r="S84" s="3" t="str">
+      <c r="S84" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T84" s="1"/>
-      <c r="V84" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="T84" s="1">
+        <v>50</v>
+      </c>
+      <c r="V84" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W84" s="1"/>
-      <c r="Y84" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="W84" s="1">
+        <v>40</v>
+      </c>
+      <c r="Y84" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z84" s="1"/>
+        <v>-25</v>
+      </c>
+      <c r="Z84" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="85" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A85" s="5" t="s">
@@ -6655,457 +6659,629 @@
       </c>
       <c r="E89" s="10">
         <f>SUM(D13:D86)</f>
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-355</v>
+        <v>-305</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>332.5</v>
+        <v>317.5</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-135</v>
+        <v>-130</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>37.5</v>
+        <v>32.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-5</v>
+        <v>-30</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="4:22" ht="19" x14ac:dyDescent="0.25">
-      <c r="E97" s="26" t="s">
+    <row r="95" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="N95" s="35"/>
+      <c r="O95" s="35"/>
+      <c r="P95" s="35"/>
+      <c r="Q95" s="35"/>
+      <c r="R95" s="35"/>
+      <c r="S95" s="35"/>
+      <c r="T95" s="35"/>
+      <c r="U95" s="35"/>
+      <c r="V95" s="35"/>
+      <c r="W95" s="35"/>
+      <c r="X95" s="35"/>
+      <c r="Y95" s="35"/>
+    </row>
+    <row r="96" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="N96" s="35"/>
+      <c r="O96" s="35"/>
+      <c r="P96" s="35"/>
+      <c r="Q96" s="35"/>
+      <c r="R96" s="35"/>
+      <c r="S96" s="35"/>
+      <c r="T96" s="35"/>
+      <c r="U96" s="35"/>
+      <c r="V96" s="35"/>
+      <c r="W96" s="35"/>
+      <c r="X96" s="35"/>
+      <c r="Y96" s="35"/>
+    </row>
+    <row r="97" spans="2:25" ht="19" x14ac:dyDescent="0.25">
+      <c r="C97" s="26" t="s">
         <v>114</v>
       </c>
+      <c r="D97" s="26"/>
+      <c r="E97" s="26"/>
       <c r="F97" s="26"/>
       <c r="G97" s="26"/>
       <c r="H97" s="26"/>
-      <c r="I97" s="27"/>
-      <c r="P97" s="28" t="s">
+      <c r="I97" s="26"/>
+      <c r="J97" s="26"/>
+      <c r="N97" s="35"/>
+      <c r="O97" s="36"/>
+      <c r="P97" s="36"/>
+      <c r="Q97" s="35"/>
+      <c r="R97" s="28" t="s">
         <v>115</v>
       </c>
-      <c r="Q97" s="29" t="s">
+      <c r="S97" s="28"/>
+      <c r="T97" s="28"/>
+      <c r="U97" s="28"/>
+      <c r="V97" s="28"/>
+      <c r="W97" s="36"/>
+      <c r="X97" s="35"/>
+      <c r="Y97" s="35"/>
+    </row>
+    <row r="98" spans="2:25" ht="19" x14ac:dyDescent="0.25">
+      <c r="C98" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="D98" s="26"/>
+      <c r="E98" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="F98" s="26"/>
+      <c r="G98" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H98" s="26"/>
+      <c r="I98" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="J98" s="26"/>
+      <c r="N98" s="35"/>
+      <c r="O98" s="36"/>
+      <c r="P98" s="36"/>
+      <c r="Q98" s="35"/>
+      <c r="R98" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="R97" s="30" t="s">
+      <c r="S98" s="28" t="s">
         <v>117</v>
       </c>
-      <c r="S97" s="31"/>
-      <c r="T97" s="32"/>
-      <c r="U97" s="29" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="98" spans="4:22" ht="19" x14ac:dyDescent="0.25">
-      <c r="E98" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="F98" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="G98" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="H98" s="15" t="s">
+      <c r="T98" s="28"/>
+      <c r="U98" s="28"/>
+      <c r="V98" s="28"/>
+      <c r="W98" s="36"/>
+      <c r="X98" s="35"/>
+      <c r="Y98" s="35"/>
+    </row>
+    <row r="99" spans="2:25" ht="19" x14ac:dyDescent="0.25">
+      <c r="C99" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="D99" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="E99" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="F99" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="G99" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="H99" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="I99" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="J99" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="K99" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="I98" s="33" t="s">
+      <c r="N99" s="35"/>
+      <c r="O99" s="35"/>
+      <c r="P99" s="35"/>
+      <c r="Q99" s="35"/>
+      <c r="R99" s="27"/>
+      <c r="S99" s="37" t="s">
         <v>120</v>
       </c>
-      <c r="P98" s="34"/>
-      <c r="Q98" s="29"/>
-      <c r="R98" s="15" t="s">
+      <c r="T99" s="37" t="s">
         <v>121</v>
       </c>
-      <c r="S98" s="15" t="s">
+      <c r="U99" s="37" t="s">
         <v>122</v>
       </c>
-      <c r="T98" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="U98" s="29"/>
-    </row>
-    <row r="99" spans="4:22" ht="21" x14ac:dyDescent="0.25">
-      <c r="D99" s="15" t="s">
+      <c r="V99" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="W99" s="36"/>
+      <c r="X99" s="35"/>
+      <c r="Y99" s="35"/>
+    </row>
+    <row r="100" spans="2:25" ht="21" x14ac:dyDescent="0.25">
+      <c r="B100" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="E99" s="1">
-        <v>4</v>
-      </c>
-      <c r="F99" s="1"/>
-      <c r="G99" s="1"/>
-      <c r="H99" s="1"/>
-      <c r="I99" s="15">
-        <f>SUM(E99:H99)</f>
-        <v>4</v>
-      </c>
-      <c r="P99" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q99" s="10">
-        <f>E89</f>
-        <v>10</v>
-      </c>
-      <c r="R99" s="35">
-        <v>-400</v>
-      </c>
-      <c r="S99" s="10">
-        <f>I99</f>
-        <v>4</v>
-      </c>
-      <c r="T99" s="10">
-        <f>IFERROR((-SUM($R$99:$R$106)/SUM($S$99:$S$106))*$S99, 0)</f>
-        <v>2133.3333333333335</v>
-      </c>
-      <c r="U99" s="37">
-        <f>SUM(Q99,R99,T99)</f>
-        <v>1743.3333333333335</v>
-      </c>
-      <c r="V99" s="15" t="str">
-        <f>P99</f>
-        <v>Jaya</v>
-      </c>
-    </row>
-    <row r="100" spans="4:22" ht="21" x14ac:dyDescent="0.25">
-      <c r="D100" s="15" t="s">
-        <v>5</v>
+      <c r="C100" s="1">
+        <v>1</v>
+      </c>
+      <c r="D100" s="1">
+        <v>3</v>
       </c>
       <c r="E100" s="1">
-        <v>0</v>
-      </c>
-      <c r="F100" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="F100" s="1">
+        <v>3</v>
+      </c>
       <c r="G100" s="1"/>
       <c r="H100" s="1"/>
-      <c r="I100" s="15">
-        <f t="shared" ref="I100:I106" si="0">SUM(E100:H100)</f>
-        <v>0</v>
-      </c>
-      <c r="P100" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q100" s="10">
-        <f>H89</f>
-        <v>80</v>
-      </c>
-      <c r="R100" s="35">
+      <c r="I100" s="1"/>
+      <c r="J100" s="1"/>
+      <c r="K100" s="15">
+        <f>SUM(C100:J100)</f>
+        <v>8</v>
+      </c>
+      <c r="Q100" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="R100" s="10">
+        <f>E89</f>
+        <v>30</v>
+      </c>
+      <c r="S100" s="29">
         <v>-400</v>
       </c>
-      <c r="S100" s="10">
-        <f t="shared" ref="S100:S106" si="1">I100</f>
-        <v>0</v>
-      </c>
       <c r="T100" s="10">
-        <f t="shared" ref="T100:T106" si="2">IFERROR((-SUM($R$99:$R$106)/SUM($S$99:$S$106))*$S100, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="U100" s="37">
-        <f t="shared" ref="U100:U106" si="3">SUM(Q100,R100,T100)</f>
-        <v>-320</v>
-      </c>
-      <c r="V100" s="15" t="str">
-        <f t="shared" ref="V100:V106" si="4">P100</f>
-        <v>Justin</v>
-      </c>
-    </row>
-    <row r="101" spans="4:22" ht="21" x14ac:dyDescent="0.25">
-      <c r="D101" s="15" t="s">
-        <v>9</v>
+        <f>K100</f>
+        <v>8</v>
+      </c>
+      <c r="U100" s="10">
+        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T100, 0)</f>
+        <v>984.61538461538464</v>
+      </c>
+      <c r="V100" s="31">
+        <f>SUM(R100,S100,U100)</f>
+        <v>614.61538461538464</v>
+      </c>
+      <c r="W100" s="15" t="str">
+        <f>Q100</f>
+        <v>Jaya</v>
+      </c>
+    </row>
+    <row r="101" spans="2:25" ht="21" x14ac:dyDescent="0.25">
+      <c r="B101" s="32" t="s">
+        <v>5</v>
+      </c>
+      <c r="C101" s="1">
+        <v>0</v>
+      </c>
+      <c r="D101" s="1">
+        <v>0</v>
       </c>
       <c r="E101" s="1">
         <v>0</v>
       </c>
-      <c r="F101" s="1"/>
+      <c r="F101" s="1">
+        <v>0</v>
+      </c>
       <c r="G101" s="1"/>
       <c r="H101" s="1"/>
-      <c r="I101" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="P101" s="15" t="s">
+      <c r="I101" s="1"/>
+      <c r="J101" s="1"/>
+      <c r="K101" s="15">
+        <f t="shared" ref="K101:K107" si="0">SUM(C101:J101)</f>
+        <v>0</v>
+      </c>
+      <c r="Q101" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="R101" s="10">
+        <f>H89</f>
+        <v>60</v>
+      </c>
+      <c r="S101" s="29">
+        <v>-400</v>
+      </c>
+      <c r="T101" s="10">
+        <f>K101</f>
+        <v>0</v>
+      </c>
+      <c r="U101" s="10">
+        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T101, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="V101" s="31">
+        <f t="shared" ref="V101:V107" si="1">SUM(R101,S101,U101)</f>
+        <v>-340</v>
+      </c>
+      <c r="W101" s="15" t="str">
+        <f t="shared" ref="W101:W107" si="2">Q101</f>
+        <v>Justin</v>
+      </c>
+    </row>
+    <row r="102" spans="2:25" ht="21" x14ac:dyDescent="0.25">
+      <c r="B102" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="Q101" s="10">
-        <f>K89</f>
-        <v>-355</v>
-      </c>
-      <c r="R101" s="35">
-        <v>-400</v>
-      </c>
-      <c r="S101" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T101" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U101" s="37">
-        <f t="shared" si="3"/>
-        <v>-755</v>
-      </c>
-      <c r="V101" s="15" t="str">
-        <f t="shared" si="4"/>
-        <v>Ram</v>
-      </c>
-    </row>
-    <row r="102" spans="4:22" ht="21" x14ac:dyDescent="0.25">
-      <c r="D102" s="15" t="s">
-        <v>12</v>
+      <c r="C102" s="1">
+        <v>0</v>
+      </c>
+      <c r="D102" s="1">
+        <v>0</v>
       </c>
       <c r="E102" s="1">
-        <v>0</v>
-      </c>
-      <c r="F102" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="F102" s="1">
+        <v>11</v>
+      </c>
       <c r="G102" s="1"/>
       <c r="H102" s="1"/>
-      <c r="I102" s="15">
+      <c r="I102" s="1"/>
+      <c r="J102" s="1"/>
+      <c r="K102" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="P102" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q102" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="R102" s="10">
+        <f>K89</f>
+        <v>-305</v>
+      </c>
+      <c r="S102" s="29">
+        <v>-400</v>
+      </c>
+      <c r="T102" s="10">
+        <f>K102</f>
+        <v>13</v>
+      </c>
+      <c r="U102" s="10">
+        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T102, 0)</f>
+        <v>1600</v>
+      </c>
+      <c r="V102" s="31">
+        <f t="shared" si="1"/>
+        <v>895</v>
+      </c>
+      <c r="W102" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>Ram</v>
+      </c>
+    </row>
+    <row r="103" spans="2:25" ht="21" x14ac:dyDescent="0.25">
+      <c r="B103" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="Q102" s="10">
-        <f>N89</f>
-        <v>332.5</v>
-      </c>
-      <c r="R102" s="35">
-        <v>-400</v>
-      </c>
-      <c r="S102" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T102" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U102" s="37">
-        <f t="shared" si="3"/>
-        <v>-67.5</v>
-      </c>
-      <c r="V102" s="15" t="str">
-        <f t="shared" si="4"/>
-        <v>Sibi</v>
-      </c>
-    </row>
-    <row r="103" spans="4:22" ht="21" x14ac:dyDescent="0.25">
-      <c r="D103" s="15" t="s">
-        <v>10</v>
+      <c r="C103" s="1">
+        <v>0</v>
+      </c>
+      <c r="D103" s="1">
+        <v>0</v>
       </c>
       <c r="E103" s="1">
-        <v>2</v>
-      </c>
-      <c r="F103" s="1"/>
+        <v>0</v>
+      </c>
+      <c r="F103" s="1">
+        <v>3</v>
+      </c>
       <c r="G103" s="1"/>
       <c r="H103" s="1"/>
-      <c r="I103" s="15">
+      <c r="I103" s="1"/>
+      <c r="J103" s="1"/>
+      <c r="K103" s="15">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="Q103" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="R103" s="10">
+        <f>N89</f>
+        <v>317.5</v>
+      </c>
+      <c r="S103" s="29">
+        <v>-400</v>
+      </c>
+      <c r="T103" s="10">
+        <f>K103</f>
+        <v>3</v>
+      </c>
+      <c r="U103" s="10">
+        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T103, 0)</f>
+        <v>369.23076923076923</v>
+      </c>
+      <c r="V103" s="31">
+        <f t="shared" si="1"/>
+        <v>286.73076923076923</v>
+      </c>
+      <c r="W103" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>Sibi</v>
+      </c>
+    </row>
+    <row r="104" spans="2:25" ht="21" x14ac:dyDescent="0.25">
+      <c r="B104" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="C104" s="1">
+        <v>2</v>
+      </c>
+      <c r="D104" s="1">
+        <v>0</v>
+      </c>
+      <c r="E104" s="1">
+        <v>0</v>
+      </c>
+      <c r="F104" s="1">
+        <v>0</v>
+      </c>
+      <c r="G104" s="1"/>
+      <c r="H104" s="1"/>
+      <c r="I104" s="1"/>
+      <c r="J104" s="1"/>
+      <c r="K104" s="15">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="P103" s="15" t="s">
+      <c r="Q104" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="Q103" s="10">
+      <c r="R104" s="10">
         <f>Q89</f>
-        <v>-135</v>
-      </c>
-      <c r="R103" s="35">
+        <v>-130</v>
+      </c>
+      <c r="S104" s="29">
         <v>-400</v>
       </c>
-      <c r="S103" s="10">
+      <c r="T104" s="10">
+        <f>K104</f>
+        <v>2</v>
+      </c>
+      <c r="U104" s="10">
+        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T104, 0)</f>
+        <v>246.15384615384616</v>
+      </c>
+      <c r="V104" s="31">
         <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="T103" s="10">
+        <v>-283.84615384615381</v>
+      </c>
+      <c r="W104" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>1066.6666666666667</v>
-      </c>
-      <c r="U103" s="37">
-        <f t="shared" si="3"/>
-        <v>531.66666666666674</v>
-      </c>
-      <c r="V103" s="15" t="str">
-        <f t="shared" si="4"/>
         <v>Sundar</v>
       </c>
     </row>
-    <row r="104" spans="4:22" ht="21" x14ac:dyDescent="0.25">
-      <c r="D104" s="15" t="s">
+    <row r="105" spans="2:25" ht="21" x14ac:dyDescent="0.25">
+      <c r="B105" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="E104" s="1">
-        <v>0</v>
-      </c>
-      <c r="F104" s="1"/>
-      <c r="G104" s="1"/>
-      <c r="H104" s="1"/>
-      <c r="I104" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="P104" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q104" s="10">
-        <f>T89</f>
-        <v>37.5</v>
-      </c>
-      <c r="R104" s="35">
-        <v>-400</v>
-      </c>
-      <c r="S104" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T104" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U104" s="37">
-        <f t="shared" si="3"/>
-        <v>-362.5</v>
-      </c>
-      <c r="V104" s="15" t="str">
-        <f t="shared" si="4"/>
-        <v>Rapaka</v>
-      </c>
-    </row>
-    <row r="105" spans="4:22" ht="21" x14ac:dyDescent="0.25">
-      <c r="D105" s="15" t="s">
-        <v>41</v>
+      <c r="C105" s="1">
+        <v>0</v>
+      </c>
+      <c r="D105" s="1">
+        <v>0</v>
       </c>
       <c r="E105" s="1">
         <v>0</v>
       </c>
-      <c r="F105" s="1"/>
+      <c r="F105" s="1">
+        <v>0</v>
+      </c>
       <c r="G105" s="1"/>
       <c r="H105" s="1"/>
-      <c r="I105" s="15">
+      <c r="I105" s="1"/>
+      <c r="J105" s="1"/>
+      <c r="K105" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="P105" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q105" s="10">
-        <f>W89</f>
-        <v>35</v>
-      </c>
-      <c r="R105" s="35">
+      <c r="Q105" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="R105" s="10">
+        <f>T89</f>
+        <v>32.5</v>
+      </c>
+      <c r="S105" s="29">
         <v>-400</v>
       </c>
-      <c r="S105" s="10">
+      <c r="T105" s="10">
+        <f>K105</f>
+        <v>0</v>
+      </c>
+      <c r="U105" s="10">
+        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T105, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="V105" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T105" s="10">
+        <v>-367.5</v>
+      </c>
+      <c r="W105" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U105" s="37">
-        <f t="shared" si="3"/>
-        <v>-365</v>
-      </c>
-      <c r="V105" s="15" t="str">
-        <f t="shared" si="4"/>
-        <v>Jayanth</v>
-      </c>
-    </row>
-    <row r="106" spans="4:22" ht="21" x14ac:dyDescent="0.25">
-      <c r="D106" s="15" t="s">
-        <v>30</v>
+        <v>Rapaka</v>
+      </c>
+    </row>
+    <row r="106" spans="2:25" ht="21" x14ac:dyDescent="0.25">
+      <c r="B106" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="C106" s="1">
+        <v>0</v>
+      </c>
+      <c r="D106" s="1">
+        <v>0</v>
       </c>
       <c r="E106" s="1">
         <v>0</v>
       </c>
-      <c r="F106" s="1"/>
+      <c r="F106" s="1">
+        <v>0</v>
+      </c>
       <c r="G106" s="1"/>
       <c r="H106" s="1"/>
-      <c r="I106" s="15">
+      <c r="I106" s="1"/>
+      <c r="J106" s="1"/>
+      <c r="K106" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="P106" s="15" t="s">
+      <c r="Q106" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="R106" s="10">
+        <f>W89</f>
+        <v>25</v>
+      </c>
+      <c r="S106" s="29">
+        <v>-400</v>
+      </c>
+      <c r="T106" s="10">
+        <f>K106</f>
+        <v>0</v>
+      </c>
+      <c r="U106" s="10">
+        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T106, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="V106" s="31">
+        <f t="shared" si="1"/>
+        <v>-375</v>
+      </c>
+      <c r="W106" s="15" t="str">
+        <f t="shared" si="2"/>
+        <v>Jayanth</v>
+      </c>
+    </row>
+    <row r="107" spans="2:25" ht="21" x14ac:dyDescent="0.25">
+      <c r="B107" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="Q106" s="10">
+      <c r="C107" s="1">
+        <v>0</v>
+      </c>
+      <c r="D107" s="1">
+        <v>0</v>
+      </c>
+      <c r="E107" s="1">
+        <v>0</v>
+      </c>
+      <c r="F107" s="1">
+        <v>0</v>
+      </c>
+      <c r="G107" s="1"/>
+      <c r="H107" s="1"/>
+      <c r="I107" s="1"/>
+      <c r="J107" s="1"/>
+      <c r="K107" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Q107" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="R107" s="10">
         <f>Z89</f>
-        <v>-5</v>
-      </c>
-      <c r="R106" s="35">
+        <v>-30</v>
+      </c>
+      <c r="S107" s="29">
         <v>-400</v>
       </c>
-      <c r="S106" s="10">
+      <c r="T107" s="10">
+        <f>K107</f>
+        <v>0</v>
+      </c>
+      <c r="U107" s="10">
+        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T107, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="V107" s="31">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T106" s="10">
+        <v>-430</v>
+      </c>
+      <c r="W107" s="15" t="str">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U106" s="37">
-        <f t="shared" si="3"/>
-        <v>-405</v>
-      </c>
-      <c r="V106" s="15" t="str">
-        <f t="shared" si="4"/>
         <v>Vikcy</v>
       </c>
     </row>
-    <row r="107" spans="4:22" ht="21" x14ac:dyDescent="0.25">
-      <c r="U107" s="36">
-        <f>SUM(U99:U106)</f>
+    <row r="108" spans="2:25" ht="21" x14ac:dyDescent="0.25">
+      <c r="R108" s="30">
+        <f>SUM(R100:R107)</f>
+        <v>0</v>
+      </c>
+      <c r="V108" s="39">
+        <f>SUM(V100:V107)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <dataConsolidate/>
-  <mergeCells count="14">
+  <mergeCells count="17">
+    <mergeCell ref="R98:R99"/>
+    <mergeCell ref="S98:V98"/>
+    <mergeCell ref="R97:V97"/>
+    <mergeCell ref="C98:D98"/>
+    <mergeCell ref="E98:F98"/>
+    <mergeCell ref="G98:H98"/>
+    <mergeCell ref="I98:J98"/>
+    <mergeCell ref="C97:J97"/>
     <mergeCell ref="Y11:Z11"/>
-    <mergeCell ref="E97:H97"/>
-    <mergeCell ref="P97:P98"/>
-    <mergeCell ref="Q97:Q98"/>
-    <mergeCell ref="R97:T97"/>
-    <mergeCell ref="U97:U98"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="J11:K11"/>
@@ -7203,7 +7379,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q99:Q106">
+  <conditionalFormatting sqref="R100:R107">
     <cfRule type="cellIs" dxfId="8" priority="4" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -7214,7 +7390,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U99:U106">
+  <conditionalFormatting sqref="V100:V107">
     <cfRule type="cellIs" dxfId="5" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -7328,7 +7504,7 @@
     <row r="23" spans="5:10" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="27" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E27" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>17</v>
@@ -7337,7 +7513,7 @@
         <v>18</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>10</v>
@@ -7354,7 +7530,7 @@
         <v>5</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J28" s="6" t="s">
         <v>8</v>
@@ -7387,7 +7563,7 @@
         <v>12</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G31" s="12" t="s">
         <v>12</v>
@@ -7417,7 +7593,7 @@
     </row>
     <row r="34" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E34" s="15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F34" s="12" t="s">
         <v>12</v>
@@ -7434,12 +7610,12 @@
         <v>20</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E38" s="6" t="s">
-        <v>31</v>
+        <v>112</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>17</v>
@@ -7448,70 +7624,106 @@
         <v>18</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J38" s="6"/>
+        <v>31</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="39" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E39" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="F39" s="12"/>
-      <c r="G39" s="12"/>
+      <c r="F39" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G39" s="12" t="s">
+        <v>10</v>
+      </c>
       <c r="I39" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="J39" s="6"/>
+        <v>32</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="40" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E40" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
+      <c r="F40" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="G40" s="12" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="41" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E41" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="F41" s="12"/>
-      <c r="G41" s="12"/>
+      <c r="F41" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G41" s="12" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="42" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E42" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="F42" s="12"/>
-      <c r="G42" s="12"/>
+      <c r="F42" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="43" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E43" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="F43" s="12"/>
-      <c r="G43" s="12"/>
+      <c r="F43" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G43" s="12" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="44" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E44" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="F44" s="12"/>
-      <c r="G44" s="12"/>
+      <c r="F44" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G44" s="12" t="s">
+        <v>40</v>
+      </c>
       <c r="I44" s="12"/>
     </row>
     <row r="45" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E45" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F45" s="12"/>
-      <c r="G45" s="12"/>
+        <v>40</v>
+      </c>
+      <c r="F45" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G45" s="12" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="46" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E46" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="F46" s="12"/>
-      <c r="G46" s="12"/>
+      <c r="F46" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="G46" s="12" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="47" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E47" s="13"/>
@@ -7520,7 +7732,7 @@
     </row>
     <row r="48" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E48" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>17</v>
@@ -7529,7 +7741,7 @@
         <v>18</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J48" s="6"/>
     </row>
@@ -7540,7 +7752,7 @@
       <c r="F49" s="12"/>
       <c r="G49" s="12"/>
       <c r="I49" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J49" s="6"/>
     </row>
@@ -7581,7 +7793,7 @@
     </row>
     <row r="55" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E55" s="15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F55" s="12"/>
       <c r="G55" s="12"/>
@@ -7600,7 +7812,7 @@
     </row>
     <row r="58" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E58" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>17</v>
@@ -7609,7 +7821,7 @@
         <v>18</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J58" s="6"/>
     </row>
@@ -7620,7 +7832,7 @@
       <c r="F59" s="12"/>
       <c r="G59" s="12"/>
       <c r="I59" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J59" s="6"/>
     </row>
@@ -7661,7 +7873,7 @@
     </row>
     <row r="65" spans="5:13" ht="19" x14ac:dyDescent="0.25">
       <c r="E65" s="15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F65" s="12"/>
       <c r="G65" s="12"/>
@@ -7678,7 +7890,7 @@
         <v>11</v>
       </c>
       <c r="J68" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K68" s="16" t="s">
         <v>7</v>
@@ -7695,7 +7907,7 @@
         <v>473.92857142857144</v>
       </c>
       <c r="L69" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="70" spans="5:13" ht="21" x14ac:dyDescent="0.25">
@@ -7709,7 +7921,7 @@
         <v>366.42857142857144</v>
       </c>
       <c r="L70" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="71" spans="5:13" ht="21" x14ac:dyDescent="0.25">
@@ -7723,7 +7935,7 @@
         <v>112.85714285714283</v>
       </c>
       <c r="L71" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="72" spans="5:13" ht="21" x14ac:dyDescent="0.25">
@@ -7737,7 +7949,7 @@
         <v>10</v>
       </c>
       <c r="L72" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="73" spans="5:13" ht="21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Finals KKR vs SRH
</commit_message>
<xml_diff>
--- a/2024/Next Gen dream 11 2024.xlsx
+++ b/2024/Next Gen dream 11 2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkpaul/Personal/Things/IPL/2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F931FC-B1F3-6644-8DB1-B9FC19EF8BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44682738-F883-6548-AC6E-CFD9C618EFE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-50420" yWindow="-3180" windowWidth="49000" windowHeight="26800" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20080" xr2:uid="{7813E1F3-AD71-F349-B41B-B75E130580BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="124">
   <si>
     <t>Points</t>
   </si>
@@ -143,12 +143,6 @@
     <t>Rank 2</t>
   </si>
   <si>
-    <t>Qualifier 2 DC vs KKR</t>
-  </si>
-  <si>
-    <t>Finals vs KKR</t>
-  </si>
-  <si>
     <t>Player</t>
   </si>
   <si>
@@ -411,6 +405,15 @@
   </si>
   <si>
     <t>Incoming</t>
+  </si>
+  <si>
+    <t>Qualifier 2 SRH vs RR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ram </t>
+  </si>
+  <si>
+    <t>Finals KKR vs SRH</t>
   </si>
 </sst>
 </file>
@@ -682,7 +685,7 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -709,18 +712,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -732,15 +723,6 @@
     </xf>
     <xf numFmtId="2" fontId="7" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -754,17 +736,34 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent6" xfId="1" builtinId="50"/>
@@ -789,6 +788,196 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -909,196 +1098,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1449,24 +1448,24 @@
       <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="I2" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
-      <c r="S2" s="21"/>
-      <c r="T2" s="21"/>
-      <c r="U2" s="21"/>
-      <c r="V2" s="21"/>
-      <c r="W2" s="21"/>
-      <c r="X2" s="21"/>
+      <c r="I2" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="37"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="37"/>
+      <c r="Q2" s="37"/>
+      <c r="R2" s="37"/>
+      <c r="S2" s="37"/>
+      <c r="T2" s="37"/>
+      <c r="U2" s="37"/>
+      <c r="V2" s="37"/>
+      <c r="W2" s="37"/>
+      <c r="X2" s="37"/>
     </row>
     <row r="3" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1475,22 +1474,22 @@
       <c r="B3" s="1">
         <v>20</v>
       </c>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="21"/>
-      <c r="P3" s="21"/>
-      <c r="Q3" s="21"/>
-      <c r="R3" s="21"/>
-      <c r="S3" s="21"/>
-      <c r="T3" s="21"/>
-      <c r="U3" s="21"/>
-      <c r="V3" s="21"/>
-      <c r="W3" s="21"/>
-      <c r="X3" s="21"/>
+      <c r="I3" s="37"/>
+      <c r="J3" s="37"/>
+      <c r="K3" s="37"/>
+      <c r="L3" s="37"/>
+      <c r="M3" s="37"/>
+      <c r="N3" s="37"/>
+      <c r="O3" s="37"/>
+      <c r="P3" s="37"/>
+      <c r="Q3" s="37"/>
+      <c r="R3" s="37"/>
+      <c r="S3" s="37"/>
+      <c r="T3" s="37"/>
+      <c r="U3" s="37"/>
+      <c r="V3" s="37"/>
+      <c r="W3" s="37"/>
+      <c r="X3" s="37"/>
     </row>
     <row r="4" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1499,22 +1498,22 @@
       <c r="B4" s="1">
         <v>5</v>
       </c>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="21"/>
-      <c r="O4" s="21"/>
-      <c r="P4" s="21"/>
-      <c r="Q4" s="21"/>
-      <c r="R4" s="21"/>
-      <c r="S4" s="21"/>
-      <c r="T4" s="21"/>
-      <c r="U4" s="21"/>
-      <c r="V4" s="21"/>
-      <c r="W4" s="21"/>
-      <c r="X4" s="21"/>
+      <c r="I4" s="37"/>
+      <c r="J4" s="37"/>
+      <c r="K4" s="37"/>
+      <c r="L4" s="37"/>
+      <c r="M4" s="37"/>
+      <c r="N4" s="37"/>
+      <c r="O4" s="37"/>
+      <c r="P4" s="37"/>
+      <c r="Q4" s="37"/>
+      <c r="R4" s="37"/>
+      <c r="S4" s="37"/>
+      <c r="T4" s="37"/>
+      <c r="U4" s="37"/>
+      <c r="V4" s="37"/>
+      <c r="W4" s="37"/>
+      <c r="X4" s="37"/>
     </row>
     <row r="5" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1523,22 +1522,22 @@
       <c r="B5" s="1">
         <v>-5</v>
       </c>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="21"/>
-      <c r="N5" s="21"/>
-      <c r="O5" s="21"/>
-      <c r="P5" s="21"/>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="21"/>
-      <c r="S5" s="21"/>
-      <c r="T5" s="21"/>
-      <c r="U5" s="21"/>
-      <c r="V5" s="21"/>
-      <c r="W5" s="21"/>
-      <c r="X5" s="21"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+      <c r="M5" s="37"/>
+      <c r="N5" s="37"/>
+      <c r="O5" s="37"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="37"/>
+      <c r="R5" s="37"/>
+      <c r="S5" s="37"/>
+      <c r="T5" s="37"/>
+      <c r="U5" s="37"/>
+      <c r="V5" s="37"/>
+      <c r="W5" s="37"/>
+      <c r="X5" s="37"/>
     </row>
     <row r="6" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -1547,22 +1546,22 @@
       <c r="B6" s="1">
         <v>-10</v>
       </c>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="21"/>
-      <c r="O6" s="21"/>
-      <c r="P6" s="21"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="21"/>
-      <c r="S6" s="21"/>
-      <c r="T6" s="21"/>
-      <c r="U6" s="21"/>
-      <c r="V6" s="21"/>
-      <c r="W6" s="21"/>
-      <c r="X6" s="21"/>
+      <c r="I6" s="37"/>
+      <c r="J6" s="37"/>
+      <c r="K6" s="37"/>
+      <c r="L6" s="37"/>
+      <c r="M6" s="37"/>
+      <c r="N6" s="37"/>
+      <c r="O6" s="37"/>
+      <c r="P6" s="37"/>
+      <c r="Q6" s="37"/>
+      <c r="R6" s="37"/>
+      <c r="S6" s="37"/>
+      <c r="T6" s="37"/>
+      <c r="U6" s="37"/>
+      <c r="V6" s="37"/>
+      <c r="W6" s="37"/>
+      <c r="X6" s="37"/>
     </row>
     <row r="7" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1571,22 +1570,22 @@
       <c r="B7" s="1">
         <v>-15</v>
       </c>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21"/>
-      <c r="T7" s="21"/>
-      <c r="U7" s="21"/>
-      <c r="V7" s="21"/>
-      <c r="W7" s="21"/>
-      <c r="X7" s="21"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="37"/>
+      <c r="K7" s="37"/>
+      <c r="L7" s="37"/>
+      <c r="M7" s="37"/>
+      <c r="N7" s="37"/>
+      <c r="O7" s="37"/>
+      <c r="P7" s="37"/>
+      <c r="Q7" s="37"/>
+      <c r="R7" s="37"/>
+      <c r="S7" s="37"/>
+      <c r="T7" s="37"/>
+      <c r="U7" s="37"/>
+      <c r="V7" s="37"/>
+      <c r="W7" s="37"/>
+      <c r="X7" s="37"/>
     </row>
     <row r="8" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1595,22 +1594,22 @@
       <c r="B8" s="1">
         <v>-20</v>
       </c>
-      <c r="I8" s="21"/>
-      <c r="J8" s="21"/>
-      <c r="K8" s="21"/>
-      <c r="L8" s="21"/>
-      <c r="M8" s="21"/>
-      <c r="N8" s="21"/>
-      <c r="O8" s="21"/>
-      <c r="P8" s="21"/>
-      <c r="Q8" s="21"/>
-      <c r="R8" s="21"/>
-      <c r="S8" s="21"/>
-      <c r="T8" s="21"/>
-      <c r="U8" s="21"/>
-      <c r="V8" s="21"/>
-      <c r="W8" s="21"/>
-      <c r="X8" s="21"/>
+      <c r="I8" s="37"/>
+      <c r="J8" s="37"/>
+      <c r="K8" s="37"/>
+      <c r="L8" s="37"/>
+      <c r="M8" s="37"/>
+      <c r="N8" s="37"/>
+      <c r="O8" s="37"/>
+      <c r="P8" s="37"/>
+      <c r="Q8" s="37"/>
+      <c r="R8" s="37"/>
+      <c r="S8" s="37"/>
+      <c r="T8" s="37"/>
+      <c r="U8" s="37"/>
+      <c r="V8" s="37"/>
+      <c r="W8" s="37"/>
+      <c r="X8" s="37"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1625,38 +1624,38 @@
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="18"/>
-      <c r="G11" s="19" t="s">
+      <c r="E11" s="36"/>
+      <c r="G11" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="20"/>
-      <c r="J11" s="19" t="s">
+      <c r="H11" s="35"/>
+      <c r="J11" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="K11" s="20"/>
-      <c r="M11" s="19" t="s">
+      <c r="K11" s="35"/>
+      <c r="M11" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="N11" s="20"/>
-      <c r="P11" s="19" t="s">
+      <c r="N11" s="35"/>
+      <c r="P11" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="Q11" s="20"/>
-      <c r="S11" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="T11" s="20"/>
-      <c r="V11" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="W11" s="20"/>
-      <c r="Y11" s="19" t="s">
+      <c r="Q11" s="35"/>
+      <c r="S11" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="T11" s="35"/>
+      <c r="V11" s="34" t="s">
+        <v>35</v>
+      </c>
+      <c r="W11" s="35"/>
+      <c r="Y11" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="Z11" s="20"/>
+      <c r="Z11" s="35"/>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
@@ -1699,13 +1698,13 @@
         <v>0</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="T12" s="6" t="s">
         <v>0</v>
       </c>
       <c r="V12" s="6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="W12" s="6" t="s">
         <v>0</v>
@@ -1792,7 +1791,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D14" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E14, ($Z14,$W14,$T14,$Q14,$N14,$K14,$H14,$E14), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1857,7 +1856,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D15" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E15, ($Z15,$W15,$T15,$Q15,$N15,$K15,$H15,$E15), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1922,7 +1921,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D16" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E16, ($Z16,$W16,$T16,$Q16,$N16,$K16,$H16,$E16), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -1989,7 +1988,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D17" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E17, ($Z17,$W17,$T17,$Q17,$N17,$K17,$H17,$E17), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2056,7 +2055,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D18" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E18, ($Z18,$W18,$T18,$Q18,$N18,$K18,$H18,$E18), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2123,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D19" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E19, ($Z19,$W19,$T19,$Q19,$N19,$K19,$H19,$E19), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E19, ($Z19,$W19,$T19,$Q19,$N19,$K19,$H19,$E19), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2190,7 +2189,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D20" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E20, ($Z20,$W20,$T20,$Q20,$N20,$K20,$H20,$E20), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E20, ($Z20,$W20,$T20,$Q20,$N20,$K20,$H20,$E20), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2257,7 +2256,7 @@
         <v>1</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D21" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E21, ($Z21,$W21,$T21,$Q21,$N21,$K21,$H21,$E21), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2324,7 +2323,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D22" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E22, ($Z22,$W22,$T22,$Q22,$N22,$K22,$H22,$E22), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2391,7 +2390,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D23" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E23, ($Z23,$W23,$T23,$Q23,$N23,$K23,$H23,$E23), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2458,7 +2457,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D24" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E24, ($Z24,$W24,$T24,$Q24,$N24,$K24,$H24,$E24), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2523,7 +2522,7 @@
         <v>1</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D25" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E25, ($Z25,$W25,$T25,$Q25,$N25,$K25,$H25,$E25), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2590,7 +2589,7 @@
         <v>1</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D26" s="3">
         <v>-22.5</v>
@@ -2655,7 +2654,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D27" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E27, ($Z27,$W27,$T27,$Q27,$N27,$K27,$H27,$E27), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2722,7 +2721,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D28" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E28, ($Z28,$W28,$T28,$Q28,$N28,$K28,$H28,$E28), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2787,7 +2786,7 @@
         <v>1</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D29" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E29, ($Z29,$W29,$T29,$Q29,$N29,$K29,$H29,$E29), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2854,7 +2853,7 @@
         <v>1</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D30" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E30, ($Z30,$W30,$T30,$Q30,$N30,$K30,$H30,$E30), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2921,7 +2920,7 @@
         <v>1</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D31" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E31, ($Z31,$W31,$T31,$Q31,$N31,$K31,$H31,$E31), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -2986,7 +2985,7 @@
         <v>1</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D32" s="3">
         <v>-22.5</v>
@@ -3051,7 +3050,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D33" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E33, ($Z33,$W33,$T33,$Q33,$N33,$K33,$H33,$E33), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3118,7 +3117,7 @@
         <v>1</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D34" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E34, ($Z34,$W34,$T34,$Q34,$N34,$K34,$H34,$E34), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3185,7 +3184,7 @@
         <v>1</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D35" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E35, ($Z35,$W35,$T35,$Q35,$N35,$K35,$H35,$E35), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3252,7 +3251,7 @@
         <v>1</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D36" s="3">
         <v>-22.5</v>
@@ -3315,7 +3314,7 @@
         <v>1</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D37" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E37, ($Z37,$W37,$T37,$Q37,$N37,$K37,$H37,$E37), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3382,7 +3381,7 @@
         <v>1</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D38" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E38, ($Z38,$W38,$T38,$Q38,$N38,$K38,$H38,$E38), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3449,7 +3448,7 @@
         <v>1</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D39" s="3">
         <v>35</v>
@@ -3514,7 +3513,7 @@
         <v>1</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D40" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E40, ($Z40,$W40,$T40,$Q40,$N40,$K40,$H40,$E40), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3581,7 +3580,7 @@
         <v>1</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D41" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E41, ($Z41,$W41,$T41,$Q41,$N41,$K41,$H41,$E41), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3648,7 +3647,7 @@
         <v>1</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D42" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E42, ($Z42,$W42,$T42,$Q42,$N42,$K42,$H42,$E42), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3715,7 +3714,7 @@
         <v>1</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D43" s="3">
         <v>-7.5</v>
@@ -3780,7 +3779,7 @@
         <v>1</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D44" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E44, ($Z44,$W44,$T44,$Q44,$N44,$K44,$H44,$E44), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3847,7 +3846,7 @@
         <v>1</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D45" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E45, ($Z45,$W45,$T45,$Q45,$N45,$K45,$H45,$E45), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3914,7 +3913,7 @@
         <v>1</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D46" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E46, ($Z46,$W46,$T46,$Q46,$N46,$K46,$H46,$E46), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -3981,7 +3980,7 @@
         <v>1</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D47" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E47, ($Z47,$W47,$T47,$Q47,$N47,$K47,$H47,$E47), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4048,7 +4047,7 @@
         <v>1</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D48" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E48, ($Z48,$W48,$T48,$Q48,$N48,$K48,$H48,$E48), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4115,7 +4114,7 @@
         <v>1</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D49" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E49, ($Z49,$W49,$T49,$Q49,$N49,$K49,$H49,$E49), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4182,7 +4181,7 @@
         <v>1</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D50" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E50, ($Z50,$W50,$T50,$Q50,$N50,$K50,$H50,$E50), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4249,7 +4248,7 @@
         <v>1</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D51" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E51, ($Z51,$W51,$T51,$Q51,$N51,$K51,$H51,$E51), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4316,7 +4315,7 @@
         <v>1</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D52" s="3">
         <v>-22.5</v>
@@ -4381,7 +4380,7 @@
         <v>1</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D53" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E53, ($Z53,$W53,$T53,$Q53,$N53,$K53,$H53,$E53), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4448,7 +4447,7 @@
         <v>1</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D54" s="3">
         <v>0</v>
@@ -4511,7 +4510,7 @@
         <v>1</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D55" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E55, ($Z55,$W55,$T55,$Q55,$N55,$K55,$H55,$E55), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4578,7 +4577,7 @@
         <v>1</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D56" s="3">
         <v>12.5</v>
@@ -4643,7 +4642,7 @@
         <v>1</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D57" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E57, ($Z57,$W57,$T57,$Q57,$N57,$K57,$H57,$E57), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4710,7 +4709,7 @@
         <v>1</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D58" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E58, ($Z58,$W58,$T58,$Q58,$N58,$K58,$H58,$E58), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4777,7 +4776,7 @@
         <v>1</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D59" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E59, ($Z59,$W59,$T59,$Q59,$N59,$K59,$H59,$E59), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4844,7 +4843,7 @@
         <v>1</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D60" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E60, ($Z60,$W60,$T60,$Q60,$N60,$K60,$H60,$E60), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4909,7 +4908,7 @@
         <v>1</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D61" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E61, ($Z61,$W61,$T61,$Q61,$N61,$K61,$H61,$E61), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -4976,7 +4975,7 @@
         <v>1</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D62" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E62, ($Z62,$W62,$T62,$Q62,$N62,$K62,$H62,$E62), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5043,7 +5042,7 @@
         <v>1</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D63" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E63, ($Z63,$W63,$T63,$Q63,$N63,$K63,$H63,$E63), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5110,7 +5109,7 @@
         <v>1</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D64" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E64, ($Z64,$W64,$T64,$Q64,$N64,$K64,$H64,$E64), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5177,7 +5176,7 @@
         <v>1</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D65" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E65, ($Z65,$W65,$T65,$Q65,$N65,$K65,$H65,$E65), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5244,7 +5243,7 @@
         <v>1</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D66" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E66, ($Z66,$W66,$T66,$Q66,$N66,$K66,$H66,$E66), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5311,7 +5310,7 @@
         <v>1</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D67" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E67, ($Z67,$W67,$T67,$Q67,$N67,$K67,$H67,$E67), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5378,7 +5377,7 @@
         <v>1</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D68" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E68, ($Z68,$W68,$T68,$Q68,$N68,$K68,$H68,$E68), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5445,7 +5444,7 @@
         <v>1</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D69" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E69, ($Z69,$W69,$T69,$Q69,$N69,$K69,$H69,$E69), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5512,7 +5511,7 @@
         <v>1</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D70" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E70, ($Z70,$W70,$T70,$Q70,$N70,$K70,$H70,$E70), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5577,7 +5576,7 @@
         <v>1</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D71" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E71, ($Z71,$W71,$T71,$Q71,$N71,$K71,$H71,$E71), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5644,7 +5643,7 @@
         <v>1</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D72" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E72, ($Z72,$W72,$T72,$Q72,$N72,$K72,$H72,$E72), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5711,7 +5710,7 @@
         <v>1</v>
       </c>
       <c r="C73" s="14" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D73" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E73, ($Z73,$W73,$T73,$Q73,$N73,$K73,$H73,$E73), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -5778,7 +5777,7 @@
         <v>1</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D74" s="3">
         <v>-7.5</v>
@@ -5843,7 +5842,7 @@
         <v>1</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D75" s="3">
         <v>0</v>
@@ -5902,7 +5901,7 @@
         <v>1</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D76" s="3">
         <v>-20</v>
@@ -5966,7 +5965,7 @@
         <v>1</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D77" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E77, ($Z77,$W77,$T77,$Q77,$N77,$K77,$H77,$E77), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -6031,7 +6030,7 @@
         <v>1</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D78" s="3">
         <v>0</v>
@@ -6090,7 +6089,7 @@
         <v>1</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D79" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E79, ($Z79,$W79,$T79,$Q79,$N79,$K79,$H79,$E79), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -6157,7 +6156,7 @@
         <v>1</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D80" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E80, ($Z80,$W80,$T80,$Q80,$N80,$K80,$H80,$E80), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -6224,7 +6223,7 @@
         <v>1</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D81" s="3">
         <v>-22.5</v>
@@ -6289,7 +6288,7 @@
         <v>1</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D82" s="3">
         <v>0</v>
@@ -6348,7 +6347,7 @@
         <v>1</v>
       </c>
       <c r="C83" s="14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D83" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E83, ($Z83,$W83,$T83,$Q83,$N83,$K83,$H83,$E83), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -6415,7 +6414,7 @@
         <v>1</v>
       </c>
       <c r="C84" s="14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D84" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E84, ($Z84,$W84,$T84,$Q84,$N84,$K84,$H84,$E84), 0),  $A$2:$B$10, 2, FALSE))</f>
@@ -6481,47 +6480,65 @@
       <c r="B85" s="1">
         <v>1</v>
       </c>
-      <c r="C85" s="14"/>
-      <c r="D85" s="3" t="str">
+      <c r="C85" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E85" s="1"/>
-      <c r="G85" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="E85" s="1">
+        <v>50</v>
+      </c>
+      <c r="G85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H85" s="1"/>
-      <c r="J85" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="H85" s="1">
+        <v>70</v>
+      </c>
+      <c r="J85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K85" s="1"/>
-      <c r="M85" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="K85" s="1">
+        <v>0</v>
+      </c>
+      <c r="M85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N85" s="1"/>
-      <c r="P85" s="3" t="str">
+        <v>-15</v>
+      </c>
+      <c r="N85" s="1">
+        <v>30</v>
+      </c>
+      <c r="P85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q85" s="1"/>
-      <c r="S85" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q85" s="1">
+        <v>100</v>
+      </c>
+      <c r="S85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T85" s="1"/>
-      <c r="V85" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="T85" s="1">
+        <v>60</v>
+      </c>
+      <c r="V85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W85" s="1"/>
-      <c r="Y85" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="W85" s="1">
+        <v>40</v>
+      </c>
+      <c r="Y85" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z85, ($Z85,$W85,$T85,$Q85,$N85,$K85,$H85,$E85), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z85" s="1"/>
+        <v>-20</v>
+      </c>
+      <c r="Z85" s="1">
+        <v>20</v>
+      </c>
     </row>
     <row r="86" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A86" s="5" t="s">
@@ -6530,47 +6547,65 @@
       <c r="B86" s="1">
         <v>1</v>
       </c>
-      <c r="C86" s="14"/>
-      <c r="D86" s="3" t="str">
+      <c r="C86" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(E86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(E86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="E86" s="1"/>
-      <c r="G86" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="E86" s="1">
+        <v>60</v>
+      </c>
+      <c r="G86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(H86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(H86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="H86" s="1"/>
-      <c r="J86" s="3" t="str">
+        <v>20</v>
+      </c>
+      <c r="H86" s="1">
+        <v>70</v>
+      </c>
+      <c r="J86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(K86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(K86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="K86" s="1"/>
-      <c r="M86" s="3" t="str">
+        <v>-10</v>
+      </c>
+      <c r="K86" s="1">
+        <v>40</v>
+      </c>
+      <c r="M86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(N86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(N86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="N86" s="1"/>
-      <c r="P86" s="3" t="str">
+        <v>-25</v>
+      </c>
+      <c r="N86" s="1">
+        <v>0</v>
+      </c>
+      <c r="P86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Q86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Q86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Q86" s="1"/>
-      <c r="S86" s="3" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q86" s="1">
+        <v>100</v>
+      </c>
+      <c r="S86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(T86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(T86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="T86" s="1"/>
-      <c r="V86" s="3" t="str">
+        <v>-20</v>
+      </c>
+      <c r="T86" s="1">
+        <v>20</v>
+      </c>
+      <c r="V86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(W86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(W86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="W86" s="1"/>
-      <c r="Y86" s="3" t="str">
+        <v>-5</v>
+      </c>
+      <c r="W86" s="1">
+        <v>50</v>
+      </c>
+      <c r="Y86" s="3">
         <f>IF(ISERROR(VLOOKUP(RANK(Z86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE)),"",VLOOKUP(RANK(Z86, ($Z86,$W86,$T86,$Q86,$N86,$K86,$H86,$E86), 0),  $A$2:$B$10, 2, FALSE))</f>
-        <v/>
-      </c>
-      <c r="Z86" s="1"/>
+        <v>-15</v>
+      </c>
+      <c r="Z86" s="1">
+        <v>30</v>
+      </c>
     </row>
     <row r="87" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A87" s="5"/>
@@ -6666,194 +6701,152 @@
       </c>
       <c r="H89" s="10">
         <f>SUM(G13:G86)</f>
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="J89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K89" s="10">
         <f>SUM(J13:J86)</f>
-        <v>-305</v>
+        <v>-340</v>
       </c>
       <c r="M89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="N89" s="10">
         <f>SUM(M13:M86)</f>
-        <v>317.5</v>
+        <v>277.5</v>
       </c>
       <c r="P89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Q89" s="10">
         <f>SUM(P13:P86)</f>
-        <v>-130</v>
+        <v>-30</v>
       </c>
       <c r="S89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="T89" s="10">
         <f>SUM(S13:S86)</f>
-        <v>32.5</v>
+        <v>17.5</v>
       </c>
       <c r="V89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="W89" s="10">
         <f>SUM(V13:V86)</f>
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="Y89" s="6" t="s">
         <v>7</v>
       </c>
       <c r="Z89" s="10">
         <f>SUM(Y13:Y86)</f>
-        <v>-30</v>
+        <v>-65</v>
       </c>
       <c r="AA89" s="1">
         <f>SUM(E89,H89,K89,N89,Q89,T89,W89,Z89)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="N95" s="35"/>
-      <c r="O95" s="35"/>
-      <c r="P95" s="35"/>
-      <c r="Q95" s="35"/>
-      <c r="R95" s="35"/>
-      <c r="S95" s="35"/>
-      <c r="T95" s="35"/>
-      <c r="U95" s="35"/>
-      <c r="V95" s="35"/>
-      <c r="W95" s="35"/>
-      <c r="X95" s="35"/>
-      <c r="Y95" s="35"/>
-    </row>
-    <row r="96" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="N96" s="35"/>
-      <c r="O96" s="35"/>
-      <c r="P96" s="35"/>
-      <c r="Q96" s="35"/>
-      <c r="R96" s="35"/>
-      <c r="S96" s="35"/>
-      <c r="T96" s="35"/>
-      <c r="U96" s="35"/>
-      <c r="V96" s="35"/>
-      <c r="W96" s="35"/>
-      <c r="X96" s="35"/>
-      <c r="Y96" s="35"/>
-    </row>
-    <row r="97" spans="2:25" ht="19" x14ac:dyDescent="0.25">
-      <c r="C97" s="26" t="s">
+    <row r="97" spans="2:23" ht="19" x14ac:dyDescent="0.25">
+      <c r="C97" s="33" t="s">
+        <v>112</v>
+      </c>
+      <c r="D97" s="33"/>
+      <c r="E97" s="33"/>
+      <c r="F97" s="33"/>
+      <c r="G97" s="33"/>
+      <c r="H97" s="33"/>
+      <c r="I97" s="33"/>
+      <c r="J97" s="33"/>
+      <c r="O97" s="28"/>
+      <c r="P97" s="28"/>
+      <c r="R97" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="S97" s="31"/>
+      <c r="T97" s="31"/>
+      <c r="U97" s="31"/>
+      <c r="V97" s="31"/>
+      <c r="W97" s="28"/>
+    </row>
+    <row r="98" spans="2:23" ht="19" x14ac:dyDescent="0.25">
+      <c r="C98" s="33" t="s">
+        <v>26</v>
+      </c>
+      <c r="D98" s="33"/>
+      <c r="E98" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="F98" s="33"/>
+      <c r="G98" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="H98" s="33"/>
+      <c r="I98" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="J98" s="33"/>
+      <c r="O98" s="28"/>
+      <c r="P98" s="28"/>
+      <c r="R98" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="D97" s="26"/>
-      <c r="E97" s="26"/>
-      <c r="F97" s="26"/>
-      <c r="G97" s="26"/>
-      <c r="H97" s="26"/>
-      <c r="I97" s="26"/>
-      <c r="J97" s="26"/>
-      <c r="N97" s="35"/>
-      <c r="O97" s="36"/>
-      <c r="P97" s="36"/>
-      <c r="Q97" s="35"/>
-      <c r="R97" s="28" t="s">
+      <c r="S98" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="S97" s="28"/>
-      <c r="T97" s="28"/>
-      <c r="U97" s="28"/>
-      <c r="V97" s="28"/>
-      <c r="W97" s="36"/>
-      <c r="X97" s="35"/>
-      <c r="Y97" s="35"/>
-    </row>
-    <row r="98" spans="2:25" ht="19" x14ac:dyDescent="0.25">
-      <c r="C98" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="D98" s="26"/>
-      <c r="E98" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="F98" s="26"/>
-      <c r="G98" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="H98" s="26"/>
-      <c r="I98" s="26" t="s">
+      <c r="T98" s="31"/>
+      <c r="U98" s="31"/>
+      <c r="V98" s="31"/>
+      <c r="W98" s="28"/>
+    </row>
+    <row r="99" spans="2:23" ht="19" x14ac:dyDescent="0.25">
+      <c r="C99" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="D99" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="E99" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="F99" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="G99" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="H99" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="I99" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="J99" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="K99" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="R99" s="32"/>
+      <c r="S99" s="29" t="s">
         <v>118</v>
       </c>
-      <c r="J98" s="26"/>
-      <c r="N98" s="35"/>
-      <c r="O98" s="36"/>
-      <c r="P98" s="36"/>
-      <c r="Q98" s="35"/>
-      <c r="R98" s="28" t="s">
-        <v>116</v>
-      </c>
-      <c r="S98" s="28" t="s">
-        <v>117</v>
-      </c>
-      <c r="T98" s="28"/>
-      <c r="U98" s="28"/>
-      <c r="V98" s="28"/>
-      <c r="W98" s="36"/>
-      <c r="X98" s="35"/>
-      <c r="Y98" s="35"/>
-    </row>
-    <row r="99" spans="2:25" ht="19" x14ac:dyDescent="0.25">
-      <c r="C99" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="D99" s="34" t="s">
-        <v>117</v>
-      </c>
-      <c r="E99" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="F99" s="34" t="s">
-        <v>117</v>
-      </c>
-      <c r="G99" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="H99" s="34" t="s">
-        <v>117</v>
-      </c>
-      <c r="I99" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="J99" s="34" t="s">
-        <v>117</v>
-      </c>
-      <c r="K99" s="33" t="s">
+      <c r="T99" s="29" t="s">
         <v>119</v>
       </c>
-      <c r="N99" s="35"/>
-      <c r="O99" s="35"/>
-      <c r="P99" s="35"/>
-      <c r="Q99" s="35"/>
-      <c r="R99" s="27"/>
-      <c r="S99" s="37" t="s">
+      <c r="U99" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="T99" s="37" t="s">
-        <v>121</v>
-      </c>
-      <c r="U99" s="37" t="s">
-        <v>122</v>
-      </c>
-      <c r="V99" s="38" t="s">
+      <c r="V99" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="W99" s="36"/>
-      <c r="X99" s="35"/>
-      <c r="Y99" s="35"/>
-    </row>
-    <row r="100" spans="2:25" ht="21" x14ac:dyDescent="0.25">
-      <c r="B100" s="32" t="s">
+      <c r="W99" s="28"/>
+    </row>
+    <row r="100" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B100" s="25" t="s">
         <v>8</v>
       </c>
       <c r="C100" s="1">
@@ -6868,13 +6861,21 @@
       <c r="F100" s="1">
         <v>3</v>
       </c>
-      <c r="G100" s="1"/>
-      <c r="H100" s="1"/>
-      <c r="I100" s="1"/>
-      <c r="J100" s="1"/>
+      <c r="G100" s="1">
+        <v>0</v>
+      </c>
+      <c r="H100" s="1">
+        <v>0</v>
+      </c>
+      <c r="I100" s="1">
+        <v>0</v>
+      </c>
+      <c r="J100" s="1">
+        <v>3</v>
+      </c>
       <c r="K100" s="15">
         <f>SUM(C100:J100)</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="Q100" s="15" t="s">
         <v>8</v>
@@ -6883,28 +6884,28 @@
         <f>E89</f>
         <v>30</v>
       </c>
-      <c r="S100" s="29">
+      <c r="S100" s="22">
         <v>-400</v>
       </c>
       <c r="T100" s="10">
-        <f>K100</f>
-        <v>8</v>
+        <f t="shared" ref="T100:T107" si="0">K100</f>
+        <v>11</v>
       </c>
       <c r="U100" s="10">
-        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T100, 0)</f>
-        <v>984.61538461538464</v>
-      </c>
-      <c r="V100" s="31">
+        <f t="shared" ref="U100:U107" si="1">IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T100, 0)</f>
+        <v>414.11764705882354</v>
+      </c>
+      <c r="V100" s="24">
         <f>SUM(R100,S100,U100)</f>
-        <v>614.61538461538464</v>
+        <v>44.117647058823536</v>
       </c>
       <c r="W100" s="15" t="str">
         <f>Q100</f>
         <v>Jaya</v>
       </c>
     </row>
-    <row r="101" spans="2:25" ht="21" x14ac:dyDescent="0.25">
-      <c r="B101" s="32" t="s">
+    <row r="101" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B101" s="25" t="s">
         <v>5</v>
       </c>
       <c r="C101" s="1">
@@ -6919,43 +6920,51 @@
       <c r="F101" s="1">
         <v>0</v>
       </c>
-      <c r="G101" s="1"/>
-      <c r="H101" s="1"/>
-      <c r="I101" s="1"/>
-      <c r="J101" s="1"/>
+      <c r="G101" s="1">
+        <v>1</v>
+      </c>
+      <c r="H101" s="1">
+        <v>0</v>
+      </c>
+      <c r="I101" s="1">
+        <v>1</v>
+      </c>
+      <c r="J101" s="1">
+        <v>0</v>
+      </c>
       <c r="K101" s="15">
-        <f t="shared" ref="K101:K107" si="0">SUM(C101:J101)</f>
-        <v>0</v>
+        <f t="shared" ref="K101:K107" si="2">SUM(C101:J101)</f>
+        <v>2</v>
       </c>
       <c r="Q101" s="15" t="s">
         <v>5</v>
       </c>
       <c r="R101" s="10">
         <f>H89</f>
-        <v>60</v>
-      </c>
-      <c r="S101" s="29">
+        <v>100</v>
+      </c>
+      <c r="S101" s="22">
         <v>-400</v>
       </c>
       <c r="T101" s="10">
-        <f>K101</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="U101" s="10">
-        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T101, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="V101" s="31">
-        <f t="shared" ref="V101:V107" si="1">SUM(R101,S101,U101)</f>
-        <v>-340</v>
+        <f t="shared" si="1"/>
+        <v>75.294117647058826</v>
+      </c>
+      <c r="V101" s="24">
+        <f t="shared" ref="V101:V107" si="3">SUM(R101,S101,U101)</f>
+        <v>-224.70588235294116</v>
       </c>
       <c r="W101" s="15" t="str">
-        <f t="shared" ref="W101:W107" si="2">Q101</f>
+        <f t="shared" ref="W101:W107" si="4">Q101</f>
         <v>Justin</v>
       </c>
     </row>
-    <row r="102" spans="2:25" ht="21" x14ac:dyDescent="0.25">
-      <c r="B102" s="32" t="s">
+    <row r="102" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B102" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C102" s="1">
@@ -6970,267 +6979,315 @@
       <c r="F102" s="1">
         <v>11</v>
       </c>
-      <c r="G102" s="1"/>
-      <c r="H102" s="1"/>
-      <c r="I102" s="1"/>
-      <c r="J102" s="1"/>
+      <c r="G102" s="1">
+        <v>0</v>
+      </c>
+      <c r="H102" s="1">
+        <v>0</v>
+      </c>
+      <c r="I102" s="1">
+        <v>0</v>
+      </c>
+      <c r="J102" s="1">
+        <v>3</v>
+      </c>
       <c r="K102" s="15">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="Q102" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="R102" s="10">
+        <f>K89</f>
+        <v>-340</v>
+      </c>
+      <c r="S102" s="22">
+        <v>-400</v>
+      </c>
+      <c r="T102" s="10">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="U102" s="10">
+        <f t="shared" si="1"/>
+        <v>602.35294117647061</v>
+      </c>
+      <c r="V102" s="24">
+        <f t="shared" si="3"/>
+        <v>-137.64705882352939</v>
+      </c>
+      <c r="W102" s="15" t="str">
+        <f t="shared" si="4"/>
+        <v>Ram</v>
+      </c>
+    </row>
+    <row r="103" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B103" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C103" s="1">
+        <v>0</v>
+      </c>
+      <c r="D103" s="1">
+        <v>0</v>
+      </c>
+      <c r="E103" s="1">
+        <v>0</v>
+      </c>
+      <c r="F103" s="1">
+        <v>3</v>
+      </c>
+      <c r="G103" s="1">
+        <v>0</v>
+      </c>
+      <c r="H103" s="1">
+        <v>0</v>
+      </c>
+      <c r="I103" s="1">
+        <v>0</v>
+      </c>
+      <c r="J103" s="1">
+        <v>11</v>
+      </c>
+      <c r="K103" s="15">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="Q103" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="R103" s="10">
+        <f>N89</f>
+        <v>277.5</v>
+      </c>
+      <c r="S103" s="22">
+        <v>-400</v>
+      </c>
+      <c r="T103" s="10">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="U103" s="10">
+        <f t="shared" si="1"/>
+        <v>527.05882352941182</v>
+      </c>
+      <c r="V103" s="24">
+        <f t="shared" si="3"/>
+        <v>404.55882352941182</v>
+      </c>
+      <c r="W103" s="15" t="str">
+        <f t="shared" si="4"/>
+        <v>Sibi</v>
+      </c>
+    </row>
+    <row r="104" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B104" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C104" s="1">
+        <v>2</v>
+      </c>
+      <c r="D104" s="1">
+        <v>0</v>
+      </c>
+      <c r="E104" s="1">
+        <v>0</v>
+      </c>
+      <c r="F104" s="1">
+        <v>0</v>
+      </c>
+      <c r="G104" s="1">
+        <v>2</v>
+      </c>
+      <c r="H104" s="1">
+        <v>11</v>
+      </c>
+      <c r="I104" s="1">
+        <v>0</v>
+      </c>
+      <c r="J104" s="1">
+        <v>11</v>
+      </c>
+      <c r="K104" s="15">
+        <f t="shared" si="2"/>
+        <v>26</v>
+      </c>
+      <c r="Q104" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="R104" s="10">
+        <f>Q89</f>
+        <v>-30</v>
+      </c>
+      <c r="S104" s="22">
+        <v>-400</v>
+      </c>
+      <c r="T104" s="10">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="U104" s="10">
+        <f t="shared" si="1"/>
+        <v>978.82352941176475</v>
+      </c>
+      <c r="V104" s="24">
+        <f t="shared" si="3"/>
+        <v>548.82352941176475</v>
+      </c>
+      <c r="W104" s="15" t="str">
+        <f t="shared" si="4"/>
+        <v>Sundar</v>
+      </c>
+    </row>
+    <row r="105" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B105" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="C105" s="1">
+        <v>0</v>
+      </c>
+      <c r="D105" s="1">
+        <v>0</v>
+      </c>
+      <c r="E105" s="1">
+        <v>0</v>
+      </c>
+      <c r="F105" s="1">
+        <v>0</v>
+      </c>
+      <c r="G105" s="1">
+        <v>0</v>
+      </c>
+      <c r="H105" s="1">
+        <v>0</v>
+      </c>
+      <c r="I105" s="1">
+        <v>2</v>
+      </c>
+      <c r="J105" s="1">
+        <v>11</v>
+      </c>
+      <c r="K105" s="15">
+        <f t="shared" si="2"/>
+        <v>13</v>
+      </c>
+      <c r="Q105" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="R105" s="10">
+        <f>T89</f>
+        <v>17.5</v>
+      </c>
+      <c r="S105" s="22">
+        <v>-400</v>
+      </c>
+      <c r="T105" s="10">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="Q102" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="R102" s="10">
-        <f>K89</f>
-        <v>-305</v>
-      </c>
-      <c r="S102" s="29">
+      <c r="U105" s="10">
+        <f t="shared" si="1"/>
+        <v>489.41176470588238</v>
+      </c>
+      <c r="V105" s="24">
+        <f t="shared" si="3"/>
+        <v>106.91176470588238</v>
+      </c>
+      <c r="W105" s="15" t="str">
+        <f t="shared" si="4"/>
+        <v>Rapaka</v>
+      </c>
+    </row>
+    <row r="106" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B106" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C106" s="1">
+        <v>0</v>
+      </c>
+      <c r="D106" s="1">
+        <v>0</v>
+      </c>
+      <c r="E106" s="1">
+        <v>0</v>
+      </c>
+      <c r="F106" s="1">
+        <v>0</v>
+      </c>
+      <c r="G106" s="1">
+        <v>0</v>
+      </c>
+      <c r="H106" s="1">
+        <v>0</v>
+      </c>
+      <c r="I106" s="1">
+        <v>0</v>
+      </c>
+      <c r="J106" s="1">
+        <v>3</v>
+      </c>
+      <c r="K106" s="15">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="Q106" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="R106" s="10">
+        <f>W89</f>
+        <v>10</v>
+      </c>
+      <c r="S106" s="22">
         <v>-400</v>
       </c>
-      <c r="T102" s="10">
-        <f>K102</f>
-        <v>13</v>
-      </c>
-      <c r="U102" s="10">
-        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T102, 0)</f>
-        <v>1600</v>
-      </c>
-      <c r="V102" s="31">
-        <f t="shared" si="1"/>
-        <v>895</v>
-      </c>
-      <c r="W102" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>Ram</v>
-      </c>
-    </row>
-    <row r="103" spans="2:25" ht="21" x14ac:dyDescent="0.25">
-      <c r="B103" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="C103" s="1">
-        <v>0</v>
-      </c>
-      <c r="D103" s="1">
-        <v>0</v>
-      </c>
-      <c r="E103" s="1">
-        <v>0</v>
-      </c>
-      <c r="F103" s="1">
-        <v>3</v>
-      </c>
-      <c r="G103" s="1"/>
-      <c r="H103" s="1"/>
-      <c r="I103" s="1"/>
-      <c r="J103" s="1"/>
-      <c r="K103" s="15">
+      <c r="T106" s="10">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="Q103" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="R103" s="10">
-        <f>N89</f>
-        <v>317.5</v>
-      </c>
-      <c r="S103" s="29">
-        <v>-400</v>
-      </c>
-      <c r="T103" s="10">
-        <f>K103</f>
-        <v>3</v>
-      </c>
-      <c r="U103" s="10">
-        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T103, 0)</f>
-        <v>369.23076923076923</v>
-      </c>
-      <c r="V103" s="31">
+      <c r="U106" s="10">
         <f t="shared" si="1"/>
-        <v>286.73076923076923</v>
-      </c>
-      <c r="W103" s="15" t="str">
+        <v>112.94117647058823</v>
+      </c>
+      <c r="V106" s="24">
+        <f t="shared" si="3"/>
+        <v>-277.05882352941177</v>
+      </c>
+      <c r="W106" s="15" t="str">
+        <f t="shared" si="4"/>
+        <v>Jayanth</v>
+      </c>
+    </row>
+    <row r="107" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="B107" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C107" s="1">
+        <v>0</v>
+      </c>
+      <c r="D107" s="1">
+        <v>0</v>
+      </c>
+      <c r="E107" s="1">
+        <v>0</v>
+      </c>
+      <c r="F107" s="1">
+        <v>0</v>
+      </c>
+      <c r="G107" s="1">
+        <v>0</v>
+      </c>
+      <c r="H107" s="1">
+        <v>0</v>
+      </c>
+      <c r="I107" s="1">
+        <v>0</v>
+      </c>
+      <c r="J107" s="1">
+        <v>0</v>
+      </c>
+      <c r="K107" s="15">
         <f t="shared" si="2"/>
-        <v>Sibi</v>
-      </c>
-    </row>
-    <row r="104" spans="2:25" ht="21" x14ac:dyDescent="0.25">
-      <c r="B104" s="32" t="s">
-        <v>10</v>
-      </c>
-      <c r="C104" s="1">
-        <v>2</v>
-      </c>
-      <c r="D104" s="1">
-        <v>0</v>
-      </c>
-      <c r="E104" s="1">
-        <v>0</v>
-      </c>
-      <c r="F104" s="1">
-        <v>0</v>
-      </c>
-      <c r="G104" s="1"/>
-      <c r="H104" s="1"/>
-      <c r="I104" s="1"/>
-      <c r="J104" s="1"/>
-      <c r="K104" s="15">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="Q104" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="R104" s="10">
-        <f>Q89</f>
-        <v>-130</v>
-      </c>
-      <c r="S104" s="29">
-        <v>-400</v>
-      </c>
-      <c r="T104" s="10">
-        <f>K104</f>
-        <v>2</v>
-      </c>
-      <c r="U104" s="10">
-        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T104, 0)</f>
-        <v>246.15384615384616</v>
-      </c>
-      <c r="V104" s="31">
-        <f t="shared" si="1"/>
-        <v>-283.84615384615381</v>
-      </c>
-      <c r="W104" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>Sundar</v>
-      </c>
-    </row>
-    <row r="105" spans="2:25" ht="21" x14ac:dyDescent="0.25">
-      <c r="B105" s="32" t="s">
-        <v>113</v>
-      </c>
-      <c r="C105" s="1">
-        <v>0</v>
-      </c>
-      <c r="D105" s="1">
-        <v>0</v>
-      </c>
-      <c r="E105" s="1">
-        <v>0</v>
-      </c>
-      <c r="F105" s="1">
-        <v>0</v>
-      </c>
-      <c r="G105" s="1"/>
-      <c r="H105" s="1"/>
-      <c r="I105" s="1"/>
-      <c r="J105" s="1"/>
-      <c r="K105" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Q105" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="R105" s="10">
-        <f>T89</f>
-        <v>32.5</v>
-      </c>
-      <c r="S105" s="29">
-        <v>-400</v>
-      </c>
-      <c r="T105" s="10">
-        <f>K105</f>
-        <v>0</v>
-      </c>
-      <c r="U105" s="10">
-        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T105, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="V105" s="31">
-        <f t="shared" si="1"/>
-        <v>-367.5</v>
-      </c>
-      <c r="W105" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>Rapaka</v>
-      </c>
-    </row>
-    <row r="106" spans="2:25" ht="21" x14ac:dyDescent="0.25">
-      <c r="B106" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="C106" s="1">
-        <v>0</v>
-      </c>
-      <c r="D106" s="1">
-        <v>0</v>
-      </c>
-      <c r="E106" s="1">
-        <v>0</v>
-      </c>
-      <c r="F106" s="1">
-        <v>0</v>
-      </c>
-      <c r="G106" s="1"/>
-      <c r="H106" s="1"/>
-      <c r="I106" s="1"/>
-      <c r="J106" s="1"/>
-      <c r="K106" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Q106" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="R106" s="10">
-        <f>W89</f>
-        <v>25</v>
-      </c>
-      <c r="S106" s="29">
-        <v>-400</v>
-      </c>
-      <c r="T106" s="10">
-        <f>K106</f>
-        <v>0</v>
-      </c>
-      <c r="U106" s="10">
-        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T106, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="V106" s="31">
-        <f t="shared" si="1"/>
-        <v>-375</v>
-      </c>
-      <c r="W106" s="15" t="str">
-        <f t="shared" si="2"/>
-        <v>Jayanth</v>
-      </c>
-    </row>
-    <row r="107" spans="2:25" ht="21" x14ac:dyDescent="0.25">
-      <c r="B107" s="32" t="s">
-        <v>30</v>
-      </c>
-      <c r="C107" s="1">
-        <v>0</v>
-      </c>
-      <c r="D107" s="1">
-        <v>0</v>
-      </c>
-      <c r="E107" s="1">
-        <v>0</v>
-      </c>
-      <c r="F107" s="1">
-        <v>0</v>
-      </c>
-      <c r="G107" s="1"/>
-      <c r="H107" s="1"/>
-      <c r="I107" s="1"/>
-      <c r="J107" s="1"/>
-      <c r="K107" s="15">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q107" s="15" t="s">
@@ -7238,34 +7295,34 @@
       </c>
       <c r="R107" s="10">
         <f>Z89</f>
-        <v>-30</v>
-      </c>
-      <c r="S107" s="29">
+        <v>-65</v>
+      </c>
+      <c r="S107" s="22">
         <v>-400</v>
       </c>
       <c r="T107" s="10">
-        <f>K107</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="U107" s="10">
-        <f>IFERROR((-SUM($S$100:$S$107)/SUM($T$100:$T$107))*$T107, 0)</f>
-        <v>0</v>
-      </c>
-      <c r="V107" s="31">
         <f t="shared" si="1"/>
-        <v>-430</v>
+        <v>0</v>
+      </c>
+      <c r="V107" s="24">
+        <f t="shared" si="3"/>
+        <v>-465</v>
       </c>
       <c r="W107" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>Vikcy</v>
       </c>
     </row>
-    <row r="108" spans="2:25" ht="21" x14ac:dyDescent="0.25">
-      <c r="R108" s="30">
+    <row r="108" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+      <c r="R108" s="23">
         <f>SUM(R100:R107)</f>
         <v>0</v>
       </c>
-      <c r="V108" s="39">
+      <c r="V108" s="30">
         <f>SUM(V100:V107)</f>
         <v>0</v>
       </c>
@@ -7273,6 +7330,15 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="17">
+    <mergeCell ref="I2:X8"/>
+    <mergeCell ref="S11:T11"/>
+    <mergeCell ref="P11:Q11"/>
+    <mergeCell ref="V11:W11"/>
+    <mergeCell ref="Y11:Z11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="M11:N11"/>
     <mergeCell ref="R98:R99"/>
     <mergeCell ref="S98:V98"/>
     <mergeCell ref="R97:V97"/>
@@ -7281,57 +7347,48 @@
     <mergeCell ref="G98:H98"/>
     <mergeCell ref="I98:J98"/>
     <mergeCell ref="C97:J97"/>
-    <mergeCell ref="Y11:Z11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="I2:X8"/>
-    <mergeCell ref="S11:T11"/>
-    <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="V11:W11"/>
   </mergeCells>
   <conditionalFormatting sqref="E89">
-    <cfRule type="cellIs" dxfId="32" priority="145" operator="lessThan">
+    <cfRule type="cellIs" dxfId="32" priority="147" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="31" priority="146" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="147" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="145" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H89">
-    <cfRule type="cellIs" dxfId="29" priority="40" operator="lessThan">
+    <cfRule type="cellIs" dxfId="29" priority="42" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="28" priority="41" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="42" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="40" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K89">
-    <cfRule type="cellIs" dxfId="26" priority="37" operator="lessThan">
+    <cfRule type="cellIs" dxfId="26" priority="39" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="25" priority="38" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="39" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="37" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N89">
-    <cfRule type="cellIs" dxfId="23" priority="34" operator="lessThan">
+    <cfRule type="cellIs" dxfId="23" priority="36" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="22" priority="35" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="36" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="34" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7339,65 +7396,65 @@
     <cfRule type="cellIs" dxfId="20" priority="31" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="32" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="33" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="33" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="32" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R100:R107">
+    <cfRule type="cellIs" dxfId="17" priority="6" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="4" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="5" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T89">
-    <cfRule type="cellIs" dxfId="17" priority="28" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="30" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="28" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="30" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="29" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V100:V107">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W89">
-    <cfRule type="cellIs" dxfId="14" priority="25" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="27" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="25" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="27" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="26" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z89">
-    <cfRule type="cellIs" dxfId="11" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="23" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="22" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="24" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R100:R107">
-    <cfRule type="cellIs" dxfId="8" priority="4" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="6" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V100:V107">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7419,79 +7476,79 @@
   <sheetData>
     <row r="7" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="8" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E8" s="22">
-        <v>5</v>
-      </c>
-      <c r="F8" s="25">
+      <c r="E8" s="18">
+        <v>5</v>
+      </c>
+      <c r="F8" s="21">
         <f>(3200/SUM($E$8:$E$15))*E8</f>
         <v>69.86899563318778</v>
       </c>
     </row>
     <row r="9" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E9" s="23">
+      <c r="E9" s="19">
         <v>100</v>
       </c>
-      <c r="F9" s="25">
+      <c r="F9" s="21">
         <f t="shared" ref="F9:F15" si="0">(3200/SUM($E$8:$E$15))*E9</f>
         <v>1397.3799126637555</v>
       </c>
     </row>
     <row r="10" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E10" s="23">
+      <c r="E10" s="19">
         <v>3</v>
       </c>
-      <c r="F10" s="25">
+      <c r="F10" s="21">
         <f t="shared" si="0"/>
         <v>41.921397379912662</v>
       </c>
     </row>
     <row r="11" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E11" s="23">
-        <v>0</v>
-      </c>
-      <c r="F11" s="25">
+      <c r="E11" s="19">
+        <v>0</v>
+      </c>
+      <c r="F11" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E12" s="23">
+      <c r="E12" s="19">
         <v>22</v>
       </c>
-      <c r="F12" s="25">
+      <c r="F12" s="21">
         <f t="shared" si="0"/>
         <v>307.42358078602621</v>
       </c>
     </row>
     <row r="13" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E13" s="23">
+      <c r="E13" s="19">
         <v>26</v>
       </c>
-      <c r="F13" s="25">
+      <c r="F13" s="21">
         <f t="shared" si="0"/>
         <v>363.31877729257644</v>
       </c>
     </row>
     <row r="14" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E14" s="23">
+      <c r="E14" s="19">
         <v>61</v>
       </c>
-      <c r="F14" s="25">
+      <c r="F14" s="21">
         <f t="shared" si="0"/>
         <v>852.40174672489081</v>
       </c>
     </row>
     <row r="15" spans="5:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="E15" s="23">
+      <c r="E15" s="19">
         <v>12</v>
       </c>
-      <c r="F15" s="25">
+      <c r="F15" s="21">
         <f t="shared" si="0"/>
         <v>167.68558951965065</v>
       </c>
     </row>
     <row r="16" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="F16" s="24">
+      <c r="F16" s="20">
         <f>SUM(F8:F15)</f>
         <v>3200</v>
       </c>
@@ -7504,7 +7561,7 @@
     <row r="23" spans="5:10" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="27" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E27" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>17</v>
@@ -7544,7 +7601,7 @@
         <v>5</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" spans="5:10" ht="19" x14ac:dyDescent="0.25">
@@ -7563,7 +7620,7 @@
         <v>12</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G31" s="12" t="s">
         <v>12</v>
@@ -7582,18 +7639,18 @@
     </row>
     <row r="33" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E33" s="15" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F33" s="12" t="s">
         <v>12</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="34" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E34" s="15" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F34" s="12" t="s">
         <v>12</v>
@@ -7610,12 +7667,12 @@
         <v>20</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="38" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E38" s="6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>17</v>
@@ -7693,22 +7750,21 @@
     </row>
     <row r="44" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E44" s="15" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F44" s="12" t="s">
         <v>12</v>
       </c>
       <c r="G44" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="I44" s="12"/>
+        <v>38</v>
+      </c>
     </row>
     <row r="45" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E45" s="15" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F45" s="12" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G45" s="12" t="s">
         <v>10</v>
@@ -7732,7 +7788,7 @@
     </row>
     <row r="48" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E48" s="6" t="s">
-        <v>33</v>
+        <v>121</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>17</v>
@@ -7743,67 +7799,103 @@
       <c r="I48" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="J48" s="6"/>
+      <c r="J48" s="6" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="49" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E49" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="F49" s="12"/>
-      <c r="G49" s="12"/>
+      <c r="F49" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G49" s="12" t="s">
+        <v>12</v>
+      </c>
       <c r="I49" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="J49" s="6"/>
+      <c r="J49" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="50" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E50" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="F50" s="12"/>
-      <c r="G50" s="12"/>
+      <c r="F50" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="G50" s="12" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="51" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E51" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="F51" s="12"/>
-      <c r="G51" s="12"/>
+      <c r="F51" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="G51" s="12" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="52" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E52" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="F52" s="12"/>
-      <c r="G52" s="12"/>
+      <c r="F52" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G52" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="53" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E53" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="F53" s="12"/>
-      <c r="G53" s="12"/>
+      <c r="F53" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G53" s="12" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="54" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E54" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="F54" s="12"/>
-      <c r="G54" s="12"/>
+        <v>111</v>
+      </c>
+      <c r="F54" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="G54" s="12" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="55" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E55" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F55" s="12"/>
-      <c r="G55" s="12"/>
+        <v>38</v>
+      </c>
+      <c r="F55" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G55" s="12" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="56" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E56" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="F56" s="12"/>
-      <c r="G56" s="12"/>
+      <c r="F56" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="G56" s="12" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="57" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E57" s="13"/>
@@ -7812,7 +7904,7 @@
     </row>
     <row r="58" spans="5:10" x14ac:dyDescent="0.2">
       <c r="E58" s="16" t="s">
-        <v>34</v>
+        <v>123</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>17</v>
@@ -7823,74 +7915,110 @@
       <c r="I58" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="J58" s="6"/>
+      <c r="J58" s="6" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="59" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E59" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="F59" s="12"/>
-      <c r="G59" s="12"/>
+      <c r="F59" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G59" s="12" t="s">
+        <v>10</v>
+      </c>
       <c r="I59" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="J59" s="6"/>
+      <c r="J59" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="60" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E60" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="F60" s="12"/>
-      <c r="G60" s="12"/>
+      <c r="F60" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="G60" s="12" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="61" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E61" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="F61" s="12"/>
-      <c r="G61" s="12"/>
+      <c r="F61" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G61" s="12" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="62" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E62" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="F62" s="12"/>
-      <c r="G62" s="12"/>
+      <c r="F62" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G62" s="12" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="63" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E63" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="F63" s="12"/>
-      <c r="G63" s="12"/>
+      <c r="F63" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G63" s="12" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="64" spans="5:10" ht="19" x14ac:dyDescent="0.25">
       <c r="E64" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="F64" s="12"/>
-      <c r="G64" s="12"/>
+        <v>111</v>
+      </c>
+      <c r="F64" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G64" s="12" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="65" spans="5:13" ht="19" x14ac:dyDescent="0.25">
       <c r="E65" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F65" s="12"/>
-      <c r="G65" s="12"/>
+        <v>38</v>
+      </c>
+      <c r="F65" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G65" s="12" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="66" spans="5:13" ht="19" x14ac:dyDescent="0.25">
       <c r="E66" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="F66" s="12"/>
-      <c r="G66" s="12"/>
+      <c r="F66" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G66" s="12" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="68" spans="5:13" x14ac:dyDescent="0.2">
       <c r="I68" s="16" t="s">
         <v>11</v>
       </c>
       <c r="J68" s="16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K68" s="16" t="s">
         <v>7</v>
@@ -7907,7 +8035,7 @@
         <v>473.92857142857144</v>
       </c>
       <c r="L69" s="16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="70" spans="5:13" ht="21" x14ac:dyDescent="0.25">
@@ -7921,7 +8049,7 @@
         <v>366.42857142857144</v>
       </c>
       <c r="L70" s="16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="71" spans="5:13" ht="21" x14ac:dyDescent="0.25">
@@ -7935,7 +8063,7 @@
         <v>112.85714285714283</v>
       </c>
       <c r="L71" s="16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72" spans="5:13" ht="21" x14ac:dyDescent="0.25">
@@ -7949,7 +8077,7 @@
         <v>10</v>
       </c>
       <c r="L72" s="16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="73" spans="5:13" ht="21" x14ac:dyDescent="0.25">

</xml_diff>